<commit_message>
docs: adds the whole budget to the documentation
</commit_message>
<xml_diff>
--- a/docs/budget.xlsx
+++ b/docs/budget.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Desktop\proyectos\IRBoard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FFC3930-7616-4036-A087-C25AF39D5A55}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965A530D-4CE8-438C-B313-7FE2C2223067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Company definition" sheetId="2" r:id="rId1"/>
@@ -685,7 +685,7 @@
     <t>total hours</t>
   </si>
   <si>
-    <t>increase per hour</t>
+    <t>Dilution increase per billable hour</t>
   </si>
 </sst>
 </file>
@@ -1122,7 +1122,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="141">
+  <cellXfs count="136">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1321,6 +1321,29 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1328,12 +1351,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1345,29 +1362,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="12" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -31009,27 +31004,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="129" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="117"/>
-      <c r="F1" s="117"/>
-      <c r="G1" s="117"/>
-      <c r="H1" s="117"/>
-      <c r="I1" s="117"/>
-      <c r="J1" s="117"/>
-      <c r="K1" s="118"/>
-      <c r="L1" s="140" t="s">
+      <c r="B1" s="130"/>
+      <c r="C1" s="130"/>
+      <c r="D1" s="130"/>
+      <c r="E1" s="130"/>
+      <c r="F1" s="130"/>
+      <c r="G1" s="130"/>
+      <c r="H1" s="130"/>
+      <c r="I1" s="130"/>
+      <c r="J1" s="130"/>
+      <c r="K1" s="131"/>
+      <c r="L1" s="125" t="s">
         <v>213</v>
       </c>
-      <c r="N1" s="119" t="s">
+      <c r="N1" s="126" t="s">
         <v>203</v>
       </c>
-      <c r="O1" s="120"/>
-      <c r="P1" s="132"/>
+      <c r="O1" s="127"/>
+      <c r="P1" s="128"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -31065,14 +31060,14 @@
       <c r="K2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="137"/>
-      <c r="N2" s="130" t="s">
+      <c r="L2" s="118"/>
+      <c r="N2" s="119" t="s">
         <v>205</v>
       </c>
-      <c r="O2" s="129" t="s">
+      <c r="O2" s="118" t="s">
         <v>204</v>
       </c>
-      <c r="P2" s="131" t="s">
+      <c r="P2" s="120" t="s">
         <v>4</v>
       </c>
     </row>
@@ -31086,7 +31081,7 @@
         <v>20</v>
       </c>
       <c r="H3" s="111" t="str">
-        <f>_xlfn.XLOOKUP(E3,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" ref="H3:H34" si="0">_xlfn.XLOOKUP(E3,$Q$20:$Q$25,$R$20:$R$25,"")</f>
         <v/>
       </c>
       <c r="I3" s="111" t="str">
@@ -31097,17 +31092,17 @@
         <f>SUM(J4:J19)</f>
         <v>1493.463760343242</v>
       </c>
-      <c r="L3" s="139" t="str">
+      <c r="L3" s="110" t="str">
         <f>IFERROR(I3+($P$10*F3),"")</f>
         <v/>
       </c>
       <c r="N3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="O3" s="125" t="s">
+      <c r="O3" t="s">
         <v>206</v>
       </c>
-      <c r="P3" s="133">
+      <c r="P3" s="121">
         <f>K74</f>
         <v>13026.517352669423</v>
       </c>
@@ -31131,11 +31126,11 @@
         <v>103</v>
       </c>
       <c r="H4" s="111">
-        <f>_xlfn.XLOOKUP(E4,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I4" s="111">
-        <f t="shared" ref="I4:I67" si="0">IFERROR(H4*F4,"")</f>
+        <f t="shared" ref="I4:I67" si="1">IFERROR(H4*F4,"")</f>
         <v>99.564250689549496</v>
       </c>
       <c r="J4" s="111">
@@ -31143,17 +31138,17 @@
         <v>99.564250689549496</v>
       </c>
       <c r="K4" s="112"/>
-      <c r="L4" s="139">
-        <f t="shared" ref="L4:L67" si="1">IFERROR(I4+($P$10*F4),"")</f>
+      <c r="L4" s="110">
+        <f t="shared" ref="L4:L67" si="2">IFERROR(I4+($P$10*F4),"")</f>
         <v>122.72425068954949</v>
       </c>
       <c r="N4" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="O4" s="125" t="s">
+      <c r="O4" t="s">
         <v>207</v>
       </c>
-      <c r="P4" s="133">
+      <c r="P4" s="121">
         <f>K81</f>
         <v>172.5</v>
       </c>
@@ -31177,11 +31172,11 @@
         <v>103</v>
       </c>
       <c r="H5" s="111">
-        <f>_xlfn.XLOOKUP(E5,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I5" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J5" s="111">
@@ -31189,14 +31184,14 @@
         <v>99.564250689549496</v>
       </c>
       <c r="K5" s="112"/>
-      <c r="L5" s="139">
-        <f t="shared" si="1"/>
+      <c r="L5" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
       <c r="N5" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="O5" s="125" t="s">
+      <c r="O5" t="s">
         <v>208</v>
       </c>
       <c r="P5" s="112">
@@ -31214,11 +31209,11 @@
         <v>23</v>
       </c>
       <c r="H6" s="111" t="str">
-        <f>_xlfn.XLOOKUP(E6,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="I6" s="111" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="J6" s="111">
@@ -31226,12 +31221,12 @@
         <v>1294.3352589641431</v>
       </c>
       <c r="K6" s="112"/>
-      <c r="L6" s="139"/>
-      <c r="N6" s="119" t="s">
+      <c r="L6" s="110"/>
+      <c r="N6" s="126" t="s">
         <v>115</v>
       </c>
-      <c r="O6" s="120"/>
-      <c r="P6" s="134">
+      <c r="O6" s="127"/>
+      <c r="P6" s="122">
         <f>SUM(P3:P5)</f>
         <v>16498.77169083678</v>
       </c>
@@ -31255,17 +31250,17 @@
         <v>103</v>
       </c>
       <c r="H7" s="111">
-        <f>_xlfn.XLOOKUP(E7,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I7" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J7" s="111"/>
       <c r="K7" s="112"/>
-      <c r="L7" s="139">
-        <f t="shared" si="1"/>
+      <c r="L7" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -31288,17 +31283,17 @@
         <v>103</v>
       </c>
       <c r="H8" s="111">
-        <f>_xlfn.XLOOKUP(E8,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I8" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J8" s="111"/>
       <c r="K8" s="112"/>
-      <c r="L8" s="139">
-        <f t="shared" si="1"/>
+      <c r="L8" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
       <c r="O8" t="s">
@@ -31328,23 +31323,23 @@
         <v>103</v>
       </c>
       <c r="H9" s="111">
-        <f>_xlfn.XLOOKUP(E9,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I9" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J9" s="111"/>
       <c r="K9" s="112"/>
-      <c r="L9" s="139">
-        <f t="shared" si="1"/>
+      <c r="L9" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
       <c r="O9" t="s">
         <v>214</v>
       </c>
-      <c r="P9" s="136">
+      <c r="P9" s="135">
         <f>SUM(F4:F73)</f>
         <v>300</v>
       </c>
@@ -31368,23 +31363,23 @@
         <v>103</v>
       </c>
       <c r="H10" s="111">
-        <f>_xlfn.XLOOKUP(E10,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I10" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J10" s="111"/>
       <c r="K10" s="112"/>
-      <c r="L10" s="139">
-        <f t="shared" si="1"/>
+      <c r="L10" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
       <c r="O10" t="s">
         <v>215</v>
       </c>
-      <c r="P10" s="136">
+      <c r="P10" s="123">
         <f>ROUNDUP(P8/P9,2)</f>
         <v>11.58</v>
       </c>
@@ -31408,17 +31403,17 @@
         <v>103</v>
       </c>
       <c r="H11" s="111">
-        <f>_xlfn.XLOOKUP(E11,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I11" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J11" s="111"/>
       <c r="K11" s="112"/>
-      <c r="L11" s="139">
-        <f t="shared" si="1"/>
+      <c r="L11" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -31441,17 +31436,17 @@
         <v>103</v>
       </c>
       <c r="H12" s="111">
-        <f>_xlfn.XLOOKUP(E12,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I12" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J12" s="111"/>
       <c r="K12" s="112"/>
-      <c r="L12" s="139">
-        <f t="shared" si="1"/>
+      <c r="L12" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -31474,17 +31469,17 @@
         <v>103</v>
       </c>
       <c r="H13" s="111">
-        <f>_xlfn.XLOOKUP(E13,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I13" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J13" s="111"/>
       <c r="K13" s="112"/>
-      <c r="L13" s="139">
-        <f t="shared" si="1"/>
+      <c r="L13" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -31507,17 +31502,17 @@
         <v>103</v>
       </c>
       <c r="H14" s="111">
-        <f>_xlfn.XLOOKUP(E14,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I14" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J14" s="111"/>
       <c r="K14" s="112"/>
-      <c r="L14" s="139">
-        <f t="shared" si="1"/>
+      <c r="L14" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -31540,17 +31535,17 @@
         <v>103</v>
       </c>
       <c r="H15" s="111">
-        <f>_xlfn.XLOOKUP(E15,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I15" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J15" s="111"/>
       <c r="K15" s="112"/>
-      <c r="L15" s="139">
-        <f t="shared" si="1"/>
+      <c r="L15" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -31573,17 +31568,17 @@
         <v>103</v>
       </c>
       <c r="H16" s="111">
-        <f>_xlfn.XLOOKUP(E16,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I16" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J16" s="111"/>
       <c r="K16" s="112"/>
-      <c r="L16" s="139">
-        <f t="shared" si="1"/>
+      <c r="L16" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -31606,17 +31601,17 @@
         <v>103</v>
       </c>
       <c r="H17" s="111">
-        <f>_xlfn.XLOOKUP(E17,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I17" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J17" s="111"/>
       <c r="K17" s="112"/>
-      <c r="L17" s="139">
-        <f t="shared" si="1"/>
+      <c r="L17" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -31639,17 +31634,17 @@
         <v>103</v>
       </c>
       <c r="H18" s="111">
-        <f>_xlfn.XLOOKUP(E18,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I18" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J18" s="111"/>
       <c r="K18" s="112"/>
-      <c r="L18" s="139">
-        <f t="shared" si="1"/>
+      <c r="L18" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -31672,17 +31667,17 @@
         <v>103</v>
       </c>
       <c r="H19" s="111">
-        <f>_xlfn.XLOOKUP(E19,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I19" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J19" s="111"/>
       <c r="K19" s="112"/>
-      <c r="L19" s="139">
-        <f t="shared" si="1"/>
+      <c r="L19" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
       <c r="Q19" s="7" t="s">
@@ -31702,11 +31697,11 @@
         <v>37</v>
       </c>
       <c r="H20" s="111" t="str">
-        <f>_xlfn.XLOOKUP(E20,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="I20" s="111" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="J20" s="111"/>
@@ -31714,8 +31709,8 @@
         <f>SUM(J21:J30)</f>
         <v>2307.2124370166389</v>
       </c>
-      <c r="L20" s="139" t="str">
-        <f t="shared" si="1"/>
+      <c r="L20" s="110" t="str">
+        <f t="shared" si="2"/>
         <v/>
       </c>
       <c r="Q20" t="s">
@@ -31745,20 +31740,20 @@
         <v>103</v>
       </c>
       <c r="H21" s="111">
-        <f>_xlfn.XLOOKUP(E21,$Q$20:$Q$25,$R$20:$R$25,"")</f>
-        <v>42.159269173306768</v>
-      </c>
-      <c r="I21" s="111">
         <f t="shared" si="0"/>
         <v>42.159269173306768</v>
       </c>
+      <c r="I21" s="111">
+        <f t="shared" si="1"/>
+        <v>42.159269173306768</v>
+      </c>
       <c r="J21" s="111">
-        <f t="shared" ref="J21:J30" si="2">I21</f>
+        <f t="shared" ref="J21:J30" si="3">I21</f>
         <v>42.159269173306768</v>
       </c>
       <c r="K21" s="112"/>
-      <c r="L21" s="139">
-        <f t="shared" si="1"/>
+      <c r="L21" s="110">
+        <f t="shared" si="2"/>
         <v>53.739269173306766</v>
       </c>
       <c r="Q21" t="s">
@@ -31788,20 +31783,20 @@
         <v>103</v>
       </c>
       <c r="H22" s="111">
-        <f>_xlfn.XLOOKUP(E22,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>45.220459339114129</v>
       </c>
       <c r="I22" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>180.88183735645651</v>
       </c>
       <c r="J22" s="111">
+        <f t="shared" si="3"/>
+        <v>180.88183735645651</v>
+      </c>
+      <c r="K22" s="112"/>
+      <c r="L22" s="110">
         <f t="shared" si="2"/>
-        <v>180.88183735645651</v>
-      </c>
-      <c r="K22" s="112"/>
-      <c r="L22" s="139">
-        <f t="shared" si="1"/>
         <v>227.20183735645651</v>
       </c>
       <c r="Q22" t="s">
@@ -31831,20 +31826,20 @@
         <v>103</v>
       </c>
       <c r="H23" s="111">
-        <f>_xlfn.XLOOKUP(E23,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>42.159269173306768</v>
       </c>
       <c r="I23" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>84.318538346613536</v>
       </c>
       <c r="J23" s="111">
+        <f t="shared" si="3"/>
+        <v>84.318538346613536</v>
+      </c>
+      <c r="K23" s="112"/>
+      <c r="L23" s="110">
         <f t="shared" si="2"/>
-        <v>84.318538346613536</v>
-      </c>
-      <c r="K23" s="112"/>
-      <c r="L23" s="139">
-        <f t="shared" si="1"/>
         <v>107.47853834661353</v>
       </c>
       <c r="Q23" t="s">
@@ -31874,20 +31869,20 @@
         <v>103</v>
       </c>
       <c r="H24" s="111">
-        <f>_xlfn.XLOOKUP(E24,$Q$20:$Q$25,$R$20:$R$25,"")</f>
-        <v>42.159269173306768</v>
-      </c>
-      <c r="I24" s="111">
         <f t="shared" si="0"/>
         <v>42.159269173306768</v>
       </c>
+      <c r="I24" s="111">
+        <f t="shared" si="1"/>
+        <v>42.159269173306768</v>
+      </c>
       <c r="J24" s="111">
+        <f t="shared" si="3"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="K24" s="112"/>
+      <c r="L24" s="110">
         <f t="shared" si="2"/>
-        <v>42.159269173306768</v>
-      </c>
-      <c r="K24" s="112"/>
-      <c r="L24" s="139">
-        <f t="shared" si="1"/>
         <v>53.739269173306766</v>
       </c>
       <c r="Q24" t="s">
@@ -31917,20 +31912,20 @@
         <v>103</v>
       </c>
       <c r="H25" s="111">
-        <f>_xlfn.XLOOKUP(E25,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>42.159269173306768</v>
       </c>
       <c r="I25" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>84.318538346613536</v>
       </c>
       <c r="J25" s="111">
+        <f t="shared" si="3"/>
+        <v>84.318538346613536</v>
+      </c>
+      <c r="K25" s="112"/>
+      <c r="L25" s="110">
         <f t="shared" si="2"/>
-        <v>84.318538346613536</v>
-      </c>
-      <c r="K25" s="112"/>
-      <c r="L25" s="139">
-        <f t="shared" si="1"/>
         <v>107.47853834661353</v>
       </c>
       <c r="Q25" t="s">
@@ -31960,20 +31955,20 @@
         <v>103</v>
       </c>
       <c r="H26" s="111">
-        <f>_xlfn.XLOOKUP(E26,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>45.220459339114129</v>
       </c>
       <c r="I26" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>271.32275603468474</v>
       </c>
       <c r="J26" s="111">
+        <f t="shared" si="3"/>
+        <v>271.32275603468474</v>
+      </c>
+      <c r="K26" s="112"/>
+      <c r="L26" s="110">
         <f t="shared" si="2"/>
-        <v>271.32275603468474</v>
-      </c>
-      <c r="K26" s="112"/>
-      <c r="L26" s="139">
-        <f t="shared" si="1"/>
         <v>340.80275603468476</v>
       </c>
     </row>
@@ -31996,20 +31991,20 @@
         <v>103</v>
       </c>
       <c r="H27" s="111">
-        <f>_xlfn.XLOOKUP(E27,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>42.159269173306768</v>
       </c>
       <c r="I27" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>927.5039218127489</v>
       </c>
       <c r="J27" s="111">
+        <f t="shared" si="3"/>
+        <v>927.5039218127489</v>
+      </c>
+      <c r="K27" s="112"/>
+      <c r="L27" s="110">
         <f t="shared" si="2"/>
-        <v>927.5039218127489</v>
-      </c>
-      <c r="K27" s="112"/>
-      <c r="L27" s="139">
-        <f t="shared" si="1"/>
         <v>1182.2639218127488</v>
       </c>
     </row>
@@ -32032,20 +32027,20 @@
         <v>103</v>
       </c>
       <c r="H28" s="111">
-        <f>_xlfn.XLOOKUP(E28,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>42.159269173306768</v>
       </c>
       <c r="I28" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>252.95561503984061</v>
       </c>
       <c r="J28" s="111">
+        <f t="shared" si="3"/>
+        <v>252.95561503984061</v>
+      </c>
+      <c r="K28" s="112"/>
+      <c r="L28" s="110">
         <f t="shared" si="2"/>
-        <v>252.95561503984061</v>
-      </c>
-      <c r="K28" s="112"/>
-      <c r="L28" s="139">
-        <f t="shared" si="1"/>
         <v>322.43561503984063</v>
       </c>
     </row>
@@ -32068,20 +32063,20 @@
         <v>103</v>
       </c>
       <c r="H29" s="111">
-        <f>_xlfn.XLOOKUP(E29,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>42.159269173306768</v>
       </c>
       <c r="I29" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>84.318538346613536</v>
       </c>
       <c r="J29" s="111">
+        <f t="shared" si="3"/>
+        <v>84.318538346613536</v>
+      </c>
+      <c r="K29" s="112"/>
+      <c r="L29" s="110">
         <f t="shared" si="2"/>
-        <v>84.318538346613536</v>
-      </c>
-      <c r="K29" s="112"/>
-      <c r="L29" s="139">
-        <f t="shared" si="1"/>
         <v>107.47853834661353</v>
       </c>
     </row>
@@ -32104,20 +32099,20 @@
         <v>103</v>
       </c>
       <c r="H30" s="111">
-        <f>_xlfn.XLOOKUP(E30,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>42.159269173306768</v>
       </c>
       <c r="I30" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>337.27415338645415</v>
       </c>
       <c r="J30" s="111">
+        <f t="shared" si="3"/>
+        <v>337.27415338645415</v>
+      </c>
+      <c r="K30" s="112"/>
+      <c r="L30" s="110">
         <f t="shared" si="2"/>
-        <v>337.27415338645415</v>
-      </c>
-      <c r="K30" s="112"/>
-      <c r="L30" s="139">
-        <f t="shared" si="1"/>
         <v>429.91415338645413</v>
       </c>
     </row>
@@ -32131,11 +32126,11 @@
         <v>48</v>
       </c>
       <c r="H31" s="111" t="str">
-        <f>_xlfn.XLOOKUP(E31,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="I31" s="111" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="J31" s="111"/>
@@ -32143,8 +32138,8 @@
         <f>SUM(J32:J38)</f>
         <v>2273.3693320555312</v>
       </c>
-      <c r="L31" s="139" t="str">
-        <f t="shared" si="1"/>
+      <c r="L31" s="110" t="str">
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -32167,20 +32162,20 @@
         <v>103</v>
       </c>
       <c r="H32" s="111">
-        <f>_xlfn.XLOOKUP(E32,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>49.154057104913683</v>
       </c>
       <c r="I32" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>491.54057104913682</v>
       </c>
       <c r="J32" s="111">
-        <f t="shared" ref="J32:J38" si="3">I32</f>
+        <f t="shared" ref="J32:J38" si="4">I32</f>
         <v>491.54057104913682</v>
       </c>
       <c r="K32" s="112"/>
-      <c r="L32" s="139">
-        <f t="shared" si="1"/>
+      <c r="L32" s="110">
+        <f t="shared" si="2"/>
         <v>607.34057104913677</v>
       </c>
     </row>
@@ -32203,20 +32198,20 @@
         <v>103</v>
       </c>
       <c r="H33" s="111">
-        <f>_xlfn.XLOOKUP(E33,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I33" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>115.65544251565169</v>
       </c>
       <c r="J33" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>115.65544251565169</v>
       </c>
       <c r="K33" s="112"/>
-      <c r="L33" s="139">
-        <f t="shared" si="1"/>
+      <c r="L33" s="110">
+        <f t="shared" si="2"/>
         <v>150.39544251565169</v>
       </c>
     </row>
@@ -32239,20 +32234,20 @@
         <v>103</v>
       </c>
       <c r="H34" s="111">
-        <f>_xlfn.XLOOKUP(E34,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="0"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I34" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>350.77333020857748</v>
       </c>
       <c r="J34" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>350.77333020857748</v>
       </c>
       <c r="K34" s="112"/>
-      <c r="L34" s="139">
-        <f t="shared" si="1"/>
+      <c r="L34" s="110">
+        <f t="shared" si="2"/>
         <v>443.41333020857746</v>
       </c>
     </row>
@@ -32275,20 +32270,20 @@
         <v>103</v>
       </c>
       <c r="H35" s="111">
-        <f>_xlfn.XLOOKUP(E35,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" ref="H35:H66" si="5">_xlfn.XLOOKUP(E35,$Q$20:$Q$25,$R$20:$R$25,"")</f>
         <v>43.846666276072185</v>
       </c>
       <c r="I35" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>175.38666510428874</v>
       </c>
       <c r="J35" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>175.38666510428874</v>
       </c>
       <c r="K35" s="112"/>
-      <c r="L35" s="139">
-        <f t="shared" si="1"/>
+      <c r="L35" s="110">
+        <f t="shared" si="2"/>
         <v>221.70666510428873</v>
       </c>
     </row>
@@ -32311,20 +32306,20 @@
         <v>103</v>
       </c>
       <c r="H36" s="111">
-        <f>_xlfn.XLOOKUP(E36,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I36" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>263.07999765643308</v>
       </c>
       <c r="J36" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>263.07999765643308</v>
       </c>
       <c r="K36" s="112"/>
-      <c r="L36" s="139">
-        <f t="shared" si="1"/>
+      <c r="L36" s="110">
+        <f t="shared" si="2"/>
         <v>332.5599976564331</v>
       </c>
     </row>
@@ -32347,20 +32342,20 @@
         <v>103</v>
       </c>
       <c r="H37" s="111">
-        <f>_xlfn.XLOOKUP(E37,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I37" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>438.46666276072187</v>
       </c>
       <c r="J37" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>438.46666276072187</v>
       </c>
       <c r="K37" s="112"/>
-      <c r="L37" s="139">
-        <f t="shared" si="1"/>
+      <c r="L37" s="110">
+        <f t="shared" si="2"/>
         <v>554.26666276072183</v>
       </c>
     </row>
@@ -32383,20 +32378,20 @@
         <v>103</v>
       </c>
       <c r="H38" s="111">
-        <f>_xlfn.XLOOKUP(E38,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I38" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>438.46666276072187</v>
       </c>
       <c r="J38" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>438.46666276072187</v>
       </c>
       <c r="K38" s="112"/>
-      <c r="L38" s="139">
-        <f t="shared" si="1"/>
+      <c r="L38" s="110">
+        <f t="shared" si="2"/>
         <v>554.26666276072183</v>
       </c>
     </row>
@@ -32419,11 +32414,11 @@
         <v>103</v>
       </c>
       <c r="H39" s="111">
-        <f>_xlfn.XLOOKUP(E39,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I39" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>131.53999882821654</v>
       </c>
       <c r="J39" s="111">
@@ -32434,8 +32429,8 @@
         <f>SUM(J39)</f>
         <v>131.53999882821654</v>
       </c>
-      <c r="L39" s="139">
-        <f t="shared" si="1"/>
+      <c r="L39" s="110">
+        <f t="shared" si="2"/>
         <v>166.27999882821655</v>
       </c>
     </row>
@@ -32449,11 +32444,11 @@
         <v>56</v>
       </c>
       <c r="H40" s="111" t="str">
-        <f>_xlfn.XLOOKUP(E40,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="I40" s="111" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="J40" s="111"/>
@@ -32461,8 +32456,8 @@
         <f>SUM(J41:J50)</f>
         <v>4386.8987937884322</v>
       </c>
-      <c r="L40" s="139" t="str">
-        <f t="shared" si="1"/>
+      <c r="L40" s="110" t="str">
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -32485,11 +32480,11 @@
         <v>103</v>
       </c>
       <c r="H41" s="111">
-        <f>_xlfn.XLOOKUP(E41,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>49.154057104913683</v>
       </c>
       <c r="I41" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>196.61622841965473</v>
       </c>
       <c r="J41" s="111">
@@ -32497,8 +32492,8 @@
         <v>196.61622841965473</v>
       </c>
       <c r="K41" s="112"/>
-      <c r="L41" s="139">
-        <f t="shared" si="1"/>
+      <c r="L41" s="110">
+        <f t="shared" si="2"/>
         <v>242.93622841965473</v>
       </c>
     </row>
@@ -32521,11 +32516,11 @@
         <v>103</v>
       </c>
       <c r="H42" s="111">
-        <f>_xlfn.XLOOKUP(E42,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>49.154057104913683</v>
       </c>
       <c r="I42" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>147.46217131474106</v>
       </c>
       <c r="J42" s="111">
@@ -32533,8 +32528,8 @@
         <v>147.46217131474106</v>
       </c>
       <c r="K42" s="112"/>
-      <c r="L42" s="139">
-        <f t="shared" si="1"/>
+      <c r="L42" s="110">
+        <f t="shared" si="2"/>
         <v>182.20217131474107</v>
       </c>
     </row>
@@ -32548,11 +32543,11 @@
         <v>59</v>
       </c>
       <c r="H43" s="111" t="str">
-        <f>_xlfn.XLOOKUP(E43,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="I43" s="111" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="J43" s="111">
@@ -32560,8 +32555,8 @@
         <v>4042.8203940540366</v>
       </c>
       <c r="K43" s="112"/>
-      <c r="L43" s="139" t="str">
-        <f t="shared" si="1"/>
+      <c r="L43" s="110" t="str">
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -32584,17 +32579,17 @@
         <v>103</v>
       </c>
       <c r="H44" s="111">
-        <f>_xlfn.XLOOKUP(E44,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I44" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>848.13991178144579</v>
       </c>
       <c r="J44" s="111"/>
       <c r="K44" s="112"/>
-      <c r="L44" s="139">
-        <f t="shared" si="1"/>
+      <c r="L44" s="110">
+        <f t="shared" si="2"/>
         <v>1102.8999117814458</v>
       </c>
     </row>
@@ -32617,17 +32612,17 @@
         <v>103</v>
       </c>
       <c r="H45" s="111">
-        <f>_xlfn.XLOOKUP(E45,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I45" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>385.51814171883899</v>
       </c>
       <c r="J45" s="111"/>
       <c r="K45" s="112"/>
-      <c r="L45" s="139">
-        <f t="shared" si="1"/>
+      <c r="L45" s="110">
+        <f t="shared" si="2"/>
         <v>501.318141718839</v>
       </c>
     </row>
@@ -32650,17 +32645,17 @@
         <v>103</v>
       </c>
       <c r="H46" s="111">
-        <f>_xlfn.XLOOKUP(E46,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I46" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>1096.1666569018046</v>
       </c>
       <c r="J46" s="111"/>
       <c r="K46" s="112"/>
-      <c r="L46" s="139">
-        <f t="shared" si="1"/>
+      <c r="L46" s="110">
+        <f t="shared" si="2"/>
         <v>1385.6666569018046</v>
       </c>
     </row>
@@ -32683,17 +32678,17 @@
         <v>103</v>
       </c>
       <c r="H47" s="111">
-        <f>_xlfn.XLOOKUP(E47,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I47" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>231.31088503130337</v>
       </c>
       <c r="J47" s="111"/>
       <c r="K47" s="112"/>
-      <c r="L47" s="139">
-        <f t="shared" si="1"/>
+      <c r="L47" s="110">
+        <f t="shared" si="2"/>
         <v>300.79088503130339</v>
       </c>
     </row>
@@ -32716,17 +32711,17 @@
         <v>103</v>
       </c>
       <c r="H48" s="111">
-        <f>_xlfn.XLOOKUP(E48,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I48" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>657.69999414108281</v>
       </c>
       <c r="J48" s="111"/>
       <c r="K48" s="112"/>
-      <c r="L48" s="139">
-        <f t="shared" si="1"/>
+      <c r="L48" s="110">
+        <f t="shared" si="2"/>
         <v>831.39999414108274</v>
       </c>
     </row>
@@ -32749,17 +32744,17 @@
         <v>103</v>
       </c>
       <c r="H49" s="111">
-        <f>_xlfn.XLOOKUP(E49,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I49" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>438.46666276072187</v>
       </c>
       <c r="J49" s="111"/>
       <c r="K49" s="112"/>
-      <c r="L49" s="139">
-        <f t="shared" si="1"/>
+      <c r="L49" s="110">
+        <f t="shared" si="2"/>
         <v>554.26666276072183</v>
       </c>
     </row>
@@ -32782,17 +32777,17 @@
         <v>103</v>
       </c>
       <c r="H50" s="111">
-        <f>_xlfn.XLOOKUP(E50,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I50" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>385.51814171883899</v>
       </c>
       <c r="J50" s="111"/>
       <c r="K50" s="112"/>
-      <c r="L50" s="139">
-        <f t="shared" si="1"/>
+      <c r="L50" s="110">
+        <f t="shared" si="2"/>
         <v>501.318141718839</v>
       </c>
     </row>
@@ -32806,11 +32801,11 @@
         <v>66</v>
       </c>
       <c r="H51" s="111" t="str">
-        <f>_xlfn.XLOOKUP(E51,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="I51" s="111" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="J51" s="111"/>
@@ -32818,8 +32813,8 @@
         <f>SUM(J52:J60)</f>
         <v>1051.4886868492417</v>
       </c>
-      <c r="L51" s="139" t="str">
-        <f t="shared" si="1"/>
+      <c r="L51" s="110" t="str">
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -32842,20 +32837,20 @@
         <v>103</v>
       </c>
       <c r="H52" s="111">
-        <f>_xlfn.XLOOKUP(E52,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I52" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>154.20725668753559</v>
       </c>
       <c r="J52" s="111">
-        <f t="shared" ref="J52:J60" si="4">I52</f>
+        <f t="shared" ref="J52:J60" si="6">I52</f>
         <v>154.20725668753559</v>
       </c>
       <c r="K52" s="112"/>
-      <c r="L52" s="139">
-        <f t="shared" si="1"/>
+      <c r="L52" s="110">
+        <f t="shared" si="2"/>
         <v>200.52725668753558</v>
       </c>
     </row>
@@ -32878,20 +32873,20 @@
         <v>103</v>
       </c>
       <c r="H53" s="111">
-        <f>_xlfn.XLOOKUP(E53,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I53" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>115.65544251565169</v>
       </c>
       <c r="J53" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>115.65544251565169</v>
       </c>
       <c r="K53" s="112"/>
-      <c r="L53" s="139">
-        <f t="shared" si="1"/>
+      <c r="L53" s="110">
+        <f t="shared" si="2"/>
         <v>150.39544251565169</v>
       </c>
     </row>
@@ -32914,20 +32909,20 @@
         <v>103</v>
       </c>
       <c r="H54" s="111">
-        <f>_xlfn.XLOOKUP(E54,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I54" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>192.7590708594195</v>
       </c>
       <c r="J54" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>192.7590708594195</v>
       </c>
       <c r="K54" s="112"/>
-      <c r="L54" s="139">
-        <f t="shared" si="1"/>
+      <c r="L54" s="110">
+        <f t="shared" si="2"/>
         <v>250.6590708594195</v>
       </c>
     </row>
@@ -32950,20 +32945,20 @@
         <v>103</v>
       </c>
       <c r="H55" s="111">
-        <f>_xlfn.XLOOKUP(E55,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I55" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>115.65544251565169</v>
       </c>
       <c r="J55" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>115.65544251565169</v>
       </c>
       <c r="K55" s="112"/>
-      <c r="L55" s="139">
-        <f t="shared" si="1"/>
+      <c r="L55" s="110">
+        <f t="shared" si="2"/>
         <v>150.39544251565169</v>
       </c>
     </row>
@@ -32986,20 +32981,20 @@
         <v>103</v>
       </c>
       <c r="H56" s="111">
-        <f>_xlfn.XLOOKUP(E56,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I56" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>115.65544251565169</v>
       </c>
       <c r="J56" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>115.65544251565169</v>
       </c>
       <c r="K56" s="112"/>
-      <c r="L56" s="139">
-        <f t="shared" si="1"/>
+      <c r="L56" s="110">
+        <f t="shared" si="2"/>
         <v>150.39544251565169</v>
       </c>
     </row>
@@ -33022,20 +33017,20 @@
         <v>103</v>
       </c>
       <c r="H57" s="111">
-        <f>_xlfn.XLOOKUP(E57,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I57" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>77.103628343767795</v>
       </c>
       <c r="J57" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>77.103628343767795</v>
       </c>
       <c r="K57" s="112"/>
-      <c r="L57" s="139">
-        <f t="shared" si="1"/>
+      <c r="L57" s="110">
+        <f t="shared" si="2"/>
         <v>100.26362834376779</v>
       </c>
     </row>
@@ -33058,20 +33053,20 @@
         <v>103</v>
       </c>
       <c r="H58" s="111">
-        <f>_xlfn.XLOOKUP(E58,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I58" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>115.65544251565169</v>
       </c>
       <c r="J58" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>115.65544251565169</v>
       </c>
       <c r="K58" s="112"/>
-      <c r="L58" s="139">
-        <f t="shared" si="1"/>
+      <c r="L58" s="110">
+        <f t="shared" si="2"/>
         <v>150.39544251565169</v>
       </c>
     </row>
@@ -33094,20 +33089,20 @@
         <v>103</v>
       </c>
       <c r="H59" s="111">
-        <f>_xlfn.XLOOKUP(E59,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>38.551814171883898</v>
       </c>
       <c r="I59" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>77.103628343767795</v>
       </c>
       <c r="J59" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>77.103628343767795</v>
       </c>
       <c r="K59" s="112"/>
-      <c r="L59" s="139">
-        <f t="shared" si="1"/>
+      <c r="L59" s="110">
+        <f t="shared" si="2"/>
         <v>100.26362834376779</v>
       </c>
     </row>
@@ -33130,20 +33125,20 @@
         <v>103</v>
       </c>
       <c r="H60" s="111">
-        <f>_xlfn.XLOOKUP(E60,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I60" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>87.693332552144369</v>
       </c>
       <c r="J60" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="6"/>
         <v>87.693332552144369</v>
       </c>
       <c r="K60" s="112"/>
-      <c r="L60" s="139">
-        <f t="shared" si="1"/>
+      <c r="L60" s="110">
+        <f t="shared" si="2"/>
         <v>110.85333255214437</v>
       </c>
     </row>
@@ -33157,11 +33152,11 @@
         <v>74</v>
       </c>
       <c r="H61" s="111" t="str">
-        <f>_xlfn.XLOOKUP(E61,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v/>
       </c>
       <c r="I61" s="111" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v/>
       </c>
       <c r="J61" s="111"/>
@@ -33169,8 +33164,8 @@
         <f>SUM(J62:J73)</f>
         <v>1382.5443437881208</v>
       </c>
-      <c r="L61" s="139" t="str">
-        <f t="shared" si="1"/>
+      <c r="L61" s="110" t="str">
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
@@ -33193,20 +33188,20 @@
         <v>103</v>
       </c>
       <c r="H62" s="111">
-        <f>_xlfn.XLOOKUP(E62,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I62" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>49.782125344774748</v>
       </c>
       <c r="J62" s="111">
-        <f t="shared" ref="J62:J73" si="5">I62</f>
+        <f t="shared" ref="J62:J73" si="7">I62</f>
         <v>49.782125344774748</v>
       </c>
       <c r="K62" s="112"/>
-      <c r="L62" s="139">
-        <f t="shared" si="1"/>
+      <c r="L62" s="110">
+        <f t="shared" si="2"/>
         <v>61.362125344774746</v>
       </c>
     </row>
@@ -33229,20 +33224,20 @@
         <v>103</v>
       </c>
       <c r="H63" s="111">
-        <f>_xlfn.XLOOKUP(E63,$Q$20:$Q$25,$R$20:$R$25,"")</f>
-        <v>49.782125344774748</v>
-      </c>
-      <c r="I63" s="111">
-        <f t="shared" si="0"/>
-        <v>49.782125344774748</v>
-      </c>
-      <c r="J63" s="111">
         <f t="shared" si="5"/>
         <v>49.782125344774748</v>
       </c>
+      <c r="I63" s="111">
+        <f t="shared" si="1"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J63" s="111">
+        <f t="shared" si="7"/>
+        <v>49.782125344774748</v>
+      </c>
       <c r="K63" s="112"/>
-      <c r="L63" s="139">
-        <f t="shared" si="1"/>
+      <c r="L63" s="110">
+        <f t="shared" si="2"/>
         <v>61.362125344774746</v>
       </c>
     </row>
@@ -33265,20 +33260,20 @@
         <v>103</v>
       </c>
       <c r="H64" s="111">
-        <f>_xlfn.XLOOKUP(E64,$Q$20:$Q$25,$R$20:$R$25,"")</f>
-        <v>45.220459339114129</v>
-      </c>
-      <c r="I64" s="111">
-        <f t="shared" si="0"/>
-        <v>45.220459339114129</v>
-      </c>
-      <c r="J64" s="111">
         <f t="shared" si="5"/>
         <v>45.220459339114129</v>
       </c>
+      <c r="I64" s="111">
+        <f t="shared" si="1"/>
+        <v>45.220459339114129</v>
+      </c>
+      <c r="J64" s="111">
+        <f t="shared" si="7"/>
+        <v>45.220459339114129</v>
+      </c>
       <c r="K64" s="112"/>
-      <c r="L64" s="139">
-        <f t="shared" si="1"/>
+      <c r="L64" s="110">
+        <f t="shared" si="2"/>
         <v>56.800459339114127</v>
       </c>
     </row>
@@ -33301,20 +33296,20 @@
         <v>103</v>
       </c>
       <c r="H65" s="111">
-        <f>_xlfn.XLOOKUP(E65,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>45.220459339114129</v>
       </c>
       <c r="I65" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>90.440918678228257</v>
       </c>
       <c r="J65" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>90.440918678228257</v>
       </c>
       <c r="K65" s="112"/>
-      <c r="L65" s="139">
-        <f t="shared" si="1"/>
+      <c r="L65" s="110">
+        <f t="shared" si="2"/>
         <v>113.60091867822825</v>
       </c>
     </row>
@@ -33337,20 +33332,20 @@
         <v>103</v>
       </c>
       <c r="H66" s="111">
-        <f>_xlfn.XLOOKUP(E66,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="5"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I66" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J66" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>99.564250689549496</v>
       </c>
       <c r="K66" s="112"/>
-      <c r="L66" s="139">
-        <f t="shared" si="1"/>
+      <c r="L66" s="110">
+        <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -33373,20 +33368,20 @@
         <v>103</v>
       </c>
       <c r="H67" s="111">
-        <f>_xlfn.XLOOKUP(E67,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" ref="H67:H73" si="8">_xlfn.XLOOKUP(E67,$Q$20:$Q$25,$R$20:$R$25,"")</f>
         <v>42.159269173306768</v>
       </c>
       <c r="I67" s="111">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>126.4778075199203</v>
       </c>
       <c r="J67" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>126.4778075199203</v>
       </c>
       <c r="K67" s="112"/>
-      <c r="L67" s="139">
-        <f t="shared" si="1"/>
+      <c r="L67" s="110">
+        <f t="shared" si="2"/>
         <v>161.21780751992031</v>
       </c>
     </row>
@@ -33409,20 +33404,20 @@
         <v>103</v>
       </c>
       <c r="H68" s="111">
-        <f>_xlfn.XLOOKUP(E68,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="8"/>
         <v>49.154057104913683</v>
       </c>
       <c r="I68" s="111">
-        <f t="shared" ref="I68:I73" si="6">IFERROR(H68*F68,"")</f>
+        <f t="shared" ref="I68:I73" si="9">IFERROR(H68*F68,"")</f>
         <v>245.77028552456841</v>
       </c>
       <c r="J68" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>245.77028552456841</v>
       </c>
       <c r="K68" s="112"/>
-      <c r="L68" s="139">
-        <f t="shared" ref="L68:L73" si="7">IFERROR(I68+($P$10*F68),"")</f>
+      <c r="L68" s="110">
+        <f t="shared" ref="L68:L73" si="10">IFERROR(I68+($P$10*F68),"")</f>
         <v>303.67028552456838</v>
       </c>
     </row>
@@ -33445,20 +33440,20 @@
         <v>103</v>
       </c>
       <c r="H69" s="111">
-        <f>_xlfn.XLOOKUP(E69,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="8"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I69" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>219.23333138036094</v>
       </c>
       <c r="J69" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>219.23333138036094</v>
       </c>
       <c r="K69" s="112"/>
-      <c r="L69" s="139">
-        <f t="shared" si="7"/>
+      <c r="L69" s="110">
+        <f t="shared" si="10"/>
         <v>277.13333138036091</v>
       </c>
     </row>
@@ -33481,20 +33476,20 @@
         <v>103</v>
       </c>
       <c r="H70" s="111">
-        <f>_xlfn.XLOOKUP(E70,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="8"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I70" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>87.693332552144369</v>
       </c>
       <c r="J70" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>87.693332552144369</v>
       </c>
       <c r="K70" s="112"/>
-      <c r="L70" s="139">
-        <f t="shared" si="7"/>
+      <c r="L70" s="110">
+        <f t="shared" si="10"/>
         <v>110.85333255214437</v>
       </c>
     </row>
@@ -33517,20 +33512,20 @@
         <v>103</v>
       </c>
       <c r="H71" s="111">
-        <f>_xlfn.XLOOKUP(E71,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="8"/>
         <v>43.846666276072185</v>
       </c>
       <c r="I71" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>219.23333138036094</v>
       </c>
       <c r="J71" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>219.23333138036094</v>
       </c>
       <c r="K71" s="112"/>
-      <c r="L71" s="139">
-        <f t="shared" si="7"/>
+      <c r="L71" s="110">
+        <f t="shared" si="10"/>
         <v>277.13333138036091</v>
       </c>
     </row>
@@ -33553,20 +33548,20 @@
         <v>103</v>
       </c>
       <c r="H72" s="111">
-        <f>_xlfn.XLOOKUP(E72,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="8"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I72" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>99.564250689549496</v>
       </c>
       <c r="J72" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>99.564250689549496</v>
       </c>
       <c r="K72" s="112"/>
-      <c r="L72" s="139">
-        <f t="shared" si="7"/>
+      <c r="L72" s="110">
+        <f t="shared" si="10"/>
         <v>122.72425068954949</v>
       </c>
     </row>
@@ -33589,41 +33584,41 @@
         <v>103</v>
       </c>
       <c r="H73" s="111">
-        <f>_xlfn.XLOOKUP(E73,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" si="8"/>
         <v>49.782125344774748</v>
       </c>
       <c r="I73" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="9"/>
         <v>49.782125344774748</v>
       </c>
       <c r="J73" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="7"/>
         <v>49.782125344774748</v>
       </c>
       <c r="K73" s="113"/>
-      <c r="L73" s="139">
-        <f t="shared" si="7"/>
+      <c r="L73" s="110">
+        <f t="shared" si="10"/>
         <v>61.362125344774746</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A74" s="119" t="s">
+      <c r="A74" s="126" t="s">
         <v>4</v>
       </c>
-      <c r="B74" s="120"/>
-      <c r="C74" s="120"/>
-      <c r="D74" s="120"/>
-      <c r="E74" s="120"/>
-      <c r="F74" s="120"/>
-      <c r="G74" s="120"/>
-      <c r="H74" s="120"/>
-      <c r="I74" s="120"/>
-      <c r="J74" s="120"/>
+      <c r="B74" s="127"/>
+      <c r="C74" s="127"/>
+      <c r="D74" s="127"/>
+      <c r="E74" s="127"/>
+      <c r="F74" s="127"/>
+      <c r="G74" s="127"/>
+      <c r="H74" s="127"/>
+      <c r="I74" s="127"/>
+      <c r="J74" s="127"/>
       <c r="K74" s="114">
         <f>SUM(K3:K73)</f>
         <v>13026.517352669423</v>
       </c>
-      <c r="L74" s="135">
+      <c r="L74" s="111">
         <f>SUM(L3:L73)</f>
         <v>16500.51735266942</v>
       </c>
@@ -33633,20 +33628,20 @@
       <c r="L75" s="2"/>
     </row>
     <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="121" t="s">
+      <c r="A76" s="132" t="s">
         <v>192</v>
       </c>
-      <c r="B76" s="122"/>
-      <c r="C76" s="122"/>
-      <c r="D76" s="122"/>
-      <c r="E76" s="122"/>
-      <c r="F76" s="122"/>
-      <c r="G76" s="122"/>
-      <c r="H76" s="122"/>
-      <c r="I76" s="122"/>
-      <c r="J76" s="122"/>
-      <c r="K76" s="123"/>
-      <c r="L76" s="138"/>
+      <c r="B76" s="133"/>
+      <c r="C76" s="133"/>
+      <c r="D76" s="133"/>
+      <c r="E76" s="133"/>
+      <c r="F76" s="133"/>
+      <c r="G76" s="133"/>
+      <c r="H76" s="133"/>
+      <c r="I76" s="133"/>
+      <c r="J76" s="133"/>
+      <c r="K76" s="134"/>
+      <c r="L76" s="124"/>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A77" s="12" t="s">
@@ -33682,108 +33677,105 @@
       <c r="K77" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="L77" s="137"/>
+      <c r="L77" s="118"/>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="B78" s="124"/>
-      <c r="C78" s="124"/>
-      <c r="D78" s="125" t="s">
+      <c r="B78" s="6"/>
+      <c r="C78" s="6"/>
+      <c r="D78" t="s">
         <v>197</v>
       </c>
-      <c r="E78" s="125"/>
-      <c r="F78" s="125"/>
-      <c r="G78" s="125"/>
-      <c r="H78" s="127"/>
-      <c r="I78" s="127"/>
-      <c r="J78" s="127">
+      <c r="H78" s="116"/>
+      <c r="I78" s="116"/>
+      <c r="J78" s="116">
         <f>SUM(I79:I80)</f>
         <v>172.5</v>
       </c>
-      <c r="K78" s="128">
+      <c r="K78" s="117">
         <f>J78</f>
         <v>172.5</v>
       </c>
-      <c r="L78" s="127"/>
+      <c r="L78" s="116"/>
     </row>
     <row r="79" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A79" s="5"/>
-      <c r="B79" s="124" t="s">
+      <c r="B79" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C79" s="124"/>
-      <c r="D79" s="125" t="s">
+      <c r="C79" s="6"/>
+      <c r="D79" t="s">
         <v>198</v>
       </c>
-      <c r="E79" s="125" t="s">
+      <c r="E79" t="s">
         <v>200</v>
       </c>
-      <c r="F79" s="125">
+      <c r="F79">
         <v>150</v>
       </c>
-      <c r="G79" s="126" t="s">
+      <c r="G79" t="s">
         <v>201</v>
       </c>
-      <c r="H79" s="127">
+      <c r="H79" s="116">
         <v>0.35</v>
       </c>
-      <c r="I79" s="127">
+      <c r="I79" s="116">
         <f>H79*F79</f>
         <v>52.5</v>
       </c>
-      <c r="J79" s="127"/>
-      <c r="K79" s="128"/>
-      <c r="L79" s="127"/>
+      <c r="J79" s="116"/>
+      <c r="K79" s="117"/>
+      <c r="L79" s="116"/>
     </row>
     <row r="80" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A80" s="5"/>
-      <c r="B80" s="124" t="s">
+      <c r="B80" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C80" s="124"/>
-      <c r="D80" s="125" t="s">
+      <c r="C80" s="6"/>
+      <c r="D80" t="s">
         <v>199</v>
       </c>
-      <c r="E80" s="125" t="s">
+      <c r="E80" t="s">
         <v>200</v>
       </c>
-      <c r="F80" s="125">
+      <c r="F80">
         <v>6</v>
       </c>
-      <c r="G80" s="126" t="s">
+      <c r="G80" t="s">
         <v>202</v>
       </c>
-      <c r="H80" s="127">
+      <c r="H80" s="116">
         <v>20</v>
       </c>
-      <c r="I80" s="127">
+      <c r="I80" s="116">
         <f>H80*F80</f>
         <v>120</v>
       </c>
-      <c r="J80" s="127"/>
-      <c r="K80" s="128"/>
-      <c r="L80" s="127"/>
+      <c r="J80" s="116"/>
+      <c r="K80" s="117"/>
+      <c r="L80" s="116"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A81" s="119" t="s">
+      <c r="A81" s="126" t="s">
         <v>4</v>
       </c>
-      <c r="B81" s="120"/>
-      <c r="C81" s="120"/>
-      <c r="D81" s="120"/>
-      <c r="E81" s="120"/>
-      <c r="F81" s="120"/>
-      <c r="G81" s="120"/>
-      <c r="H81" s="120"/>
-      <c r="I81" s="120"/>
-      <c r="J81" s="120"/>
+      <c r="B81" s="127"/>
+      <c r="C81" s="127"/>
+      <c r="D81" s="127"/>
+      <c r="E81" s="127"/>
+      <c r="F81" s="127"/>
+      <c r="G81" s="127"/>
+      <c r="H81" s="127"/>
+      <c r="I81" s="127"/>
+      <c r="J81" s="127"/>
       <c r="K81" s="114">
         <f>SUM(K78:K80)</f>
         <v>172.5</v>
       </c>
-      <c r="L81" s="135"/>
+      <c r="L81" s="111"/>
     </row>
     <row r="82" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A82" s="6"/>
@@ -33828,18 +33820,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="116" t="s">
+      <c r="A1" s="129" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="117"/>
-      <c r="C1" s="117"/>
-      <c r="D1" s="117"/>
-      <c r="E1" s="118"/>
-      <c r="G1" s="119" t="s">
+      <c r="B1" s="130"/>
+      <c r="C1" s="130"/>
+      <c r="D1" s="130"/>
+      <c r="E1" s="131"/>
+      <c r="G1" s="126" t="s">
         <v>209</v>
       </c>
-      <c r="H1" s="120"/>
-      <c r="I1" s="132"/>
+      <c r="H1" s="127"/>
+      <c r="I1" s="128"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -33857,13 +33849,13 @@
       <c r="E2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="G2" s="130" t="s">
+      <c r="G2" s="119" t="s">
         <v>205</v>
       </c>
-      <c r="H2" s="129" t="s">
+      <c r="H2" s="118" t="s">
         <v>204</v>
       </c>
-      <c r="I2" s="131" t="s">
+      <c r="I2" s="120" t="s">
         <v>4</v>
       </c>
     </row>
@@ -33875,7 +33867,7 @@
       <c r="C3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="D3" s="136"/>
+      <c r="D3" s="123"/>
       <c r="E3" s="115">
         <f>SUM(D4:D6)</f>
         <v>1840.8637603432428</v>
@@ -33883,10 +33875,10 @@
       <c r="G3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="H3" s="125" t="s">
+      <c r="H3" t="s">
         <v>206</v>
       </c>
-      <c r="I3" s="133">
+      <c r="I3" s="121">
         <f>E54</f>
         <v>16500.517352669427</v>
       </c>
@@ -33899,16 +33891,16 @@
       <c r="C4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="136">
+      <c r="D4" s="123">
         <f>Costs_init!L4</f>
         <v>122.72425068954949</v>
       </c>
       <c r="E4" s="112"/>
-      <c r="G4" s="119" t="s">
+      <c r="G4" s="126" t="s">
         <v>115</v>
       </c>
-      <c r="H4" s="120"/>
-      <c r="I4" s="134">
+      <c r="H4" s="127"/>
+      <c r="I4" s="122">
         <f>SUM(I3)</f>
         <v>16500.517352669427</v>
       </c>
@@ -33921,14 +33913,13 @@
       <c r="C5" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="136">
+      <c r="D5" s="123">
         <f>Costs_init!L5</f>
         <v>122.72425068954949</v>
       </c>
       <c r="E5" s="112"/>
-      <c r="G5" s="124"/>
-      <c r="H5" s="125"/>
-      <c r="I5" s="135"/>
+      <c r="G5" s="6"/>
+      <c r="I5" s="111"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
@@ -33938,7 +33929,7 @@
       <c r="C6" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="D6" s="136">
+      <c r="D6" s="123">
         <f>SUM(Costs_init!L7:L19)</f>
         <v>1595.4152589641437</v>
       </c>
@@ -33952,7 +33943,7 @@
       <c r="C7" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="D7" s="136"/>
+      <c r="D7" s="123"/>
       <c r="E7" s="112">
         <f>SUM(D8:D17)</f>
         <v>2932.5324370166391</v>
@@ -33967,7 +33958,7 @@
       <c r="C8" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="136">
+      <c r="D8" s="123">
         <f>Costs_init!L21</f>
         <v>53.739269173306766</v>
       </c>
@@ -33982,7 +33973,7 @@
       <c r="C9" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="136">
+      <c r="D9" s="123">
         <f>Costs_init!L22</f>
         <v>227.20183735645651</v>
       </c>
@@ -33997,7 +33988,7 @@
       <c r="C10" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="136">
+      <c r="D10" s="123">
         <f>Costs_init!L23</f>
         <v>107.47853834661353</v>
       </c>
@@ -34012,7 +34003,7 @@
       <c r="C11" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="136">
+      <c r="D11" s="123">
         <f>Costs_init!L24</f>
         <v>53.739269173306766</v>
       </c>
@@ -34027,7 +34018,7 @@
       <c r="C12" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D12" s="136">
+      <c r="D12" s="123">
         <f>Costs_init!L25</f>
         <v>107.47853834661353</v>
       </c>
@@ -34042,7 +34033,7 @@
       <c r="C13" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="136">
+      <c r="D13" s="123">
         <f>Costs_init!L26</f>
         <v>340.80275603468476</v>
       </c>
@@ -34056,7 +34047,7 @@
       <c r="C14" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="D14" s="136">
+      <c r="D14" s="123">
         <f>Costs_init!L27</f>
         <v>1182.2639218127488</v>
       </c>
@@ -34070,7 +34061,7 @@
       <c r="C15" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="D15" s="136">
+      <c r="D15" s="123">
         <f>Costs_init!L28</f>
         <v>322.43561503984063</v>
       </c>
@@ -34084,7 +34075,7 @@
       <c r="C16" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="D16" s="136">
+      <c r="D16" s="123">
         <f>Costs_init!L29</f>
         <v>107.47853834661353</v>
       </c>
@@ -34098,7 +34089,7 @@
       <c r="C17" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="D17" s="136">
+      <c r="D17" s="123">
         <f>Costs_init!L30</f>
         <v>429.91415338645413</v>
       </c>
@@ -34112,7 +34103,7 @@
       <c r="C18" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="D18" s="136" t="str">
+      <c r="D18" s="123" t="str">
         <f>Costs_init!L31</f>
         <v/>
       </c>
@@ -34129,7 +34120,7 @@
       <c r="C19" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D19" s="136">
+      <c r="D19" s="123">
         <f>Costs_init!L32</f>
         <v>607.34057104913677</v>
       </c>
@@ -34143,7 +34134,7 @@
       <c r="C20" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="D20" s="136">
+      <c r="D20" s="123">
         <f>Costs_init!L33</f>
         <v>150.39544251565169</v>
       </c>
@@ -34157,7 +34148,7 @@
       <c r="C21" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="136">
+      <c r="D21" s="123">
         <f>Costs_init!L34</f>
         <v>443.41333020857746</v>
       </c>
@@ -34171,7 +34162,7 @@
       <c r="C22" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="136">
+      <c r="D22" s="123">
         <f>Costs_init!L35</f>
         <v>221.70666510428873</v>
       </c>
@@ -34185,7 +34176,7 @@
       <c r="C23" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="D23" s="136">
+      <c r="D23" s="123">
         <f>Costs_init!L36</f>
         <v>332.5599976564331</v>
       </c>
@@ -34199,7 +34190,7 @@
       <c r="C24" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="D24" s="136">
+      <c r="D24" s="123">
         <f>Costs_init!L37</f>
         <v>554.26666276072183</v>
       </c>
@@ -34213,7 +34204,7 @@
       <c r="C25" s="1" t="s">
         <v>194</v>
       </c>
-      <c r="D25" s="136">
+      <c r="D25" s="123">
         <f>Costs_init!L38</f>
         <v>554.26666276072183</v>
       </c>
@@ -34227,7 +34218,7 @@
       <c r="C26" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="D26" s="136">
+      <c r="D26" s="123">
         <f>Costs_init!L39</f>
         <v>166.27999882821655</v>
       </c>
@@ -34244,7 +34235,7 @@
       <c r="C27" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="D27" s="136" t="str">
+      <c r="D27" s="123" t="str">
         <f>Costs_init!L40</f>
         <v/>
       </c>
@@ -34261,7 +34252,7 @@
       <c r="C28" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="D28" s="136">
+      <c r="D28" s="123">
         <f>Costs_init!L41</f>
         <v>242.93622841965473</v>
       </c>
@@ -34275,7 +34266,7 @@
       <c r="C29" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="D29" s="136">
+      <c r="D29" s="123">
         <f>Costs_init!L42</f>
         <v>182.20217131474107</v>
       </c>
@@ -34289,7 +34280,7 @@
       <c r="C30" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="D30" s="136">
+      <c r="D30" s="123">
         <f>SUM(Costs_init!L44:L50)</f>
         <v>5177.6603940540372</v>
       </c>
@@ -34303,7 +34294,7 @@
       <c r="C31" s="7" t="s">
         <v>66</v>
       </c>
-      <c r="D31" s="136"/>
+      <c r="D31" s="123"/>
       <c r="E31" s="112">
         <f>SUM(D32:D40)</f>
         <v>1364.1486868492418</v>
@@ -34317,7 +34308,7 @@
       <c r="C32" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="D32" s="136">
+      <c r="D32" s="123">
         <f>Costs_init!L52</f>
         <v>200.52725668753558</v>
       </c>
@@ -34331,7 +34322,7 @@
       <c r="C33" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="D33" s="136">
+      <c r="D33" s="123">
         <f>Costs_init!L53</f>
         <v>150.39544251565169</v>
       </c>
@@ -34345,7 +34336,7 @@
       <c r="C34" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="D34" s="136">
+      <c r="D34" s="123">
         <f>Costs_init!L54</f>
         <v>250.6590708594195</v>
       </c>
@@ -34359,7 +34350,7 @@
       <c r="C35" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="D35" s="136">
+      <c r="D35" s="123">
         <f>Costs_init!L55</f>
         <v>150.39544251565169</v>
       </c>
@@ -34373,7 +34364,7 @@
       <c r="C36" s="1" t="s">
         <v>196</v>
       </c>
-      <c r="D36" s="136">
+      <c r="D36" s="123">
         <f>Costs_init!L56</f>
         <v>150.39544251565169</v>
       </c>
@@ -34387,7 +34378,7 @@
       <c r="C37" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="D37" s="136">
+      <c r="D37" s="123">
         <f>Costs_init!L57</f>
         <v>100.26362834376779</v>
       </c>
@@ -34401,7 +34392,7 @@
       <c r="C38" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D38" s="136">
+      <c r="D38" s="123">
         <f>Costs_init!L58</f>
         <v>150.39544251565169</v>
       </c>
@@ -34415,7 +34406,7 @@
       <c r="C39" s="1" t="s">
         <v>193</v>
       </c>
-      <c r="D39" s="136">
+      <c r="D39" s="123">
         <f>Costs_init!L59</f>
         <v>100.26362834376779</v>
       </c>
@@ -34429,7 +34420,7 @@
       <c r="C40" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="D40" s="136">
+      <c r="D40" s="123">
         <f>Costs_init!L60</f>
         <v>110.85333255214437</v>
       </c>
@@ -34443,7 +34434,7 @@
       <c r="C41" s="7" t="s">
         <v>74</v>
       </c>
-      <c r="D41" s="136" t="str">
+      <c r="D41" s="123" t="str">
         <f>Costs_init!L61</f>
         <v/>
       </c>
@@ -34460,7 +34451,7 @@
       <c r="C42" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="D42" s="136">
+      <c r="D42" s="123">
         <f>Costs_init!L62</f>
         <v>61.362125344774746</v>
       </c>
@@ -34474,7 +34465,7 @@
       <c r="C43" s="1" t="s">
         <v>76</v>
       </c>
-      <c r="D43" s="136">
+      <c r="D43" s="123">
         <f>Costs_init!L63</f>
         <v>61.362125344774746</v>
       </c>
@@ -34488,7 +34479,7 @@
       <c r="C44" s="1" t="s">
         <v>77</v>
       </c>
-      <c r="D44" s="136">
+      <c r="D44" s="123">
         <f>Costs_init!L64</f>
         <v>56.800459339114127</v>
       </c>
@@ -34502,7 +34493,7 @@
       <c r="C45" s="1" t="s">
         <v>78</v>
       </c>
-      <c r="D45" s="136">
+      <c r="D45" s="123">
         <f>Costs_init!L65</f>
         <v>113.60091867822825</v>
       </c>
@@ -34516,7 +34507,7 @@
       <c r="C46" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="D46" s="136">
+      <c r="D46" s="123">
         <f>Costs_init!L66</f>
         <v>122.72425068954949</v>
       </c>
@@ -34530,7 +34521,7 @@
       <c r="C47" s="1" t="s">
         <v>80</v>
       </c>
-      <c r="D47" s="136">
+      <c r="D47" s="123">
         <f>Costs_init!L67</f>
         <v>161.21780751992031</v>
       </c>
@@ -34544,7 +34535,7 @@
       <c r="C48" s="1" t="s">
         <v>81</v>
       </c>
-      <c r="D48" s="136">
+      <c r="D48" s="123">
         <f>Costs_init!L68</f>
         <v>303.67028552456838</v>
       </c>
@@ -34558,7 +34549,7 @@
       <c r="C49" s="1" t="s">
         <v>82</v>
       </c>
-      <c r="D49" s="136">
+      <c r="D49" s="123">
         <f>Costs_init!L69</f>
         <v>277.13333138036091</v>
       </c>
@@ -34572,7 +34563,7 @@
       <c r="C50" s="1" t="s">
         <v>83</v>
       </c>
-      <c r="D50" s="136">
+      <c r="D50" s="123">
         <f>Costs_init!L70</f>
         <v>110.85333255214437</v>
       </c>
@@ -34586,7 +34577,7 @@
       <c r="C51" s="1" t="s">
         <v>84</v>
       </c>
-      <c r="D51" s="136">
+      <c r="D51" s="123">
         <f>Costs_init!L71</f>
         <v>277.13333138036091</v>
       </c>
@@ -34600,7 +34591,7 @@
       <c r="C52" s="1" t="s">
         <v>85</v>
       </c>
-      <c r="D52" s="136">
+      <c r="D52" s="123">
         <f>Costs_init!L72</f>
         <v>122.72425068954949</v>
       </c>
@@ -34614,19 +34605,19 @@
       <c r="C53" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="D53" s="136">
+      <c r="D53" s="123">
         <f>Costs_init!L73</f>
         <v>61.362125344774746</v>
       </c>
       <c r="E53" s="113"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="119" t="s">
+      <c r="A54" s="126" t="s">
         <v>4</v>
       </c>
-      <c r="B54" s="120"/>
-      <c r="C54" s="120"/>
-      <c r="D54" s="120"/>
+      <c r="B54" s="127"/>
+      <c r="C54" s="127"/>
+      <c r="D54" s="127"/>
       <c r="E54" s="114">
         <f>SUM(E3:E53)</f>
         <v>16500.517352669427</v>

</xml_diff>

<commit_message>
docs: documents final budget and final planning
</commit_message>
<xml_diff>
--- a/docs/budget.xlsx
+++ b/docs/budget.xlsx
@@ -8,14 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Desktop\proyectos\IRBoard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{965A530D-4CE8-438C-B313-7FE2C2223067}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE692509-35D9-4BFA-B51B-C27FC9234824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Company definition" sheetId="2" r:id="rId1"/>
     <sheet name="Costs_init" sheetId="1" r:id="rId2"/>
     <sheet name="Client_init" sheetId="5" r:id="rId3"/>
+    <sheet name="Costs_final" sheetId="6" r:id="rId4"/>
+    <sheet name="Client_final" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="571" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="216">
   <si>
     <t>I1</t>
   </si>
@@ -1335,6 +1337,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1362,7 +1365,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -31004,27 +31006,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="129" t="s">
+      <c r="A1" s="130" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="130"/>
-      <c r="D1" s="130"/>
-      <c r="E1" s="130"/>
-      <c r="F1" s="130"/>
-      <c r="G1" s="130"/>
-      <c r="H1" s="130"/>
-      <c r="I1" s="130"/>
-      <c r="J1" s="130"/>
-      <c r="K1" s="131"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
+      <c r="F1" s="131"/>
+      <c r="G1" s="131"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="131"/>
+      <c r="J1" s="131"/>
+      <c r="K1" s="132"/>
       <c r="L1" s="125" t="s">
         <v>213</v>
       </c>
-      <c r="N1" s="126" t="s">
+      <c r="N1" s="127" t="s">
         <v>203</v>
       </c>
-      <c r="O1" s="127"/>
-      <c r="P1" s="128"/>
+      <c r="O1" s="128"/>
+      <c r="P1" s="129"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -31222,10 +31224,10 @@
       </c>
       <c r="K6" s="112"/>
       <c r="L6" s="110"/>
-      <c r="N6" s="126" t="s">
+      <c r="N6" s="127" t="s">
         <v>115</v>
       </c>
-      <c r="O6" s="127"/>
+      <c r="O6" s="128"/>
       <c r="P6" s="122">
         <f>SUM(P3:P5)</f>
         <v>16498.77169083678</v>
@@ -31339,7 +31341,7 @@
       <c r="O9" t="s">
         <v>214</v>
       </c>
-      <c r="P9" s="135">
+      <c r="P9" s="126">
         <f>SUM(F4:F73)</f>
         <v>300</v>
       </c>
@@ -33602,18 +33604,18 @@
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A74" s="126" t="s">
+      <c r="A74" s="127" t="s">
         <v>4</v>
       </c>
-      <c r="B74" s="127"/>
-      <c r="C74" s="127"/>
-      <c r="D74" s="127"/>
-      <c r="E74" s="127"/>
-      <c r="F74" s="127"/>
-      <c r="G74" s="127"/>
-      <c r="H74" s="127"/>
-      <c r="I74" s="127"/>
-      <c r="J74" s="127"/>
+      <c r="B74" s="128"/>
+      <c r="C74" s="128"/>
+      <c r="D74" s="128"/>
+      <c r="E74" s="128"/>
+      <c r="F74" s="128"/>
+      <c r="G74" s="128"/>
+      <c r="H74" s="128"/>
+      <c r="I74" s="128"/>
+      <c r="J74" s="128"/>
       <c r="K74" s="114">
         <f>SUM(K3:K73)</f>
         <v>13026.517352669423</v>
@@ -33628,19 +33630,19 @@
       <c r="L75" s="2"/>
     </row>
     <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="132" t="s">
+      <c r="A76" s="133" t="s">
         <v>192</v>
       </c>
-      <c r="B76" s="133"/>
-      <c r="C76" s="133"/>
-      <c r="D76" s="133"/>
-      <c r="E76" s="133"/>
-      <c r="F76" s="133"/>
-      <c r="G76" s="133"/>
-      <c r="H76" s="133"/>
-      <c r="I76" s="133"/>
-      <c r="J76" s="133"/>
-      <c r="K76" s="134"/>
+      <c r="B76" s="134"/>
+      <c r="C76" s="134"/>
+      <c r="D76" s="134"/>
+      <c r="E76" s="134"/>
+      <c r="F76" s="134"/>
+      <c r="G76" s="134"/>
+      <c r="H76" s="134"/>
+      <c r="I76" s="134"/>
+      <c r="J76" s="134"/>
+      <c r="K76" s="135"/>
       <c r="L76" s="124"/>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.3">
@@ -33759,18 +33761,18 @@
       <c r="L80" s="116"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A81" s="126" t="s">
+      <c r="A81" s="127" t="s">
         <v>4</v>
       </c>
-      <c r="B81" s="127"/>
-      <c r="C81" s="127"/>
-      <c r="D81" s="127"/>
-      <c r="E81" s="127"/>
-      <c r="F81" s="127"/>
-      <c r="G81" s="127"/>
-      <c r="H81" s="127"/>
-      <c r="I81" s="127"/>
-      <c r="J81" s="127"/>
+      <c r="B81" s="128"/>
+      <c r="C81" s="128"/>
+      <c r="D81" s="128"/>
+      <c r="E81" s="128"/>
+      <c r="F81" s="128"/>
+      <c r="G81" s="128"/>
+      <c r="H81" s="128"/>
+      <c r="I81" s="128"/>
+      <c r="J81" s="128"/>
       <c r="K81" s="114">
         <f>SUM(K78:K80)</f>
         <v>172.5</v>
@@ -33820,18 +33822,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="129" t="s">
+      <c r="A1" s="130" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="130"/>
-      <c r="C1" s="130"/>
-      <c r="D1" s="130"/>
-      <c r="E1" s="131"/>
-      <c r="G1" s="126" t="s">
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="132"/>
+      <c r="G1" s="127" t="s">
         <v>209</v>
       </c>
-      <c r="H1" s="127"/>
-      <c r="I1" s="128"/>
+      <c r="H1" s="128"/>
+      <c r="I1" s="129"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -33896,10 +33898,10 @@
         <v>122.72425068954949</v>
       </c>
       <c r="E4" s="112"/>
-      <c r="G4" s="126" t="s">
+      <c r="G4" s="127" t="s">
         <v>115</v>
       </c>
-      <c r="H4" s="127"/>
+      <c r="H4" s="128"/>
       <c r="I4" s="122">
         <f>SUM(I3)</f>
         <v>16500.517352669427</v>
@@ -34612,12 +34614,12 @@
       <c r="E53" s="113"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="126" t="s">
+      <c r="A54" s="127" t="s">
         <v>4</v>
       </c>
-      <c r="B54" s="127"/>
-      <c r="C54" s="127"/>
-      <c r="D54" s="127"/>
+      <c r="B54" s="128"/>
+      <c r="C54" s="128"/>
+      <c r="D54" s="128"/>
       <c r="E54" s="114">
         <f>SUM(E3:E53)</f>
         <v>16500.517352669427</v>
@@ -34640,4 +34642,3663 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C034FB62-BD60-4D19-91EB-FF898F716C5A}">
+  <dimension ref="A1:R82"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="38.5546875" customWidth="1"/>
+    <col min="5" max="5" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="14.109375" customWidth="1"/>
+    <col min="14" max="14" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="33" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="23.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="130" t="s">
+        <v>191</v>
+      </c>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
+      <c r="F1" s="131"/>
+      <c r="G1" s="131"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="131"/>
+      <c r="J1" s="131"/>
+      <c r="K1" s="132"/>
+      <c r="L1" s="125" t="s">
+        <v>213</v>
+      </c>
+      <c r="N1" s="127" t="s">
+        <v>203</v>
+      </c>
+      <c r="O1" s="128"/>
+      <c r="P1" s="129"/>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F2" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I2" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="J2" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="K2" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="L2" s="118"/>
+      <c r="N2" s="119" t="s">
+        <v>205</v>
+      </c>
+      <c r="O2" s="118" t="s">
+        <v>204</v>
+      </c>
+      <c r="P2" s="120" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="H3" s="111" t="str">
+        <f t="shared" ref="H3:H66" si="0">_xlfn.XLOOKUP(E3,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <v/>
+      </c>
+      <c r="I3" s="111" t="str">
+        <f>IFERROR(H3*F3,"")</f>
+        <v/>
+      </c>
+      <c r="K3" s="115">
+        <f>SUM(J4:J19)</f>
+        <v>1194.7710082745937</v>
+      </c>
+      <c r="L3" s="110" t="str">
+        <f>IFERROR(I3+($P$10*F3),"")</f>
+        <v/>
+      </c>
+      <c r="N3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="O3" t="s">
+        <v>206</v>
+      </c>
+      <c r="P3" s="121">
+        <f>K74</f>
+        <v>13383.612572529586</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A4" s="5"/>
+      <c r="B4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="6"/>
+      <c r="D4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E4" t="s">
+        <v>104</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4" t="s">
+        <v>103</v>
+      </c>
+      <c r="H4" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I4" s="111">
+        <f t="shared" ref="I4:I67" si="1">IFERROR(H4*F4,"")</f>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="J4" s="111">
+        <f>I4</f>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="K4" s="112"/>
+      <c r="L4" s="110">
+        <f t="shared" ref="L4:L67" si="2">IFERROR(I4+($P$10*F4),"")</f>
+        <v>122.5442506895495</v>
+      </c>
+      <c r="N4" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="O4" t="s">
+        <v>207</v>
+      </c>
+      <c r="P4" s="121">
+        <f>K81</f>
+        <v>172.5</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A5" s="5"/>
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="6"/>
+      <c r="D5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" t="s">
+        <v>104</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5" t="s">
+        <v>103</v>
+      </c>
+      <c r="H5" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I5" s="111">
+        <f t="shared" si="1"/>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="J5" s="111">
+        <f>I5</f>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="K5" s="112"/>
+      <c r="L5" s="110">
+        <f t="shared" si="2"/>
+        <v>122.5442506895495</v>
+      </c>
+      <c r="N5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="O5" t="s">
+        <v>208</v>
+      </c>
+      <c r="P5" s="112">
+        <f>0.25*(P3+P4)</f>
+        <v>3389.0281431323965</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A6" s="5"/>
+      <c r="B6" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="6"/>
+      <c r="D6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H6" s="111" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I6" s="111" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J6" s="111">
+        <f>SUM(I7:I19)</f>
+        <v>995.64250689549476</v>
+      </c>
+      <c r="K6" s="112"/>
+      <c r="L6" s="110"/>
+      <c r="N6" s="127" t="s">
+        <v>115</v>
+      </c>
+      <c r="O6" s="128"/>
+      <c r="P6" s="122">
+        <f>SUM(P3:P5)</f>
+        <v>16945.140715661983</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A7" s="5"/>
+      <c r="B7" s="6"/>
+      <c r="C7" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7">
+        <v>1</v>
+      </c>
+      <c r="G7" t="s">
+        <v>103</v>
+      </c>
+      <c r="H7" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I7" s="111">
+        <f t="shared" si="1"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J7" s="111"/>
+      <c r="K7" s="112"/>
+      <c r="L7" s="110">
+        <f t="shared" si="2"/>
+        <v>61.27212534477475</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A8" s="5"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E8" t="s">
+        <v>104</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8" t="s">
+        <v>103</v>
+      </c>
+      <c r="H8" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I8" s="111">
+        <f t="shared" si="1"/>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="J8" s="111"/>
+      <c r="K8" s="112"/>
+      <c r="L8" s="110">
+        <f t="shared" si="2"/>
+        <v>122.5442506895495</v>
+      </c>
+      <c r="O8" t="s">
+        <v>211</v>
+      </c>
+      <c r="P8" s="111">
+        <f>P6-P3</f>
+        <v>3561.5281431323965</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A9" s="5"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E9" t="s">
+        <v>104</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+      <c r="G9" t="s">
+        <v>103</v>
+      </c>
+      <c r="H9" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I9" s="111">
+        <f t="shared" si="1"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J9" s="111"/>
+      <c r="K9" s="112"/>
+      <c r="L9" s="110">
+        <f t="shared" si="2"/>
+        <v>61.27212534477475</v>
+      </c>
+      <c r="O9" t="s">
+        <v>214</v>
+      </c>
+      <c r="P9" s="126">
+        <f>SUM(F4:F73)</f>
+        <v>310</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A10" s="5"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" t="s">
+        <v>104</v>
+      </c>
+      <c r="F10">
+        <v>2</v>
+      </c>
+      <c r="G10" t="s">
+        <v>103</v>
+      </c>
+      <c r="H10" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I10" s="111">
+        <f t="shared" si="1"/>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="J10" s="111"/>
+      <c r="K10" s="112"/>
+      <c r="L10" s="110">
+        <f t="shared" si="2"/>
+        <v>122.5442506895495</v>
+      </c>
+      <c r="O10" t="s">
+        <v>215</v>
+      </c>
+      <c r="P10" s="123">
+        <f>ROUNDUP(P8/P9,2)</f>
+        <v>11.49</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A11" s="5"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>103</v>
+      </c>
+      <c r="H11" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I11" s="111">
+        <f t="shared" si="1"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J11" s="111"/>
+      <c r="K11" s="112"/>
+      <c r="L11" s="110">
+        <f t="shared" si="2"/>
+        <v>61.27212534477475</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A12" s="5"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="E12" t="s">
+        <v>104</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12" t="s">
+        <v>103</v>
+      </c>
+      <c r="H12" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I12" s="111">
+        <f t="shared" si="1"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J12" s="111"/>
+      <c r="K12" s="112"/>
+      <c r="L12" s="110">
+        <f t="shared" si="2"/>
+        <v>61.27212534477475</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A13" s="5"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="E13" t="s">
+        <v>104</v>
+      </c>
+      <c r="F13">
+        <v>2</v>
+      </c>
+      <c r="G13" t="s">
+        <v>103</v>
+      </c>
+      <c r="H13" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I13" s="111">
+        <f t="shared" si="1"/>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="J13" s="111"/>
+      <c r="K13" s="112"/>
+      <c r="L13" s="110">
+        <f t="shared" si="2"/>
+        <v>122.5442506895495</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A14" s="5"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" t="s">
+        <v>104</v>
+      </c>
+      <c r="F14">
+        <v>2</v>
+      </c>
+      <c r="G14" t="s">
+        <v>103</v>
+      </c>
+      <c r="H14" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I14" s="111">
+        <f t="shared" si="1"/>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="J14" s="111"/>
+      <c r="K14" s="112"/>
+      <c r="L14" s="110">
+        <f t="shared" si="2"/>
+        <v>122.5442506895495</v>
+      </c>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A15" s="5"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E15" t="s">
+        <v>104</v>
+      </c>
+      <c r="F15">
+        <v>2</v>
+      </c>
+      <c r="G15" t="s">
+        <v>103</v>
+      </c>
+      <c r="H15" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I15" s="111">
+        <f t="shared" si="1"/>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="J15" s="111"/>
+      <c r="K15" s="112"/>
+      <c r="L15" s="110">
+        <f t="shared" si="2"/>
+        <v>122.5442506895495</v>
+      </c>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A16" s="5"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E16" t="s">
+        <v>104</v>
+      </c>
+      <c r="F16">
+        <v>2</v>
+      </c>
+      <c r="G16" t="s">
+        <v>103</v>
+      </c>
+      <c r="H16" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I16" s="111">
+        <f t="shared" si="1"/>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="J16" s="111"/>
+      <c r="K16" s="112"/>
+      <c r="L16" s="110">
+        <f t="shared" si="2"/>
+        <v>122.5442506895495</v>
+      </c>
+    </row>
+    <row r="17" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A17" s="5"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E17" t="s">
+        <v>104</v>
+      </c>
+      <c r="F17">
+        <v>1</v>
+      </c>
+      <c r="G17" t="s">
+        <v>103</v>
+      </c>
+      <c r="H17" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I17" s="111">
+        <f t="shared" si="1"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J17" s="111"/>
+      <c r="K17" s="112"/>
+      <c r="L17" s="110">
+        <f t="shared" si="2"/>
+        <v>61.27212534477475</v>
+      </c>
+    </row>
+    <row r="18" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A18" s="5"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" t="s">
+        <v>104</v>
+      </c>
+      <c r="F18">
+        <v>1</v>
+      </c>
+      <c r="G18" t="s">
+        <v>103</v>
+      </c>
+      <c r="H18" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I18" s="111">
+        <f t="shared" si="1"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J18" s="111"/>
+      <c r="K18" s="112"/>
+      <c r="L18" s="110">
+        <f t="shared" si="2"/>
+        <v>61.27212534477475</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A19" s="5"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E19" t="s">
+        <v>104</v>
+      </c>
+      <c r="F19">
+        <v>2</v>
+      </c>
+      <c r="G19" t="s">
+        <v>103</v>
+      </c>
+      <c r="H19" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I19" s="111">
+        <f t="shared" si="1"/>
+        <v>99.564250689549496</v>
+      </c>
+      <c r="J19" s="111"/>
+      <c r="K19" s="112"/>
+      <c r="L19" s="110">
+        <f t="shared" si="2"/>
+        <v>122.5442506895495</v>
+      </c>
+      <c r="Q19" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="R19" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="20" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A20" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H20" s="111" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I20" s="111" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J20" s="111"/>
+      <c r="K20" s="112">
+        <f>SUM(J21:J30)</f>
+        <v>2433.690244536559</v>
+      </c>
+      <c r="L20" s="110" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="Q20" t="s">
+        <v>104</v>
+      </c>
+      <c r="R20" s="110">
+        <f>'Company definition'!F82</f>
+        <v>49.782125344774748</v>
+      </c>
+    </row>
+    <row r="21" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A21" s="5"/>
+      <c r="B21" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C21" s="6"/>
+      <c r="D21" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" t="s">
+        <v>106</v>
+      </c>
+      <c r="F21">
+        <v>1</v>
+      </c>
+      <c r="G21" t="s">
+        <v>103</v>
+      </c>
+      <c r="H21" s="111">
+        <f t="shared" si="0"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="I21" s="111">
+        <f t="shared" si="1"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="J21" s="111">
+        <f t="shared" ref="J21:J30" si="3">I21</f>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="K21" s="112"/>
+      <c r="L21" s="110">
+        <f t="shared" si="2"/>
+        <v>53.64926917330677</v>
+      </c>
+      <c r="Q21" t="s">
+        <v>107</v>
+      </c>
+      <c r="R21" s="110">
+        <f>'Company definition'!F85</f>
+        <v>45.220459339114129</v>
+      </c>
+    </row>
+    <row r="22" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A22" s="5"/>
+      <c r="B22" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C22" s="6"/>
+      <c r="D22" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" t="s">
+        <v>107</v>
+      </c>
+      <c r="F22">
+        <v>4</v>
+      </c>
+      <c r="G22" t="s">
+        <v>103</v>
+      </c>
+      <c r="H22" s="111">
+        <f t="shared" si="0"/>
+        <v>45.220459339114129</v>
+      </c>
+      <c r="I22" s="111">
+        <f t="shared" si="1"/>
+        <v>180.88183735645651</v>
+      </c>
+      <c r="J22" s="111">
+        <f t="shared" si="3"/>
+        <v>180.88183735645651</v>
+      </c>
+      <c r="K22" s="112"/>
+      <c r="L22" s="110">
+        <f t="shared" si="2"/>
+        <v>226.84183735645652</v>
+      </c>
+      <c r="Q22" t="s">
+        <v>106</v>
+      </c>
+      <c r="R22" s="110">
+        <f>'Company definition'!F84</f>
+        <v>42.159269173306768</v>
+      </c>
+    </row>
+    <row r="23" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A23" s="5"/>
+      <c r="B23" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C23" s="6"/>
+      <c r="D23" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="E23" t="s">
+        <v>106</v>
+      </c>
+      <c r="F23">
+        <v>1</v>
+      </c>
+      <c r="G23" t="s">
+        <v>103</v>
+      </c>
+      <c r="H23" s="111">
+        <f t="shared" si="0"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="I23" s="111">
+        <f t="shared" si="1"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="J23" s="111">
+        <f t="shared" si="3"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="K23" s="112"/>
+      <c r="L23" s="110">
+        <f t="shared" si="2"/>
+        <v>53.64926917330677</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>108</v>
+      </c>
+      <c r="R23" s="110">
+        <f>'Company definition'!F86</f>
+        <v>49.154057104913683</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A24" s="5"/>
+      <c r="B24" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C24" s="6"/>
+      <c r="D24" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E24" t="s">
+        <v>106</v>
+      </c>
+      <c r="F24">
+        <v>1</v>
+      </c>
+      <c r="G24" t="s">
+        <v>103</v>
+      </c>
+      <c r="H24" s="111">
+        <f t="shared" si="0"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="I24" s="111">
+        <f t="shared" si="1"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="J24" s="111">
+        <f t="shared" si="3"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="K24" s="112"/>
+      <c r="L24" s="110">
+        <f t="shared" si="2"/>
+        <v>53.64926917330677</v>
+      </c>
+      <c r="Q24" t="s">
+        <v>109</v>
+      </c>
+      <c r="R24" s="110">
+        <f>'Company definition'!F87</f>
+        <v>43.846666276072185</v>
+      </c>
+    </row>
+    <row r="25" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A25" s="5"/>
+      <c r="B25" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C25" s="6"/>
+      <c r="D25" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E25" t="s">
+        <v>106</v>
+      </c>
+      <c r="F25">
+        <v>2</v>
+      </c>
+      <c r="G25" t="s">
+        <v>103</v>
+      </c>
+      <c r="H25" s="111">
+        <f t="shared" si="0"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="I25" s="111">
+        <f t="shared" si="1"/>
+        <v>84.318538346613536</v>
+      </c>
+      <c r="J25" s="111">
+        <f t="shared" si="3"/>
+        <v>84.318538346613536</v>
+      </c>
+      <c r="K25" s="112"/>
+      <c r="L25" s="110">
+        <f t="shared" si="2"/>
+        <v>107.29853834661354</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>110</v>
+      </c>
+      <c r="R25" s="110">
+        <f>'Company definition'!F88</f>
+        <v>38.551814171883898</v>
+      </c>
+    </row>
+    <row r="26" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A26" s="5"/>
+      <c r="B26" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C26" s="6"/>
+      <c r="D26" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="E26" t="s">
+        <v>107</v>
+      </c>
+      <c r="F26">
+        <v>6</v>
+      </c>
+      <c r="G26" t="s">
+        <v>103</v>
+      </c>
+      <c r="H26" s="111">
+        <f t="shared" si="0"/>
+        <v>45.220459339114129</v>
+      </c>
+      <c r="I26" s="111">
+        <f t="shared" si="1"/>
+        <v>271.32275603468474</v>
+      </c>
+      <c r="J26" s="111">
+        <f t="shared" si="3"/>
+        <v>271.32275603468474</v>
+      </c>
+      <c r="K26" s="112"/>
+      <c r="L26" s="110">
+        <f t="shared" si="2"/>
+        <v>340.26275603468474</v>
+      </c>
+    </row>
+    <row r="27" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A27" s="5"/>
+      <c r="B27" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C27" s="6"/>
+      <c r="D27" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="E27" t="s">
+        <v>106</v>
+      </c>
+      <c r="F27">
+        <v>22</v>
+      </c>
+      <c r="G27" t="s">
+        <v>103</v>
+      </c>
+      <c r="H27" s="111">
+        <f t="shared" si="0"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="I27" s="111">
+        <f t="shared" si="1"/>
+        <v>927.5039218127489</v>
+      </c>
+      <c r="J27" s="111">
+        <f t="shared" si="3"/>
+        <v>927.5039218127489</v>
+      </c>
+      <c r="K27" s="112"/>
+      <c r="L27" s="110">
+        <f t="shared" si="2"/>
+        <v>1180.283921812749</v>
+      </c>
+    </row>
+    <row r="28" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A28" s="5"/>
+      <c r="B28" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C28" s="6"/>
+      <c r="D28" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E28" t="s">
+        <v>106</v>
+      </c>
+      <c r="F28">
+        <v>8</v>
+      </c>
+      <c r="G28" t="s">
+        <v>103</v>
+      </c>
+      <c r="H28" s="111">
+        <f t="shared" si="0"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="I28" s="111">
+        <f t="shared" si="1"/>
+        <v>337.27415338645415</v>
+      </c>
+      <c r="J28" s="111">
+        <f t="shared" si="3"/>
+        <v>337.27415338645415</v>
+      </c>
+      <c r="K28" s="112"/>
+      <c r="L28" s="110">
+        <f t="shared" si="2"/>
+        <v>429.19415338645416</v>
+      </c>
+    </row>
+    <row r="29" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A29" s="5"/>
+      <c r="B29" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C29" s="6"/>
+      <c r="D29" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E29" t="s">
+        <v>106</v>
+      </c>
+      <c r="F29">
+        <v>4</v>
+      </c>
+      <c r="G29" t="s">
+        <v>103</v>
+      </c>
+      <c r="H29" s="111">
+        <f t="shared" si="0"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="I29" s="111">
+        <f t="shared" si="1"/>
+        <v>168.63707669322707</v>
+      </c>
+      <c r="J29" s="111">
+        <f t="shared" si="3"/>
+        <v>168.63707669322707</v>
+      </c>
+      <c r="K29" s="112"/>
+      <c r="L29" s="110">
+        <f t="shared" si="2"/>
+        <v>214.59707669322708</v>
+      </c>
+    </row>
+    <row r="30" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A30" s="5"/>
+      <c r="B30" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C30" s="6"/>
+      <c r="D30" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="E30" t="s">
+        <v>106</v>
+      </c>
+      <c r="F30">
+        <v>8</v>
+      </c>
+      <c r="G30" t="s">
+        <v>103</v>
+      </c>
+      <c r="H30" s="111">
+        <f t="shared" si="0"/>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="I30" s="111">
+        <f t="shared" si="1"/>
+        <v>337.27415338645415</v>
+      </c>
+      <c r="J30" s="111">
+        <f t="shared" si="3"/>
+        <v>337.27415338645415</v>
+      </c>
+      <c r="K30" s="112"/>
+      <c r="L30" s="110">
+        <f t="shared" si="2"/>
+        <v>429.19415338645416</v>
+      </c>
+    </row>
+    <row r="31" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A31" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="6"/>
+      <c r="D31" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="H31" s="111" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I31" s="111" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J31" s="111"/>
+      <c r="K31" s="112">
+        <f>SUM(J32:J38)</f>
+        <v>2361.0626646076757</v>
+      </c>
+      <c r="L31" s="110" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="1:18" x14ac:dyDescent="0.3">
+      <c r="A32" s="5"/>
+      <c r="B32" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="6"/>
+      <c r="D32" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E32" t="s">
+        <v>108</v>
+      </c>
+      <c r="F32">
+        <v>10</v>
+      </c>
+      <c r="G32" t="s">
+        <v>103</v>
+      </c>
+      <c r="H32" s="111">
+        <f t="shared" si="0"/>
+        <v>49.154057104913683</v>
+      </c>
+      <c r="I32" s="111">
+        <f t="shared" si="1"/>
+        <v>491.54057104913682</v>
+      </c>
+      <c r="J32" s="111">
+        <f t="shared" ref="J32:J38" si="4">I32</f>
+        <v>491.54057104913682</v>
+      </c>
+      <c r="K32" s="112"/>
+      <c r="L32" s="110">
+        <f t="shared" si="2"/>
+        <v>606.44057104913679</v>
+      </c>
+    </row>
+    <row r="33" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A33" s="5"/>
+      <c r="B33" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="6"/>
+      <c r="D33" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33" t="s">
+        <v>110</v>
+      </c>
+      <c r="F33">
+        <v>3</v>
+      </c>
+      <c r="G33" t="s">
+        <v>103</v>
+      </c>
+      <c r="H33" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I33" s="111">
+        <f t="shared" si="1"/>
+        <v>115.65544251565169</v>
+      </c>
+      <c r="J33" s="111">
+        <f t="shared" si="4"/>
+        <v>115.65544251565169</v>
+      </c>
+      <c r="K33" s="112"/>
+      <c r="L33" s="110">
+        <f t="shared" si="2"/>
+        <v>150.12544251565168</v>
+      </c>
+    </row>
+    <row r="34" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A34" s="5"/>
+      <c r="B34" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="6"/>
+      <c r="D34" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="E34" t="s">
+        <v>109</v>
+      </c>
+      <c r="F34">
+        <v>8</v>
+      </c>
+      <c r="G34" t="s">
+        <v>103</v>
+      </c>
+      <c r="H34" s="111">
+        <f t="shared" si="0"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I34" s="111">
+        <f t="shared" si="1"/>
+        <v>350.77333020857748</v>
+      </c>
+      <c r="J34" s="111">
+        <f t="shared" si="4"/>
+        <v>350.77333020857748</v>
+      </c>
+      <c r="K34" s="112"/>
+      <c r="L34" s="110">
+        <f t="shared" si="2"/>
+        <v>442.69333020857749</v>
+      </c>
+    </row>
+    <row r="35" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A35" s="5"/>
+      <c r="B35" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C35" s="6"/>
+      <c r="D35" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E35" t="s">
+        <v>109</v>
+      </c>
+      <c r="F35">
+        <v>4</v>
+      </c>
+      <c r="G35" t="s">
+        <v>103</v>
+      </c>
+      <c r="H35" s="111">
+        <f t="shared" si="0"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I35" s="111">
+        <f t="shared" si="1"/>
+        <v>175.38666510428874</v>
+      </c>
+      <c r="J35" s="111">
+        <f t="shared" si="4"/>
+        <v>175.38666510428874</v>
+      </c>
+      <c r="K35" s="112"/>
+      <c r="L35" s="110">
+        <f t="shared" si="2"/>
+        <v>221.34666510428875</v>
+      </c>
+    </row>
+    <row r="36" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A36" s="5"/>
+      <c r="B36" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C36" s="6"/>
+      <c r="D36" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="E36" t="s">
+        <v>109</v>
+      </c>
+      <c r="F36">
+        <v>6</v>
+      </c>
+      <c r="G36" t="s">
+        <v>103</v>
+      </c>
+      <c r="H36" s="111">
+        <f t="shared" si="0"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I36" s="111">
+        <f t="shared" si="1"/>
+        <v>263.07999765643308</v>
+      </c>
+      <c r="J36" s="111">
+        <f t="shared" si="4"/>
+        <v>263.07999765643308</v>
+      </c>
+      <c r="K36" s="112"/>
+      <c r="L36" s="110">
+        <f t="shared" si="2"/>
+        <v>332.01999765643308</v>
+      </c>
+    </row>
+    <row r="37" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A37" s="5"/>
+      <c r="B37" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C37" s="6"/>
+      <c r="D37" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E37" t="s">
+        <v>109</v>
+      </c>
+      <c r="F37">
+        <v>12</v>
+      </c>
+      <c r="G37" t="s">
+        <v>103</v>
+      </c>
+      <c r="H37" s="111">
+        <f t="shared" si="0"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I37" s="111">
+        <f t="shared" si="1"/>
+        <v>526.15999531286616</v>
+      </c>
+      <c r="J37" s="111">
+        <f t="shared" si="4"/>
+        <v>526.15999531286616</v>
+      </c>
+      <c r="K37" s="112"/>
+      <c r="L37" s="110">
+        <f t="shared" si="2"/>
+        <v>664.03999531286615</v>
+      </c>
+    </row>
+    <row r="38" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A38" s="5"/>
+      <c r="B38" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" s="6"/>
+      <c r="D38" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E38" t="s">
+        <v>109</v>
+      </c>
+      <c r="F38">
+        <v>10</v>
+      </c>
+      <c r="G38" t="s">
+        <v>103</v>
+      </c>
+      <c r="H38" s="111">
+        <f t="shared" si="0"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I38" s="111">
+        <f t="shared" si="1"/>
+        <v>438.46666276072187</v>
+      </c>
+      <c r="J38" s="111">
+        <f t="shared" si="4"/>
+        <v>438.46666276072187</v>
+      </c>
+      <c r="K38" s="112"/>
+      <c r="L38" s="110">
+        <f t="shared" si="2"/>
+        <v>553.36666276072185</v>
+      </c>
+    </row>
+    <row r="39" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A39" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6"/>
+      <c r="D39" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E39" t="s">
+        <v>109</v>
+      </c>
+      <c r="F39">
+        <v>6</v>
+      </c>
+      <c r="G39" t="s">
+        <v>103</v>
+      </c>
+      <c r="H39" s="111">
+        <f t="shared" si="0"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I39" s="111">
+        <f t="shared" si="1"/>
+        <v>263.07999765643308</v>
+      </c>
+      <c r="J39" s="111">
+        <f>SUM(I39)</f>
+        <v>263.07999765643308</v>
+      </c>
+      <c r="K39" s="111">
+        <f>SUM(J39)</f>
+        <v>263.07999765643308</v>
+      </c>
+      <c r="L39" s="110">
+        <f t="shared" si="2"/>
+        <v>332.01999765643308</v>
+      </c>
+    </row>
+    <row r="40" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A40" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6"/>
+      <c r="D40" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="H40" s="111" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I40" s="111" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J40" s="111"/>
+      <c r="K40" s="112">
+        <f>SUM(J41:J50)</f>
+        <v>4485.1818305489533</v>
+      </c>
+      <c r="L40" s="110" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A41" s="5"/>
+      <c r="B41" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C41" s="6"/>
+      <c r="D41" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="E41" t="s">
+        <v>108</v>
+      </c>
+      <c r="F41">
+        <v>6</v>
+      </c>
+      <c r="G41" t="s">
+        <v>103</v>
+      </c>
+      <c r="H41" s="111">
+        <f t="shared" si="0"/>
+        <v>49.154057104913683</v>
+      </c>
+      <c r="I41" s="111">
+        <f t="shared" si="1"/>
+        <v>294.92434262948211</v>
+      </c>
+      <c r="J41" s="111">
+        <f>I41</f>
+        <v>294.92434262948211</v>
+      </c>
+      <c r="K41" s="112"/>
+      <c r="L41" s="110">
+        <f t="shared" si="2"/>
+        <v>363.86434262948211</v>
+      </c>
+    </row>
+    <row r="42" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A42" s="5"/>
+      <c r="B42" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" s="6"/>
+      <c r="D42" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E42" t="s">
+        <v>108</v>
+      </c>
+      <c r="F42">
+        <v>1</v>
+      </c>
+      <c r="G42" t="s">
+        <v>103</v>
+      </c>
+      <c r="H42" s="111">
+        <f t="shared" si="0"/>
+        <v>49.154057104913683</v>
+      </c>
+      <c r="I42" s="111">
+        <f t="shared" si="1"/>
+        <v>49.154057104913683</v>
+      </c>
+      <c r="J42" s="111">
+        <f>I42</f>
+        <v>49.154057104913683</v>
+      </c>
+      <c r="K42" s="112"/>
+      <c r="L42" s="110">
+        <f t="shared" si="2"/>
+        <v>60.644057104913685</v>
+      </c>
+    </row>
+    <row r="43" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A43" s="5"/>
+      <c r="B43" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C43" s="6"/>
+      <c r="D43" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="H43" s="111" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I43" s="111" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J43" s="111">
+        <f>SUM(I44:I50)</f>
+        <v>4141.1034308145572</v>
+      </c>
+      <c r="K43" s="112"/>
+      <c r="L43" s="110" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A44" s="5"/>
+      <c r="B44" s="6"/>
+      <c r="C44" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="E44" t="s">
+        <v>110</v>
+      </c>
+      <c r="F44">
+        <v>22</v>
+      </c>
+      <c r="G44" t="s">
+        <v>103</v>
+      </c>
+      <c r="H44" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I44" s="111">
+        <f t="shared" si="1"/>
+        <v>848.13991178144579</v>
+      </c>
+      <c r="J44" s="111"/>
+      <c r="K44" s="112"/>
+      <c r="L44" s="110">
+        <f t="shared" si="2"/>
+        <v>1100.9199117814458</v>
+      </c>
+    </row>
+    <row r="45" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="5"/>
+      <c r="B45" s="6"/>
+      <c r="C45" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="E45" t="s">
+        <v>110</v>
+      </c>
+      <c r="F45">
+        <v>6</v>
+      </c>
+      <c r="G45" t="s">
+        <v>103</v>
+      </c>
+      <c r="H45" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I45" s="111">
+        <f t="shared" si="1"/>
+        <v>231.31088503130337</v>
+      </c>
+      <c r="J45" s="111"/>
+      <c r="K45" s="112"/>
+      <c r="L45" s="110">
+        <f t="shared" si="2"/>
+        <v>300.25088503130337</v>
+      </c>
+    </row>
+    <row r="46" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="5"/>
+      <c r="B46" s="6"/>
+      <c r="C46" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E46" t="s">
+        <v>109</v>
+      </c>
+      <c r="F46">
+        <v>24</v>
+      </c>
+      <c r="G46" t="s">
+        <v>103</v>
+      </c>
+      <c r="H46" s="111">
+        <f t="shared" si="0"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I46" s="111">
+        <f t="shared" si="1"/>
+        <v>1052.3199906257323</v>
+      </c>
+      <c r="J46" s="111"/>
+      <c r="K46" s="112"/>
+      <c r="L46" s="110">
+        <f t="shared" si="2"/>
+        <v>1328.0799906257323</v>
+      </c>
+    </row>
+    <row r="47" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A47" s="5"/>
+      <c r="B47" s="6"/>
+      <c r="C47" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="E47" t="s">
+        <v>110</v>
+      </c>
+      <c r="F47">
+        <v>12</v>
+      </c>
+      <c r="G47" t="s">
+        <v>103</v>
+      </c>
+      <c r="H47" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I47" s="111">
+        <f t="shared" si="1"/>
+        <v>462.62177006260674</v>
+      </c>
+      <c r="J47" s="111"/>
+      <c r="K47" s="112"/>
+      <c r="L47" s="110">
+        <f t="shared" si="2"/>
+        <v>600.50177006260674</v>
+      </c>
+    </row>
+    <row r="48" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A48" s="5"/>
+      <c r="B48" s="6"/>
+      <c r="C48" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="E48" t="s">
+        <v>109</v>
+      </c>
+      <c r="F48">
+        <v>20</v>
+      </c>
+      <c r="G48" t="s">
+        <v>103</v>
+      </c>
+      <c r="H48" s="111">
+        <f t="shared" si="0"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I48" s="111">
+        <f t="shared" si="1"/>
+        <v>876.93332552144375</v>
+      </c>
+      <c r="J48" s="111"/>
+      <c r="K48" s="112"/>
+      <c r="L48" s="110">
+        <f t="shared" si="2"/>
+        <v>1106.7333255214437</v>
+      </c>
+    </row>
+    <row r="49" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A49" s="5"/>
+      <c r="B49" s="6"/>
+      <c r="C49" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="E49" t="s">
+        <v>109</v>
+      </c>
+      <c r="F49">
+        <v>10</v>
+      </c>
+      <c r="G49" t="s">
+        <v>103</v>
+      </c>
+      <c r="H49" s="111">
+        <f t="shared" si="0"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I49" s="111">
+        <f t="shared" si="1"/>
+        <v>438.46666276072187</v>
+      </c>
+      <c r="J49" s="111"/>
+      <c r="K49" s="112"/>
+      <c r="L49" s="110">
+        <f t="shared" si="2"/>
+        <v>553.36666276072185</v>
+      </c>
+    </row>
+    <row r="50" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A50" s="5"/>
+      <c r="B50" s="6"/>
+      <c r="C50" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E50" t="s">
+        <v>110</v>
+      </c>
+      <c r="F50">
+        <v>6</v>
+      </c>
+      <c r="G50" t="s">
+        <v>103</v>
+      </c>
+      <c r="H50" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I50" s="111">
+        <f t="shared" si="1"/>
+        <v>231.31088503130337</v>
+      </c>
+      <c r="J50" s="111"/>
+      <c r="K50" s="112"/>
+      <c r="L50" s="110">
+        <f t="shared" si="2"/>
+        <v>300.25088503130337</v>
+      </c>
+    </row>
+    <row r="51" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A51" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B51" s="6"/>
+      <c r="C51" s="6"/>
+      <c r="D51" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="H51" s="111" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I51" s="111" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J51" s="111"/>
+      <c r="K51" s="112">
+        <f>SUM(J52:J60)</f>
+        <v>1359.9032002243127</v>
+      </c>
+      <c r="L51" s="110" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A52" s="5"/>
+      <c r="B52" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C52" s="6"/>
+      <c r="D52" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E52" t="s">
+        <v>110</v>
+      </c>
+      <c r="F52">
+        <v>6</v>
+      </c>
+      <c r="G52" t="s">
+        <v>103</v>
+      </c>
+      <c r="H52" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I52" s="111">
+        <f t="shared" si="1"/>
+        <v>231.31088503130337</v>
+      </c>
+      <c r="J52" s="111">
+        <f t="shared" ref="J52:J60" si="5">I52</f>
+        <v>231.31088503130337</v>
+      </c>
+      <c r="K52" s="112"/>
+      <c r="L52" s="110">
+        <f t="shared" si="2"/>
+        <v>300.25088503130337</v>
+      </c>
+    </row>
+    <row r="53" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A53" s="5"/>
+      <c r="B53" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C53" s="6"/>
+      <c r="D53" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E53" t="s">
+        <v>110</v>
+      </c>
+      <c r="F53">
+        <v>4</v>
+      </c>
+      <c r="G53" t="s">
+        <v>103</v>
+      </c>
+      <c r="H53" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I53" s="111">
+        <f t="shared" si="1"/>
+        <v>154.20725668753559</v>
+      </c>
+      <c r="J53" s="111">
+        <f t="shared" si="5"/>
+        <v>154.20725668753559</v>
+      </c>
+      <c r="K53" s="112"/>
+      <c r="L53" s="110">
+        <f t="shared" si="2"/>
+        <v>200.1672566875356</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A54" s="5"/>
+      <c r="B54" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C54" s="6"/>
+      <c r="D54" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E54" t="s">
+        <v>110</v>
+      </c>
+      <c r="F54">
+        <v>5</v>
+      </c>
+      <c r="G54" t="s">
+        <v>103</v>
+      </c>
+      <c r="H54" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I54" s="111">
+        <f t="shared" si="1"/>
+        <v>192.7590708594195</v>
+      </c>
+      <c r="J54" s="111">
+        <f t="shared" si="5"/>
+        <v>192.7590708594195</v>
+      </c>
+      <c r="K54" s="112"/>
+      <c r="L54" s="110">
+        <f t="shared" si="2"/>
+        <v>250.20907085941951</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A55" s="5"/>
+      <c r="B55" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C55" s="6"/>
+      <c r="D55" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E55" t="s">
+        <v>110</v>
+      </c>
+      <c r="F55">
+        <v>3</v>
+      </c>
+      <c r="G55" t="s">
+        <v>103</v>
+      </c>
+      <c r="H55" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I55" s="111">
+        <f t="shared" si="1"/>
+        <v>115.65544251565169</v>
+      </c>
+      <c r="J55" s="111">
+        <f t="shared" si="5"/>
+        <v>115.65544251565169</v>
+      </c>
+      <c r="K55" s="112"/>
+      <c r="L55" s="110">
+        <f t="shared" si="2"/>
+        <v>150.12544251565168</v>
+      </c>
+    </row>
+    <row r="56" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A56" s="5"/>
+      <c r="B56" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C56" s="6"/>
+      <c r="D56" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="E56" t="s">
+        <v>110</v>
+      </c>
+      <c r="F56">
+        <v>4</v>
+      </c>
+      <c r="G56" t="s">
+        <v>103</v>
+      </c>
+      <c r="H56" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I56" s="111">
+        <f t="shared" si="1"/>
+        <v>154.20725668753559</v>
+      </c>
+      <c r="J56" s="111">
+        <f t="shared" si="5"/>
+        <v>154.20725668753559</v>
+      </c>
+      <c r="K56" s="112"/>
+      <c r="L56" s="110">
+        <f t="shared" si="2"/>
+        <v>200.1672566875356</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A57" s="5"/>
+      <c r="B57" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C57" s="6"/>
+      <c r="D57" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E57" t="s">
+        <v>110</v>
+      </c>
+      <c r="F57">
+        <v>5</v>
+      </c>
+      <c r="G57" t="s">
+        <v>103</v>
+      </c>
+      <c r="H57" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I57" s="111">
+        <f t="shared" si="1"/>
+        <v>192.7590708594195</v>
+      </c>
+      <c r="J57" s="111">
+        <f t="shared" si="5"/>
+        <v>192.7590708594195</v>
+      </c>
+      <c r="K57" s="112"/>
+      <c r="L57" s="110">
+        <f t="shared" si="2"/>
+        <v>250.20907085941951</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A58" s="5"/>
+      <c r="B58" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C58" s="6"/>
+      <c r="D58" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E58" t="s">
+        <v>110</v>
+      </c>
+      <c r="F58">
+        <v>3</v>
+      </c>
+      <c r="G58" t="s">
+        <v>103</v>
+      </c>
+      <c r="H58" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I58" s="111">
+        <f t="shared" si="1"/>
+        <v>115.65544251565169</v>
+      </c>
+      <c r="J58" s="111">
+        <f t="shared" si="5"/>
+        <v>115.65544251565169</v>
+      </c>
+      <c r="K58" s="112"/>
+      <c r="L58" s="110">
+        <f t="shared" si="2"/>
+        <v>150.12544251565168</v>
+      </c>
+    </row>
+    <row r="59" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A59" s="5"/>
+      <c r="B59" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C59" s="6"/>
+      <c r="D59" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="E59" t="s">
+        <v>110</v>
+      </c>
+      <c r="F59">
+        <v>3</v>
+      </c>
+      <c r="G59" t="s">
+        <v>103</v>
+      </c>
+      <c r="H59" s="111">
+        <f t="shared" si="0"/>
+        <v>38.551814171883898</v>
+      </c>
+      <c r="I59" s="111">
+        <f t="shared" si="1"/>
+        <v>115.65544251565169</v>
+      </c>
+      <c r="J59" s="111">
+        <f t="shared" si="5"/>
+        <v>115.65544251565169</v>
+      </c>
+      <c r="K59" s="112"/>
+      <c r="L59" s="110">
+        <f t="shared" si="2"/>
+        <v>150.12544251565168</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A60" s="5"/>
+      <c r="B60" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C60" s="6"/>
+      <c r="D60" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E60" t="s">
+        <v>109</v>
+      </c>
+      <c r="F60">
+        <v>2</v>
+      </c>
+      <c r="G60" t="s">
+        <v>103</v>
+      </c>
+      <c r="H60" s="111">
+        <f t="shared" si="0"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I60" s="111">
+        <f t="shared" si="1"/>
+        <v>87.693332552144369</v>
+      </c>
+      <c r="J60" s="111">
+        <f t="shared" si="5"/>
+        <v>87.693332552144369</v>
+      </c>
+      <c r="K60" s="112"/>
+      <c r="L60" s="110">
+        <f t="shared" si="2"/>
+        <v>110.67333255214437</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A61" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B61" s="6"/>
+      <c r="C61" s="6"/>
+      <c r="D61" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="H61" s="111" t="str">
+        <f t="shared" si="0"/>
+        <v/>
+      </c>
+      <c r="I61" s="111" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="J61" s="111"/>
+      <c r="K61" s="112">
+        <f>SUM(J62:J73)</f>
+        <v>1285.9236266810587</v>
+      </c>
+      <c r="L61" s="110" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+    </row>
+    <row r="62" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A62" s="5"/>
+      <c r="B62" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C62" s="6"/>
+      <c r="D62" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E62" t="s">
+        <v>104</v>
+      </c>
+      <c r="F62">
+        <v>1</v>
+      </c>
+      <c r="G62" t="s">
+        <v>103</v>
+      </c>
+      <c r="H62" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I62" s="111">
+        <f t="shared" si="1"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J62" s="111">
+        <f t="shared" ref="J62:J73" si="6">I62</f>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="K62" s="112"/>
+      <c r="L62" s="110">
+        <f t="shared" si="2"/>
+        <v>61.27212534477475</v>
+      </c>
+    </row>
+    <row r="63" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A63" s="5"/>
+      <c r="B63" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C63" s="6"/>
+      <c r="D63" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E63" t="s">
+        <v>104</v>
+      </c>
+      <c r="F63">
+        <v>1</v>
+      </c>
+      <c r="G63" t="s">
+        <v>103</v>
+      </c>
+      <c r="H63" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I63" s="111">
+        <f t="shared" si="1"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J63" s="111">
+        <f t="shared" si="6"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="K63" s="112"/>
+      <c r="L63" s="110">
+        <f t="shared" si="2"/>
+        <v>61.27212534477475</v>
+      </c>
+    </row>
+    <row r="64" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A64" s="5"/>
+      <c r="B64" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C64" s="6"/>
+      <c r="D64" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="E64" t="s">
+        <v>107</v>
+      </c>
+      <c r="F64">
+        <v>1</v>
+      </c>
+      <c r="G64" t="s">
+        <v>103</v>
+      </c>
+      <c r="H64" s="111">
+        <f t="shared" si="0"/>
+        <v>45.220459339114129</v>
+      </c>
+      <c r="I64" s="111">
+        <f t="shared" si="1"/>
+        <v>45.220459339114129</v>
+      </c>
+      <c r="J64" s="111">
+        <f t="shared" si="6"/>
+        <v>45.220459339114129</v>
+      </c>
+      <c r="K64" s="112"/>
+      <c r="L64" s="110">
+        <f t="shared" si="2"/>
+        <v>56.710459339114131</v>
+      </c>
+    </row>
+    <row r="65" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A65" s="5"/>
+      <c r="B65" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C65" s="6"/>
+      <c r="D65" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E65" t="s">
+        <v>107</v>
+      </c>
+      <c r="F65">
+        <v>2</v>
+      </c>
+      <c r="G65" t="s">
+        <v>103</v>
+      </c>
+      <c r="H65" s="111">
+        <f t="shared" si="0"/>
+        <v>45.220459339114129</v>
+      </c>
+      <c r="I65" s="111">
+        <f t="shared" si="1"/>
+        <v>90.440918678228257</v>
+      </c>
+      <c r="J65" s="111">
+        <f t="shared" si="6"/>
+        <v>90.440918678228257</v>
+      </c>
+      <c r="K65" s="112"/>
+      <c r="L65" s="110">
+        <f t="shared" si="2"/>
+        <v>113.42091867822826</v>
+      </c>
+    </row>
+    <row r="66" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A66" s="5"/>
+      <c r="B66" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C66" s="6"/>
+      <c r="D66" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="E66" t="s">
+        <v>104</v>
+      </c>
+      <c r="F66">
+        <v>3</v>
+      </c>
+      <c r="G66" t="s">
+        <v>103</v>
+      </c>
+      <c r="H66" s="111">
+        <f t="shared" si="0"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I66" s="111">
+        <f t="shared" si="1"/>
+        <v>149.34637603432424</v>
+      </c>
+      <c r="J66" s="111">
+        <f t="shared" si="6"/>
+        <v>149.34637603432424</v>
+      </c>
+      <c r="K66" s="112"/>
+      <c r="L66" s="110">
+        <f t="shared" si="2"/>
+        <v>183.81637603432424</v>
+      </c>
+    </row>
+    <row r="67" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A67" s="5"/>
+      <c r="B67" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C67" s="6"/>
+      <c r="D67" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="E67" t="s">
+        <v>106</v>
+      </c>
+      <c r="F67">
+        <v>2</v>
+      </c>
+      <c r="G67" t="s">
+        <v>103</v>
+      </c>
+      <c r="H67" s="111">
+        <f t="shared" ref="H67:H73" si="7">_xlfn.XLOOKUP(E67,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <v>42.159269173306768</v>
+      </c>
+      <c r="I67" s="111">
+        <f t="shared" si="1"/>
+        <v>84.318538346613536</v>
+      </c>
+      <c r="J67" s="111">
+        <f t="shared" si="6"/>
+        <v>84.318538346613536</v>
+      </c>
+      <c r="K67" s="112"/>
+      <c r="L67" s="110">
+        <f t="shared" si="2"/>
+        <v>107.29853834661354</v>
+      </c>
+    </row>
+    <row r="68" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A68" s="5"/>
+      <c r="B68" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C68" s="6"/>
+      <c r="D68" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E68" t="s">
+        <v>108</v>
+      </c>
+      <c r="F68">
+        <v>3</v>
+      </c>
+      <c r="G68" t="s">
+        <v>103</v>
+      </c>
+      <c r="H68" s="111">
+        <f t="shared" si="7"/>
+        <v>49.154057104913683</v>
+      </c>
+      <c r="I68" s="111">
+        <f t="shared" ref="I68:I73" si="8">IFERROR(H68*F68,"")</f>
+        <v>147.46217131474106</v>
+      </c>
+      <c r="J68" s="111">
+        <f t="shared" si="6"/>
+        <v>147.46217131474106</v>
+      </c>
+      <c r="K68" s="112"/>
+      <c r="L68" s="110">
+        <f t="shared" ref="L68:L73" si="9">IFERROR(I68+($P$10*F68),"")</f>
+        <v>181.93217131474105</v>
+      </c>
+    </row>
+    <row r="69" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A69" s="5"/>
+      <c r="B69" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C69" s="6"/>
+      <c r="D69" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E69" t="s">
+        <v>109</v>
+      </c>
+      <c r="F69">
+        <v>6</v>
+      </c>
+      <c r="G69" t="s">
+        <v>103</v>
+      </c>
+      <c r="H69" s="111">
+        <f t="shared" si="7"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I69" s="111">
+        <f t="shared" si="8"/>
+        <v>263.07999765643308</v>
+      </c>
+      <c r="J69" s="111">
+        <f t="shared" si="6"/>
+        <v>263.07999765643308</v>
+      </c>
+      <c r="K69" s="112"/>
+      <c r="L69" s="110">
+        <f t="shared" si="9"/>
+        <v>332.01999765643308</v>
+      </c>
+    </row>
+    <row r="70" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A70" s="5"/>
+      <c r="B70" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C70" s="6"/>
+      <c r="D70" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="E70" t="s">
+        <v>109</v>
+      </c>
+      <c r="F70">
+        <v>2</v>
+      </c>
+      <c r="G70" t="s">
+        <v>103</v>
+      </c>
+      <c r="H70" s="111">
+        <f t="shared" si="7"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I70" s="111">
+        <f t="shared" si="8"/>
+        <v>87.693332552144369</v>
+      </c>
+      <c r="J70" s="111">
+        <f t="shared" si="6"/>
+        <v>87.693332552144369</v>
+      </c>
+      <c r="K70" s="112"/>
+      <c r="L70" s="110">
+        <f t="shared" si="9"/>
+        <v>110.67333255214437</v>
+      </c>
+    </row>
+    <row r="71" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A71" s="5"/>
+      <c r="B71" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C71" s="6"/>
+      <c r="D71" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E71" t="s">
+        <v>109</v>
+      </c>
+      <c r="F71">
+        <v>5</v>
+      </c>
+      <c r="G71" t="s">
+        <v>103</v>
+      </c>
+      <c r="H71" s="111">
+        <f t="shared" si="7"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I71" s="111">
+        <f t="shared" si="8"/>
+        <v>219.23333138036094</v>
+      </c>
+      <c r="J71" s="111">
+        <f t="shared" si="6"/>
+        <v>219.23333138036094</v>
+      </c>
+      <c r="K71" s="112"/>
+      <c r="L71" s="110">
+        <f t="shared" si="9"/>
+        <v>276.68333138036093</v>
+      </c>
+    </row>
+    <row r="72" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A72" s="5"/>
+      <c r="B72" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C72" s="6"/>
+      <c r="D72" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="E72" t="s">
+        <v>104</v>
+      </c>
+      <c r="F72">
+        <v>1</v>
+      </c>
+      <c r="G72" t="s">
+        <v>103</v>
+      </c>
+      <c r="H72" s="111">
+        <f t="shared" si="7"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I72" s="111">
+        <f t="shared" si="8"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J72" s="111">
+        <f t="shared" si="6"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="K72" s="112"/>
+      <c r="L72" s="110">
+        <f t="shared" si="9"/>
+        <v>61.27212534477475</v>
+      </c>
+    </row>
+    <row r="73" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A73" s="8"/>
+      <c r="B73" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C73" s="9"/>
+      <c r="D73" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="E73" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="F73" s="11">
+        <v>1</v>
+      </c>
+      <c r="G73" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="H73" s="111">
+        <f t="shared" si="7"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I73" s="111">
+        <f t="shared" si="8"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="J73" s="111">
+        <f t="shared" si="6"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="K73" s="113"/>
+      <c r="L73" s="110">
+        <f t="shared" si="9"/>
+        <v>61.27212534477475</v>
+      </c>
+    </row>
+    <row r="74" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A74" s="127" t="s">
+        <v>4</v>
+      </c>
+      <c r="B74" s="128"/>
+      <c r="C74" s="128"/>
+      <c r="D74" s="128"/>
+      <c r="E74" s="128"/>
+      <c r="F74" s="128"/>
+      <c r="G74" s="128"/>
+      <c r="H74" s="128"/>
+      <c r="I74" s="128"/>
+      <c r="J74" s="128"/>
+      <c r="K74" s="114">
+        <f>SUM(K3:K73)</f>
+        <v>13383.612572529586</v>
+      </c>
+      <c r="L74" s="111">
+        <f>SUM(L3:L73)</f>
+        <v>16945.512572529584</v>
+      </c>
+    </row>
+    <row r="75" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="K75" s="2"/>
+      <c r="L75" s="2"/>
+    </row>
+    <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A76" s="133" t="s">
+        <v>192</v>
+      </c>
+      <c r="B76" s="134"/>
+      <c r="C76" s="134"/>
+      <c r="D76" s="134"/>
+      <c r="E76" s="134"/>
+      <c r="F76" s="134"/>
+      <c r="G76" s="134"/>
+      <c r="H76" s="134"/>
+      <c r="I76" s="134"/>
+      <c r="J76" s="134"/>
+      <c r="K76" s="135"/>
+      <c r="L76" s="124"/>
+    </row>
+    <row r="77" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A77" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B77" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C77" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="D77" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="E77" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="F77" s="13" t="s">
+        <v>16</v>
+      </c>
+      <c r="G77" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="H77" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="I77" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="J77" s="13" t="s">
+        <v>5</v>
+      </c>
+      <c r="K77" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="L77" s="118"/>
+    </row>
+    <row r="78" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A78" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B78" s="6"/>
+      <c r="C78" s="6"/>
+      <c r="D78" t="s">
+        <v>197</v>
+      </c>
+      <c r="H78" s="116"/>
+      <c r="I78" s="116"/>
+      <c r="J78" s="116">
+        <f>SUM(I79:I80)</f>
+        <v>172.5</v>
+      </c>
+      <c r="K78" s="117">
+        <f>J78</f>
+        <v>172.5</v>
+      </c>
+      <c r="L78" s="116"/>
+    </row>
+    <row r="79" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A79" s="5"/>
+      <c r="B79" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C79" s="6"/>
+      <c r="D79" t="s">
+        <v>198</v>
+      </c>
+      <c r="E79" t="s">
+        <v>200</v>
+      </c>
+      <c r="F79">
+        <v>150</v>
+      </c>
+      <c r="G79" t="s">
+        <v>201</v>
+      </c>
+      <c r="H79" s="116">
+        <v>0.35</v>
+      </c>
+      <c r="I79" s="116">
+        <f>H79*F79</f>
+        <v>52.5</v>
+      </c>
+      <c r="J79" s="116"/>
+      <c r="K79" s="117"/>
+      <c r="L79" s="116"/>
+    </row>
+    <row r="80" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A80" s="5"/>
+      <c r="B80" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C80" s="6"/>
+      <c r="D80" t="s">
+        <v>199</v>
+      </c>
+      <c r="E80" t="s">
+        <v>200</v>
+      </c>
+      <c r="F80">
+        <v>6</v>
+      </c>
+      <c r="G80" t="s">
+        <v>202</v>
+      </c>
+      <c r="H80" s="116">
+        <v>20</v>
+      </c>
+      <c r="I80" s="116">
+        <f>H80*F80</f>
+        <v>120</v>
+      </c>
+      <c r="J80" s="116"/>
+      <c r="K80" s="117"/>
+      <c r="L80" s="116"/>
+    </row>
+    <row r="81" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A81" s="127" t="s">
+        <v>4</v>
+      </c>
+      <c r="B81" s="128"/>
+      <c r="C81" s="128"/>
+      <c r="D81" s="128"/>
+      <c r="E81" s="128"/>
+      <c r="F81" s="128"/>
+      <c r="G81" s="128"/>
+      <c r="H81" s="128"/>
+      <c r="I81" s="128"/>
+      <c r="J81" s="128"/>
+      <c r="K81" s="114">
+        <f>SUM(K78:K80)</f>
+        <v>172.5</v>
+      </c>
+      <c r="L81" s="111"/>
+    </row>
+    <row r="82" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A82" s="6"/>
+      <c r="B82" s="6"/>
+      <c r="C82" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="N1:P1"/>
+    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="A74:J74"/>
+    <mergeCell ref="A76:K76"/>
+    <mergeCell ref="A81:J81"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E73" xr:uid="{C5BB27AF-9B30-4FCF-8E44-DCCBC0FC7FF5}">
+      <formula1>$Q$20:$Q$25</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84438618-631B-43FB-9820-9583257CBFE8}">
+  <dimension ref="A1:K56"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="37.109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="8.88671875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.77734375" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="23.77734375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="130" t="s">
+        <v>210</v>
+      </c>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="132"/>
+      <c r="G1" s="127" t="s">
+        <v>209</v>
+      </c>
+      <c r="H1" s="128"/>
+      <c r="I1" s="129"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A2" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>212</v>
+      </c>
+      <c r="E2" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" s="119" t="s">
+        <v>205</v>
+      </c>
+      <c r="H2" s="118" t="s">
+        <v>204</v>
+      </c>
+      <c r="I2" s="120" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="6"/>
+      <c r="C3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="123"/>
+      <c r="E3" s="115">
+        <f>SUM(D4:D6)</f>
+        <v>1470.5310082745939</v>
+      </c>
+      <c r="G3" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="H3" t="s">
+        <v>206</v>
+      </c>
+      <c r="I3" s="121">
+        <f>E54</f>
+        <v>16945.512572529587</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A4" s="5"/>
+      <c r="B4" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="123">
+        <f>Costs_final!L4</f>
+        <v>122.5442506895495</v>
+      </c>
+      <c r="E4" s="112"/>
+      <c r="G4" s="127" t="s">
+        <v>115</v>
+      </c>
+      <c r="H4" s="128"/>
+      <c r="I4" s="122">
+        <f>SUM(I3)</f>
+        <v>16945.512572529587</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A5" s="5"/>
+      <c r="B5" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="123">
+        <f>Costs_final!L5</f>
+        <v>122.5442506895495</v>
+      </c>
+      <c r="E5" s="112"/>
+      <c r="G5" s="6"/>
+      <c r="I5" s="111"/>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A6" s="5"/>
+      <c r="B6" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="123">
+        <f>SUM(Costs_final!L7:L19)</f>
+        <v>1225.4425068954949</v>
+      </c>
+      <c r="E6" s="112"/>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A7" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="6"/>
+      <c r="C7" s="7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" s="123"/>
+      <c r="E7" s="112">
+        <f>SUM(D8:D17)</f>
+        <v>3088.6202445365593</v>
+      </c>
+      <c r="K7" s="110"/>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A8" s="5"/>
+      <c r="B8" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="123">
+        <f>Costs_final!L21</f>
+        <v>53.64926917330677</v>
+      </c>
+      <c r="E8" s="112"/>
+      <c r="K8" s="110"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A9" s="5"/>
+      <c r="B9" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D9" s="123">
+        <f>Costs_final!L22</f>
+        <v>226.84183735645652</v>
+      </c>
+      <c r="E9" s="112"/>
+      <c r="K9" s="110"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A10" s="5"/>
+      <c r="B10" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="123">
+        <f>Costs_final!L23</f>
+        <v>53.64926917330677</v>
+      </c>
+      <c r="E10" s="112"/>
+      <c r="K10" s="110"/>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A11" s="5"/>
+      <c r="B11" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D11" s="123">
+        <f>Costs_final!L24</f>
+        <v>53.64926917330677</v>
+      </c>
+      <c r="E11" s="112"/>
+      <c r="K11" s="110"/>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A12" s="5"/>
+      <c r="B12" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="D12" s="123">
+        <f>Costs_final!L25</f>
+        <v>107.29853834661354</v>
+      </c>
+      <c r="E12" s="112"/>
+      <c r="K12" s="110"/>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A13" s="5"/>
+      <c r="B13" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="D13" s="123">
+        <f>Costs_final!L26</f>
+        <v>340.26275603468474</v>
+      </c>
+      <c r="E13" s="112"/>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A14" s="5"/>
+      <c r="B14" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D14" s="123">
+        <f>Costs_final!L27</f>
+        <v>1180.283921812749</v>
+      </c>
+      <c r="E14" s="112"/>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A15" s="5"/>
+      <c r="B15" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="D15" s="123">
+        <f>Costs_final!L28</f>
+        <v>429.19415338645416</v>
+      </c>
+      <c r="E15" s="112"/>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A16" s="5"/>
+      <c r="B16" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="D16" s="123">
+        <f>Costs_final!L29</f>
+        <v>214.59707669322708</v>
+      </c>
+      <c r="E16" s="112"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="5"/>
+      <c r="B17" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D17" s="123">
+        <f>Costs_final!L30</f>
+        <v>429.19415338645416</v>
+      </c>
+      <c r="E17" s="112"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B18" s="6"/>
+      <c r="C18" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="123" t="str">
+        <f>Costs_final!L31</f>
+        <v/>
+      </c>
+      <c r="E18" s="112">
+        <f>SUM(D19:D25)</f>
+        <v>2970.032664607676</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="5"/>
+      <c r="B19" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="D19" s="123">
+        <f>Costs_final!L32</f>
+        <v>606.44057104913679</v>
+      </c>
+      <c r="E19" s="112"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="5"/>
+      <c r="B20" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="D20" s="123">
+        <f>Costs_final!L33</f>
+        <v>150.12544251565168</v>
+      </c>
+      <c r="E20" s="112"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="5"/>
+      <c r="B21" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="123">
+        <f>Costs_final!L34</f>
+        <v>442.69333020857749</v>
+      </c>
+      <c r="E21" s="112"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="5"/>
+      <c r="B22" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="123">
+        <f>Costs_final!L35</f>
+        <v>221.34666510428875</v>
+      </c>
+      <c r="E22" s="112"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="5"/>
+      <c r="B23" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="D23" s="123">
+        <f>Costs_final!L36</f>
+        <v>332.01999765643308</v>
+      </c>
+      <c r="E23" s="112"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="5"/>
+      <c r="B24" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="D24" s="123">
+        <f>Costs_final!L37</f>
+        <v>664.03999531286615</v>
+      </c>
+      <c r="E24" s="112"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="5"/>
+      <c r="B25" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="D25" s="123">
+        <f>Costs_final!L38</f>
+        <v>553.36666276072185</v>
+      </c>
+      <c r="E25" s="112"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B26" s="6"/>
+      <c r="C26" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="123">
+        <f>Costs_final!L39</f>
+        <v>332.01999765643308</v>
+      </c>
+      <c r="E26" s="111">
+        <f>D26</f>
+        <v>332.01999765643308</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="B27" s="6"/>
+      <c r="C27" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="123" t="str">
+        <f>Costs_final!L40</f>
+        <v/>
+      </c>
+      <c r="E27" s="112">
+        <f>SUM(D28:D30)</f>
+        <v>5714.6118305489526</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="5"/>
+      <c r="B28" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="D28" s="123">
+        <f>Costs_final!L41</f>
+        <v>363.86434262948211</v>
+      </c>
+      <c r="E28" s="112"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="5"/>
+      <c r="B29" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="123">
+        <f>Costs_final!L42</f>
+        <v>60.644057104913685</v>
+      </c>
+      <c r="E29" s="112"/>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="5"/>
+      <c r="B30" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" s="123">
+        <f>SUM(Costs_final!L44:L50)</f>
+        <v>5290.1034308145572</v>
+      </c>
+      <c r="E30" s="112"/>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="B31" s="6"/>
+      <c r="C31" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D31" s="123"/>
+      <c r="E31" s="112">
+        <f>SUM(D32:D40)</f>
+        <v>1762.0532002243128</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="5"/>
+      <c r="B32" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="D32" s="123">
+        <f>Costs_final!L52</f>
+        <v>300.25088503130337</v>
+      </c>
+      <c r="E32" s="112"/>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A33" s="5"/>
+      <c r="B33" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="D33" s="123">
+        <f>Costs_final!L53</f>
+        <v>200.1672566875356</v>
+      </c>
+      <c r="E33" s="112"/>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A34" s="5"/>
+      <c r="B34" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D34" s="123">
+        <f>Costs_final!L54</f>
+        <v>250.20907085941951</v>
+      </c>
+      <c r="E34" s="112"/>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="5"/>
+      <c r="B35" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D35" s="123">
+        <f>Costs_final!L55</f>
+        <v>150.12544251565168</v>
+      </c>
+      <c r="E35" s="112"/>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="5"/>
+      <c r="B36" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="D36" s="123">
+        <f>Costs_final!L56</f>
+        <v>200.1672566875356</v>
+      </c>
+      <c r="E36" s="112"/>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A37" s="5"/>
+      <c r="B37" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D37" s="123">
+        <f>Costs_final!L57</f>
+        <v>250.20907085941951</v>
+      </c>
+      <c r="E37" s="112"/>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A38" s="5"/>
+      <c r="B38" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D38" s="123">
+        <f>Costs_final!L58</f>
+        <v>150.12544251565168</v>
+      </c>
+      <c r="E38" s="112"/>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="5"/>
+      <c r="B39" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="D39" s="123">
+        <f>Costs_final!L59</f>
+        <v>150.12544251565168</v>
+      </c>
+      <c r="E39" s="112"/>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A40" s="5"/>
+      <c r="B40" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D40" s="123">
+        <f>Costs_final!L60</f>
+        <v>110.67333255214437</v>
+      </c>
+      <c r="E40" s="112"/>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A41" s="5" t="s">
+        <v>87</v>
+      </c>
+      <c r="B41" s="6"/>
+      <c r="C41" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="D41" s="123" t="str">
+        <f>Costs_final!L61</f>
+        <v/>
+      </c>
+      <c r="E41" s="112">
+        <f>SUM(D42:D53)</f>
+        <v>1607.6436266810585</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A42" s="5"/>
+      <c r="B42" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="D42" s="123">
+        <f>Costs_final!L62</f>
+        <v>61.27212534477475</v>
+      </c>
+      <c r="E42" s="112"/>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A43" s="5"/>
+      <c r="B43" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="D43" s="123">
+        <f>Costs_final!L63</f>
+        <v>61.27212534477475</v>
+      </c>
+      <c r="E43" s="112"/>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A44" s="5"/>
+      <c r="B44" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D44" s="123">
+        <f>Costs_final!L64</f>
+        <v>56.710459339114131</v>
+      </c>
+      <c r="E44" s="112"/>
+    </row>
+    <row r="45" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A45" s="5"/>
+      <c r="B45" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="D45" s="123">
+        <f>Costs_final!L65</f>
+        <v>113.42091867822826</v>
+      </c>
+      <c r="E45" s="112"/>
+    </row>
+    <row r="46" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="A46" s="5"/>
+      <c r="B46" s="6" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="D46" s="123">
+        <f>Costs_final!L66</f>
+        <v>183.81637603432424</v>
+      </c>
+      <c r="E46" s="112"/>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A47" s="5"/>
+      <c r="B47" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="D47" s="123">
+        <f>Costs_final!L67</f>
+        <v>107.29853834661354</v>
+      </c>
+      <c r="E47" s="112"/>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="5"/>
+      <c r="B48" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="D48" s="123">
+        <f>Costs_final!L68</f>
+        <v>181.93217131474105</v>
+      </c>
+      <c r="E48" s="112"/>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="5"/>
+      <c r="B49" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="D49" s="123">
+        <f>Costs_final!L69</f>
+        <v>332.01999765643308</v>
+      </c>
+      <c r="E49" s="112"/>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A50" s="5"/>
+      <c r="B50" s="6" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D50" s="123">
+        <f>Costs_final!L70</f>
+        <v>110.67333255214437</v>
+      </c>
+      <c r="E50" s="112"/>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A51" s="5"/>
+      <c r="B51" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="D51" s="123">
+        <f>Costs_final!L71</f>
+        <v>276.68333138036093</v>
+      </c>
+      <c r="E51" s="112"/>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A52" s="5"/>
+      <c r="B52" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="D52" s="123">
+        <f>Costs_final!L72</f>
+        <v>61.27212534477475</v>
+      </c>
+      <c r="E52" s="112"/>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A53" s="8"/>
+      <c r="B53" s="9" t="s">
+        <v>102</v>
+      </c>
+      <c r="C53" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="D53" s="123">
+        <f>Costs_final!L73</f>
+        <v>61.27212534477475</v>
+      </c>
+      <c r="E53" s="113"/>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" s="127" t="s">
+        <v>4</v>
+      </c>
+      <c r="B54" s="128"/>
+      <c r="C54" s="128"/>
+      <c r="D54" s="128"/>
+      <c r="E54" s="114">
+        <f>SUM(E3:E53)</f>
+        <v>16945.512572529587</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="E55" s="2"/>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A56" s="6"/>
+      <c r="B56" s="6"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="A54:D54"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: adds final usability test
</commit_message>
<xml_diff>
--- a/docs/budget.xlsx
+++ b/docs/budget.xlsx
@@ -8,16 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Desktop\proyectos\IRBoard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE692509-35D9-4BFA-B51B-C27FC9234824}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACF91FD6-6829-470F-87AD-E183670224AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" firstSheet="3" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Company definition" sheetId="2" r:id="rId1"/>
     <sheet name="Costs_init" sheetId="1" r:id="rId2"/>
     <sheet name="Client_init" sheetId="5" r:id="rId3"/>
     <sheet name="Costs_final" sheetId="6" r:id="rId4"/>
-    <sheet name="Client_final" sheetId="7" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1014" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="217">
   <si>
     <t>I1</t>
   </si>
@@ -689,6 +688,9 @@
   <si>
     <t>Dilution increase per billable hour</t>
   </si>
+  <si>
+    <t>deviation from original</t>
+  </si>
 </sst>
 </file>
 
@@ -1124,7 +1126,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="136">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1338,15 +1340,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1354,6 +1347,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1365,6 +1364,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -31006,27 +31010,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="130" t="s">
+      <c r="A1" s="127" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="131"/>
-      <c r="C1" s="131"/>
-      <c r="D1" s="131"/>
-      <c r="E1" s="131"/>
-      <c r="F1" s="131"/>
-      <c r="G1" s="131"/>
-      <c r="H1" s="131"/>
-      <c r="I1" s="131"/>
-      <c r="J1" s="131"/>
-      <c r="K1" s="132"/>
+      <c r="B1" s="128"/>
+      <c r="C1" s="128"/>
+      <c r="D1" s="128"/>
+      <c r="E1" s="128"/>
+      <c r="F1" s="128"/>
+      <c r="G1" s="128"/>
+      <c r="H1" s="128"/>
+      <c r="I1" s="128"/>
+      <c r="J1" s="128"/>
+      <c r="K1" s="129"/>
       <c r="L1" s="125" t="s">
         <v>213</v>
       </c>
-      <c r="N1" s="127" t="s">
+      <c r="N1" s="130" t="s">
         <v>203</v>
       </c>
-      <c r="O1" s="128"/>
-      <c r="P1" s="129"/>
+      <c r="O1" s="131"/>
+      <c r="P1" s="135"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -31190,15 +31194,13 @@
         <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
-      <c r="N5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="O5" t="s">
-        <v>208</v>
-      </c>
-      <c r="P5" s="112">
-        <f>0.25*(P3+P4)</f>
-        <v>3299.7543381673559</v>
+      <c r="N5" s="130" t="s">
+        <v>115</v>
+      </c>
+      <c r="O5" s="131"/>
+      <c r="P5" s="122">
+        <f>SUM(P3:P4)</f>
+        <v>13199.017352669423</v>
       </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.3">
@@ -31224,14 +31226,6 @@
       </c>
       <c r="K6" s="112"/>
       <c r="L6" s="110"/>
-      <c r="N6" s="127" t="s">
-        <v>115</v>
-      </c>
-      <c r="O6" s="128"/>
-      <c r="P6" s="122">
-        <f>SUM(P3:P5)</f>
-        <v>16498.77169083678</v>
-      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
@@ -31265,6 +31259,13 @@
         <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
+      <c r="O7" t="s">
+        <v>208</v>
+      </c>
+      <c r="P7" s="111">
+        <f>0.25*(P3+P4)</f>
+        <v>3299.7543381673559</v>
+      </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
@@ -31302,7 +31303,7 @@
         <v>211</v>
       </c>
       <c r="P8" s="111">
-        <f>P6-P3</f>
+        <f>P5+P7-P3</f>
         <v>3472.2543381673568</v>
       </c>
     </row>
@@ -33604,18 +33605,18 @@
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A74" s="127" t="s">
+      <c r="A74" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="B74" s="128"/>
-      <c r="C74" s="128"/>
-      <c r="D74" s="128"/>
-      <c r="E74" s="128"/>
-      <c r="F74" s="128"/>
-      <c r="G74" s="128"/>
-      <c r="H74" s="128"/>
-      <c r="I74" s="128"/>
-      <c r="J74" s="128"/>
+      <c r="B74" s="131"/>
+      <c r="C74" s="131"/>
+      <c r="D74" s="131"/>
+      <c r="E74" s="131"/>
+      <c r="F74" s="131"/>
+      <c r="G74" s="131"/>
+      <c r="H74" s="131"/>
+      <c r="I74" s="131"/>
+      <c r="J74" s="131"/>
       <c r="K74" s="114">
         <f>SUM(K3:K73)</f>
         <v>13026.517352669423</v>
@@ -33630,19 +33631,19 @@
       <c r="L75" s="2"/>
     </row>
     <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="133" t="s">
+      <c r="A76" s="132" t="s">
         <v>192</v>
       </c>
-      <c r="B76" s="134"/>
-      <c r="C76" s="134"/>
-      <c r="D76" s="134"/>
-      <c r="E76" s="134"/>
-      <c r="F76" s="134"/>
-      <c r="G76" s="134"/>
-      <c r="H76" s="134"/>
-      <c r="I76" s="134"/>
-      <c r="J76" s="134"/>
-      <c r="K76" s="135"/>
+      <c r="B76" s="133"/>
+      <c r="C76" s="133"/>
+      <c r="D76" s="133"/>
+      <c r="E76" s="133"/>
+      <c r="F76" s="133"/>
+      <c r="G76" s="133"/>
+      <c r="H76" s="133"/>
+      <c r="I76" s="133"/>
+      <c r="J76" s="133"/>
+      <c r="K76" s="134"/>
       <c r="L76" s="124"/>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.3">
@@ -33761,18 +33762,18 @@
       <c r="L80" s="116"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A81" s="127" t="s">
+      <c r="A81" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="B81" s="128"/>
-      <c r="C81" s="128"/>
-      <c r="D81" s="128"/>
-      <c r="E81" s="128"/>
-      <c r="F81" s="128"/>
-      <c r="G81" s="128"/>
-      <c r="H81" s="128"/>
-      <c r="I81" s="128"/>
-      <c r="J81" s="128"/>
+      <c r="B81" s="131"/>
+      <c r="C81" s="131"/>
+      <c r="D81" s="131"/>
+      <c r="E81" s="131"/>
+      <c r="F81" s="131"/>
+      <c r="G81" s="131"/>
+      <c r="H81" s="131"/>
+      <c r="I81" s="131"/>
+      <c r="J81" s="131"/>
       <c r="K81" s="114">
         <f>SUM(K78:K80)</f>
         <v>172.5</v>
@@ -33791,7 +33792,7 @@
     <mergeCell ref="A76:K76"/>
     <mergeCell ref="A81:J81"/>
     <mergeCell ref="N1:P1"/>
-    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="N5:O5"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="1">
@@ -33822,18 +33823,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="130" t="s">
+      <c r="A1" s="127" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="131"/>
-      <c r="C1" s="131"/>
-      <c r="D1" s="131"/>
-      <c r="E1" s="132"/>
-      <c r="G1" s="127" t="s">
+      <c r="B1" s="128"/>
+      <c r="C1" s="128"/>
+      <c r="D1" s="128"/>
+      <c r="E1" s="129"/>
+      <c r="G1" s="130" t="s">
         <v>209</v>
       </c>
-      <c r="H1" s="128"/>
-      <c r="I1" s="129"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="135"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -33898,10 +33899,10 @@
         <v>122.72425068954949</v>
       </c>
       <c r="E4" s="112"/>
-      <c r="G4" s="127" t="s">
+      <c r="G4" s="130" t="s">
         <v>115</v>
       </c>
-      <c r="H4" s="128"/>
+      <c r="H4" s="131"/>
       <c r="I4" s="122">
         <f>SUM(I3)</f>
         <v>16500.517352669427</v>
@@ -34614,12 +34615,12 @@
       <c r="E53" s="113"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="127" t="s">
+      <c r="A54" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="B54" s="128"/>
-      <c r="C54" s="128"/>
-      <c r="D54" s="128"/>
+      <c r="B54" s="131"/>
+      <c r="C54" s="131"/>
+      <c r="D54" s="131"/>
       <c r="E54" s="114">
         <f>SUM(E3:E53)</f>
         <v>16500.517352669427</v>
@@ -34665,30 +34666,30 @@
     <col min="18" max="18" width="23.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="130" t="s">
+    <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="127" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="131"/>
-      <c r="C1" s="131"/>
-      <c r="D1" s="131"/>
-      <c r="E1" s="131"/>
-      <c r="F1" s="131"/>
-      <c r="G1" s="131"/>
-      <c r="H1" s="131"/>
-      <c r="I1" s="131"/>
-      <c r="J1" s="131"/>
-      <c r="K1" s="132"/>
+      <c r="B1" s="128"/>
+      <c r="C1" s="128"/>
+      <c r="D1" s="128"/>
+      <c r="E1" s="128"/>
+      <c r="F1" s="128"/>
+      <c r="G1" s="128"/>
+      <c r="H1" s="128"/>
+      <c r="I1" s="128"/>
+      <c r="J1" s="128"/>
+      <c r="K1" s="129"/>
       <c r="L1" s="125" t="s">
         <v>213</v>
       </c>
-      <c r="N1" s="127" t="s">
+      <c r="N1" s="130" t="s">
         <v>203</v>
       </c>
-      <c r="O1" s="128"/>
-      <c r="P1" s="129"/>
+      <c r="O1" s="131"/>
+      <c r="P1" s="135"/>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
         <v>0</v>
       </c>
@@ -34732,8 +34733,11 @@
       <c r="P2" s="120" t="s">
         <v>4</v>
       </c>
+      <c r="Q2" s="136" t="s">
+        <v>216</v>
+      </c>
     </row>
-    <row r="3" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
@@ -34768,8 +34772,12 @@
         <f>K74</f>
         <v>13383.612572529586</v>
       </c>
+      <c r="Q3" s="137">
+        <f>((P3-Costs_init!P3)/Costs_init!P3)</f>
+        <v>2.7412946238235029E-2</v>
+      </c>
     </row>
-    <row r="4" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="5"/>
       <c r="B4" s="6" t="s">
         <v>7</v>
@@ -34802,7 +34810,7 @@
       <c r="K4" s="112"/>
       <c r="L4" s="110">
         <f t="shared" ref="L4:L67" si="2">IFERROR(I4+($P$10*F4),"")</f>
-        <v>122.5442506895495</v>
+        <v>121.9842506895495</v>
       </c>
       <c r="N4" s="5" t="s">
         <v>8</v>
@@ -34814,8 +34822,12 @@
         <f>K81</f>
         <v>172.5</v>
       </c>
+      <c r="Q4" s="137">
+        <f>((P4-Costs_init!P4)/Costs_init!P4)</f>
+        <v>0</v>
+      </c>
     </row>
-    <row r="5" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A5" s="5"/>
       <c r="B5" s="6" t="s">
         <v>13</v>
@@ -34848,20 +34860,22 @@
       <c r="K5" s="112"/>
       <c r="L5" s="110">
         <f t="shared" si="2"/>
-        <v>122.5442506895495</v>
-      </c>
-      <c r="N5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="O5" t="s">
-        <v>208</v>
-      </c>
-      <c r="P5" s="112">
-        <f>0.25*(P3+P4)</f>
-        <v>3389.0281431323965</v>
+        <v>121.9842506895495</v>
+      </c>
+      <c r="N5" s="130" t="s">
+        <v>115</v>
+      </c>
+      <c r="O5" s="131"/>
+      <c r="P5" s="122">
+        <f>SUM(P3:P4)</f>
+        <v>13556.112572529586</v>
+      </c>
+      <c r="Q5" s="137">
+        <f>((P5-Costs_init!P5)/Costs_init!P5)</f>
+        <v>2.7054682202379422E-2</v>
       </c>
     </row>
-    <row r="6" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A6" s="5"/>
       <c r="B6" s="6" t="s">
         <v>14</v>
@@ -34884,16 +34898,9 @@
       </c>
       <c r="K6" s="112"/>
       <c r="L6" s="110"/>
-      <c r="N6" s="127" t="s">
-        <v>115</v>
-      </c>
-      <c r="O6" s="128"/>
-      <c r="P6" s="122">
-        <f>SUM(P3:P5)</f>
-        <v>16945.140715661983</v>
-      </c>
+      <c r="Q6" s="137"/>
     </row>
-    <row r="7" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6" t="s">
@@ -34923,10 +34930,18 @@
       <c r="K7" s="112"/>
       <c r="L7" s="110">
         <f t="shared" si="2"/>
-        <v>61.27212534477475</v>
-      </c>
+        <v>60.992125344774749</v>
+      </c>
+      <c r="O7" t="s">
+        <v>208</v>
+      </c>
+      <c r="P7">
+        <f>Costs_init!P7</f>
+        <v>3299.7543381673559</v>
+      </c>
+      <c r="Q7" s="137"/>
     </row>
-    <row r="8" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
       <c r="B8" s="6"/>
       <c r="C8" s="6" t="s">
@@ -34956,17 +34971,17 @@
       <c r="K8" s="112"/>
       <c r="L8" s="110">
         <f t="shared" si="2"/>
-        <v>122.5442506895495</v>
+        <v>121.9842506895495</v>
       </c>
       <c r="O8" t="s">
         <v>211</v>
       </c>
       <c r="P8" s="111">
-        <f>P6-P3</f>
-        <v>3561.5281431323965</v>
+        <f>P5+P7-P3</f>
+        <v>3472.2543381673568</v>
       </c>
     </row>
-    <row r="9" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="5"/>
       <c r="B9" s="6"/>
       <c r="C9" s="6" t="s">
@@ -34996,7 +35011,7 @@
       <c r="K9" s="112"/>
       <c r="L9" s="110">
         <f t="shared" si="2"/>
-        <v>61.27212534477475</v>
+        <v>60.992125344774749</v>
       </c>
       <c r="O9" t="s">
         <v>214</v>
@@ -35006,7 +35021,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="10" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A10" s="5"/>
       <c r="B10" s="6"/>
       <c r="C10" s="6" t="s">
@@ -35036,17 +35051,17 @@
       <c r="K10" s="112"/>
       <c r="L10" s="110">
         <f t="shared" si="2"/>
-        <v>122.5442506895495</v>
+        <v>121.9842506895495</v>
       </c>
       <c r="O10" t="s">
         <v>215</v>
       </c>
       <c r="P10" s="123">
         <f>ROUNDUP(P8/P9,2)</f>
-        <v>11.49</v>
+        <v>11.209999999999999</v>
       </c>
     </row>
-    <row r="11" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="5"/>
       <c r="B11" s="6"/>
       <c r="C11" s="6" t="s">
@@ -35076,10 +35091,10 @@
       <c r="K11" s="112"/>
       <c r="L11" s="110">
         <f t="shared" si="2"/>
-        <v>61.27212534477475</v>
+        <v>60.992125344774749</v>
       </c>
     </row>
-    <row r="12" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
       <c r="B12" s="6"/>
       <c r="C12" s="6" t="s">
@@ -35109,10 +35124,10 @@
       <c r="K12" s="112"/>
       <c r="L12" s="110">
         <f t="shared" si="2"/>
-        <v>61.27212534477475</v>
+        <v>60.992125344774749</v>
       </c>
     </row>
-    <row r="13" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="5"/>
       <c r="B13" s="6"/>
       <c r="C13" s="6" t="s">
@@ -35142,10 +35157,10 @@
       <c r="K13" s="112"/>
       <c r="L13" s="110">
         <f t="shared" si="2"/>
-        <v>122.5442506895495</v>
+        <v>121.9842506895495</v>
       </c>
     </row>
-    <row r="14" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A14" s="5"/>
       <c r="B14" s="6"/>
       <c r="C14" s="6" t="s">
@@ -35175,10 +35190,10 @@
       <c r="K14" s="112"/>
       <c r="L14" s="110">
         <f t="shared" si="2"/>
-        <v>122.5442506895495</v>
+        <v>121.9842506895495</v>
       </c>
     </row>
-    <row r="15" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A15" s="5"/>
       <c r="B15" s="6"/>
       <c r="C15" s="6" t="s">
@@ -35208,10 +35223,10 @@
       <c r="K15" s="112"/>
       <c r="L15" s="110">
         <f t="shared" si="2"/>
-        <v>122.5442506895495</v>
+        <v>121.9842506895495</v>
       </c>
     </row>
-    <row r="16" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A16" s="5"/>
       <c r="B16" s="6"/>
       <c r="C16" s="6" t="s">
@@ -35241,7 +35256,7 @@
       <c r="K16" s="112"/>
       <c r="L16" s="110">
         <f t="shared" si="2"/>
-        <v>122.5442506895495</v>
+        <v>121.9842506895495</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
@@ -35274,7 +35289,7 @@
       <c r="K17" s="112"/>
       <c r="L17" s="110">
         <f t="shared" si="2"/>
-        <v>61.27212534477475</v>
+        <v>60.992125344774749</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
@@ -35307,7 +35322,7 @@
       <c r="K18" s="112"/>
       <c r="L18" s="110">
         <f t="shared" si="2"/>
-        <v>61.27212534477475</v>
+        <v>60.992125344774749</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
@@ -35340,7 +35355,7 @@
       <c r="K19" s="112"/>
       <c r="L19" s="110">
         <f t="shared" si="2"/>
-        <v>122.5442506895495</v>
+        <v>121.9842506895495</v>
       </c>
       <c r="Q19" s="7" t="s">
         <v>105</v>
@@ -35416,7 +35431,7 @@
       <c r="K21" s="112"/>
       <c r="L21" s="110">
         <f t="shared" si="2"/>
-        <v>53.64926917330677</v>
+        <v>53.369269173306769</v>
       </c>
       <c r="Q21" t="s">
         <v>107</v>
@@ -35459,7 +35474,7 @@
       <c r="K22" s="112"/>
       <c r="L22" s="110">
         <f t="shared" si="2"/>
-        <v>226.84183735645652</v>
+        <v>225.72183735645652</v>
       </c>
       <c r="Q22" t="s">
         <v>106</v>
@@ -35502,7 +35517,7 @@
       <c r="K23" s="112"/>
       <c r="L23" s="110">
         <f t="shared" si="2"/>
-        <v>53.64926917330677</v>
+        <v>53.369269173306769</v>
       </c>
       <c r="Q23" t="s">
         <v>108</v>
@@ -35545,7 +35560,7 @@
       <c r="K24" s="112"/>
       <c r="L24" s="110">
         <f t="shared" si="2"/>
-        <v>53.64926917330677</v>
+        <v>53.369269173306769</v>
       </c>
       <c r="Q24" t="s">
         <v>109</v>
@@ -35588,7 +35603,7 @@
       <c r="K25" s="112"/>
       <c r="L25" s="110">
         <f t="shared" si="2"/>
-        <v>107.29853834661354</v>
+        <v>106.73853834661354</v>
       </c>
       <c r="Q25" t="s">
         <v>110</v>
@@ -35631,7 +35646,7 @@
       <c r="K26" s="112"/>
       <c r="L26" s="110">
         <f t="shared" si="2"/>
-        <v>340.26275603468474</v>
+        <v>338.58275603468473</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.3">
@@ -35667,7 +35682,7 @@
       <c r="K27" s="112"/>
       <c r="L27" s="110">
         <f t="shared" si="2"/>
-        <v>1180.283921812749</v>
+        <v>1174.1239218127489</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
@@ -35703,7 +35718,7 @@
       <c r="K28" s="112"/>
       <c r="L28" s="110">
         <f t="shared" si="2"/>
-        <v>429.19415338645416</v>
+        <v>426.95415338645415</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.3">
@@ -35739,7 +35754,7 @@
       <c r="K29" s="112"/>
       <c r="L29" s="110">
         <f t="shared" si="2"/>
-        <v>214.59707669322708</v>
+        <v>213.47707669322708</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.3">
@@ -35775,7 +35790,7 @@
       <c r="K30" s="112"/>
       <c r="L30" s="110">
         <f t="shared" si="2"/>
-        <v>429.19415338645416</v>
+        <v>426.95415338645415</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
@@ -35838,7 +35853,7 @@
       <c r="K32" s="112"/>
       <c r="L32" s="110">
         <f t="shared" si="2"/>
-        <v>606.44057104913679</v>
+        <v>603.64057104913684</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
@@ -35874,7 +35889,7 @@
       <c r="K33" s="112"/>
       <c r="L33" s="110">
         <f t="shared" si="2"/>
-        <v>150.12544251565168</v>
+        <v>149.28544251565168</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
@@ -35910,7 +35925,7 @@
       <c r="K34" s="112"/>
       <c r="L34" s="110">
         <f t="shared" si="2"/>
-        <v>442.69333020857749</v>
+        <v>440.45333020857748</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
@@ -35946,7 +35961,7 @@
       <c r="K35" s="112"/>
       <c r="L35" s="110">
         <f t="shared" si="2"/>
-        <v>221.34666510428875</v>
+        <v>220.22666510428874</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
@@ -35982,7 +35997,7 @@
       <c r="K36" s="112"/>
       <c r="L36" s="110">
         <f t="shared" si="2"/>
-        <v>332.01999765643308</v>
+        <v>330.33999765643307</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
@@ -36018,7 +36033,7 @@
       <c r="K37" s="112"/>
       <c r="L37" s="110">
         <f t="shared" si="2"/>
-        <v>664.03999531286615</v>
+        <v>660.67999531286614</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
@@ -36054,7 +36069,7 @@
       <c r="K38" s="112"/>
       <c r="L38" s="110">
         <f t="shared" si="2"/>
-        <v>553.36666276072185</v>
+        <v>550.5666627607219</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
@@ -36093,7 +36108,7 @@
       </c>
       <c r="L39" s="110">
         <f t="shared" si="2"/>
-        <v>332.01999765643308</v>
+        <v>330.33999765643307</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
@@ -36156,7 +36171,7 @@
       <c r="K41" s="112"/>
       <c r="L41" s="110">
         <f t="shared" si="2"/>
-        <v>363.86434262948211</v>
+        <v>362.1843426294821</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
@@ -36192,7 +36207,7 @@
       <c r="K42" s="112"/>
       <c r="L42" s="110">
         <f t="shared" si="2"/>
-        <v>60.644057104913685</v>
+        <v>60.364057104913684</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.3">
@@ -36252,7 +36267,7 @@
       <c r="K44" s="112"/>
       <c r="L44" s="110">
         <f t="shared" si="2"/>
-        <v>1100.9199117814458</v>
+        <v>1094.7599117814457</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -36285,7 +36300,7 @@
       <c r="K45" s="112"/>
       <c r="L45" s="110">
         <f t="shared" si="2"/>
-        <v>300.25088503130337</v>
+        <v>298.57088503130336</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -36318,7 +36333,7 @@
       <c r="K46" s="112"/>
       <c r="L46" s="110">
         <f t="shared" si="2"/>
-        <v>1328.0799906257323</v>
+        <v>1321.3599906257323</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
@@ -36351,7 +36366,7 @@
       <c r="K47" s="112"/>
       <c r="L47" s="110">
         <f t="shared" si="2"/>
-        <v>600.50177006260674</v>
+        <v>597.14177006260672</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
@@ -36384,7 +36399,7 @@
       <c r="K48" s="112"/>
       <c r="L48" s="110">
         <f t="shared" si="2"/>
-        <v>1106.7333255214437</v>
+        <v>1101.1333255214438</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.3">
@@ -36417,7 +36432,7 @@
       <c r="K49" s="112"/>
       <c r="L49" s="110">
         <f t="shared" si="2"/>
-        <v>553.36666276072185</v>
+        <v>550.5666627607219</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.3">
@@ -36450,7 +36465,7 @@
       <c r="K50" s="112"/>
       <c r="L50" s="110">
         <f t="shared" si="2"/>
-        <v>300.25088503130337</v>
+        <v>298.57088503130336</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.3">
@@ -36513,7 +36528,7 @@
       <c r="K52" s="112"/>
       <c r="L52" s="110">
         <f t="shared" si="2"/>
-        <v>300.25088503130337</v>
+        <v>298.57088503130336</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.3">
@@ -36549,7 +36564,7 @@
       <c r="K53" s="112"/>
       <c r="L53" s="110">
         <f t="shared" si="2"/>
-        <v>200.1672566875356</v>
+        <v>199.04725668753559</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.3">
@@ -36585,7 +36600,7 @@
       <c r="K54" s="112"/>
       <c r="L54" s="110">
         <f t="shared" si="2"/>
-        <v>250.20907085941951</v>
+        <v>248.80907085941948</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.3">
@@ -36621,7 +36636,7 @@
       <c r="K55" s="112"/>
       <c r="L55" s="110">
         <f t="shared" si="2"/>
-        <v>150.12544251565168</v>
+        <v>149.28544251565168</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.3">
@@ -36657,7 +36672,7 @@
       <c r="K56" s="112"/>
       <c r="L56" s="110">
         <f t="shared" si="2"/>
-        <v>200.1672566875356</v>
+        <v>199.04725668753559</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.3">
@@ -36693,7 +36708,7 @@
       <c r="K57" s="112"/>
       <c r="L57" s="110">
         <f t="shared" si="2"/>
-        <v>250.20907085941951</v>
+        <v>248.80907085941948</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.3">
@@ -36729,7 +36744,7 @@
       <c r="K58" s="112"/>
       <c r="L58" s="110">
         <f t="shared" si="2"/>
-        <v>150.12544251565168</v>
+        <v>149.28544251565168</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.3">
@@ -36765,7 +36780,7 @@
       <c r="K59" s="112"/>
       <c r="L59" s="110">
         <f t="shared" si="2"/>
-        <v>150.12544251565168</v>
+        <v>149.28544251565168</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
@@ -36801,7 +36816,7 @@
       <c r="K60" s="112"/>
       <c r="L60" s="110">
         <f t="shared" si="2"/>
-        <v>110.67333255214437</v>
+        <v>110.11333255214437</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.3">
@@ -36864,7 +36879,7 @@
       <c r="K62" s="112"/>
       <c r="L62" s="110">
         <f t="shared" si="2"/>
-        <v>61.27212534477475</v>
+        <v>60.992125344774749</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.3">
@@ -36900,7 +36915,7 @@
       <c r="K63" s="112"/>
       <c r="L63" s="110">
         <f t="shared" si="2"/>
-        <v>61.27212534477475</v>
+        <v>60.992125344774749</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.3">
@@ -36936,7 +36951,7 @@
       <c r="K64" s="112"/>
       <c r="L64" s="110">
         <f t="shared" si="2"/>
-        <v>56.710459339114131</v>
+        <v>56.43045933911413</v>
       </c>
     </row>
     <row r="65" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -36972,7 +36987,7 @@
       <c r="K65" s="112"/>
       <c r="L65" s="110">
         <f t="shared" si="2"/>
-        <v>113.42091867822826</v>
+        <v>112.86091867822826</v>
       </c>
     </row>
     <row r="66" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -37008,7 +37023,7 @@
       <c r="K66" s="112"/>
       <c r="L66" s="110">
         <f t="shared" si="2"/>
-        <v>183.81637603432424</v>
+        <v>182.97637603432423</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.3">
@@ -37044,7 +37059,7 @@
       <c r="K67" s="112"/>
       <c r="L67" s="110">
         <f t="shared" si="2"/>
-        <v>107.29853834661354</v>
+        <v>106.73853834661354</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.3">
@@ -37080,7 +37095,7 @@
       <c r="K68" s="112"/>
       <c r="L68" s="110">
         <f t="shared" ref="L68:L73" si="9">IFERROR(I68+($P$10*F68),"")</f>
-        <v>181.93217131474105</v>
+        <v>181.09217131474105</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.3">
@@ -37116,7 +37131,7 @@
       <c r="K69" s="112"/>
       <c r="L69" s="110">
         <f t="shared" si="9"/>
-        <v>332.01999765643308</v>
+        <v>330.33999765643307</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.3">
@@ -37152,7 +37167,7 @@
       <c r="K70" s="112"/>
       <c r="L70" s="110">
         <f t="shared" si="9"/>
-        <v>110.67333255214437</v>
+        <v>110.11333255214437</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.3">
@@ -37188,7 +37203,7 @@
       <c r="K71" s="112"/>
       <c r="L71" s="110">
         <f t="shared" si="9"/>
-        <v>276.68333138036093</v>
+        <v>275.28333138036095</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.3">
@@ -37224,7 +37239,7 @@
       <c r="K72" s="112"/>
       <c r="L72" s="110">
         <f t="shared" si="9"/>
-        <v>61.27212534477475</v>
+        <v>60.992125344774749</v>
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.3">
@@ -37260,29 +37275,29 @@
       <c r="K73" s="113"/>
       <c r="L73" s="110">
         <f t="shared" si="9"/>
-        <v>61.27212534477475</v>
+        <v>60.992125344774749</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A74" s="127" t="s">
+      <c r="A74" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="B74" s="128"/>
-      <c r="C74" s="128"/>
-      <c r="D74" s="128"/>
-      <c r="E74" s="128"/>
-      <c r="F74" s="128"/>
-      <c r="G74" s="128"/>
-      <c r="H74" s="128"/>
-      <c r="I74" s="128"/>
-      <c r="J74" s="128"/>
+      <c r="B74" s="131"/>
+      <c r="C74" s="131"/>
+      <c r="D74" s="131"/>
+      <c r="E74" s="131"/>
+      <c r="F74" s="131"/>
+      <c r="G74" s="131"/>
+      <c r="H74" s="131"/>
+      <c r="I74" s="131"/>
+      <c r="J74" s="131"/>
       <c r="K74" s="114">
         <f>SUM(K3:K73)</f>
         <v>13383.612572529586</v>
       </c>
       <c r="L74" s="111">
         <f>SUM(L3:L73)</f>
-        <v>16945.512572529584</v>
+        <v>16858.712572529592</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.3">
@@ -37290,19 +37305,19 @@
       <c r="L75" s="2"/>
     </row>
     <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="133" t="s">
+      <c r="A76" s="132" t="s">
         <v>192</v>
       </c>
-      <c r="B76" s="134"/>
-      <c r="C76" s="134"/>
-      <c r="D76" s="134"/>
-      <c r="E76" s="134"/>
-      <c r="F76" s="134"/>
-      <c r="G76" s="134"/>
-      <c r="H76" s="134"/>
-      <c r="I76" s="134"/>
-      <c r="J76" s="134"/>
-      <c r="K76" s="135"/>
+      <c r="B76" s="133"/>
+      <c r="C76" s="133"/>
+      <c r="D76" s="133"/>
+      <c r="E76" s="133"/>
+      <c r="F76" s="133"/>
+      <c r="G76" s="133"/>
+      <c r="H76" s="133"/>
+      <c r="I76" s="133"/>
+      <c r="J76" s="133"/>
+      <c r="K76" s="134"/>
       <c r="L76" s="124"/>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.3">
@@ -37421,18 +37436,18 @@
       <c r="L80" s="116"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A81" s="127" t="s">
+      <c r="A81" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="B81" s="128"/>
-      <c r="C81" s="128"/>
-      <c r="D81" s="128"/>
-      <c r="E81" s="128"/>
-      <c r="F81" s="128"/>
-      <c r="G81" s="128"/>
-      <c r="H81" s="128"/>
-      <c r="I81" s="128"/>
-      <c r="J81" s="128"/>
+      <c r="B81" s="131"/>
+      <c r="C81" s="131"/>
+      <c r="D81" s="131"/>
+      <c r="E81" s="131"/>
+      <c r="F81" s="131"/>
+      <c r="G81" s="131"/>
+      <c r="H81" s="131"/>
+      <c r="I81" s="131"/>
+      <c r="J81" s="131"/>
       <c r="K81" s="114">
         <f>SUM(K78:K80)</f>
         <v>172.5</v>
@@ -37446,12 +37461,12 @@
     </row>
   </sheetData>
   <mergeCells count="6">
+    <mergeCell ref="A81:J81"/>
     <mergeCell ref="A1:K1"/>
     <mergeCell ref="N1:P1"/>
-    <mergeCell ref="N6:O6"/>
+    <mergeCell ref="N5:O5"/>
     <mergeCell ref="A74:J74"/>
     <mergeCell ref="A76:K76"/>
-    <mergeCell ref="A81:J81"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E73" xr:uid="{C5BB27AF-9B30-4FCF-8E44-DCCBC0FC7FF5}">
@@ -37461,844 +37476,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84438618-631B-43FB-9820-9583257CBFE8}">
-  <dimension ref="A1:K56"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="1" max="1" width="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="37.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23.77734375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.88671875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="33" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.77734375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="21.6640625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="23.77734375" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="130" t="s">
-        <v>210</v>
-      </c>
-      <c r="B1" s="131"/>
-      <c r="C1" s="131"/>
-      <c r="D1" s="131"/>
-      <c r="E1" s="132"/>
-      <c r="G1" s="127" t="s">
-        <v>209</v>
-      </c>
-      <c r="H1" s="128"/>
-      <c r="I1" s="129"/>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="13" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="E2" s="14" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" s="119" t="s">
-        <v>205</v>
-      </c>
-      <c r="H2" s="118" t="s">
-        <v>204</v>
-      </c>
-      <c r="I2" s="120" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="123"/>
-      <c r="E3" s="115">
-        <f>SUM(D4:D6)</f>
-        <v>1470.5310082745939</v>
-      </c>
-      <c r="G3" s="5" t="s">
-        <v>6</v>
-      </c>
-      <c r="H3" t="s">
-        <v>206</v>
-      </c>
-      <c r="I3" s="121">
-        <f>E54</f>
-        <v>16945.512572529587</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D4" s="123">
-        <f>Costs_final!L4</f>
-        <v>122.5442506895495</v>
-      </c>
-      <c r="E4" s="112"/>
-      <c r="G4" s="127" t="s">
-        <v>115</v>
-      </c>
-      <c r="H4" s="128"/>
-      <c r="I4" s="122">
-        <f>SUM(I3)</f>
-        <v>16945.512572529587</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D5" s="123">
-        <f>Costs_final!L5</f>
-        <v>122.5442506895495</v>
-      </c>
-      <c r="E5" s="112"/>
-      <c r="G5" s="6"/>
-      <c r="I5" s="111"/>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
-      <c r="B6" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="123">
-        <f>SUM(Costs_final!L7:L19)</f>
-        <v>1225.4425068954949</v>
-      </c>
-      <c r="E6" s="112"/>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="6"/>
-      <c r="C7" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="123"/>
-      <c r="E7" s="112">
-        <f>SUM(D8:D17)</f>
-        <v>3088.6202445365593</v>
-      </c>
-      <c r="K7" s="110"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" s="5"/>
-      <c r="B8" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D8" s="123">
-        <f>Costs_final!L21</f>
-        <v>53.64926917330677</v>
-      </c>
-      <c r="E8" s="112"/>
-      <c r="K8" s="110"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" s="5"/>
-      <c r="B9" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" s="123">
-        <f>Costs_final!L22</f>
-        <v>226.84183735645652</v>
-      </c>
-      <c r="E9" s="112"/>
-      <c r="K9" s="110"/>
-    </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" s="5"/>
-      <c r="B10" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="D10" s="123">
-        <f>Costs_final!L23</f>
-        <v>53.64926917330677</v>
-      </c>
-      <c r="E10" s="112"/>
-      <c r="K10" s="110"/>
-    </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" s="5"/>
-      <c r="B11" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="D11" s="123">
-        <f>Costs_final!L24</f>
-        <v>53.64926917330677</v>
-      </c>
-      <c r="E11" s="112"/>
-      <c r="K11" s="110"/>
-    </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" s="5"/>
-      <c r="B12" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" s="123">
-        <f>Costs_final!L25</f>
-        <v>107.29853834661354</v>
-      </c>
-      <c r="E12" s="112"/>
-      <c r="K12" s="110"/>
-    </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" s="5"/>
-      <c r="B13" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="D13" s="123">
-        <f>Costs_final!L26</f>
-        <v>340.26275603468474</v>
-      </c>
-      <c r="E13" s="112"/>
-    </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" s="5"/>
-      <c r="B14" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D14" s="123">
-        <f>Costs_final!L27</f>
-        <v>1180.283921812749</v>
-      </c>
-      <c r="E14" s="112"/>
-    </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" s="5"/>
-      <c r="B15" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="D15" s="123">
-        <f>Costs_final!L28</f>
-        <v>429.19415338645416</v>
-      </c>
-      <c r="E15" s="112"/>
-    </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" s="5"/>
-      <c r="B16" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="D16" s="123">
-        <f>Costs_final!L29</f>
-        <v>214.59707669322708</v>
-      </c>
-      <c r="E16" s="112"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A17" s="5"/>
-      <c r="B17" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D17" s="123">
-        <f>Costs_final!L30</f>
-        <v>429.19415338645416</v>
-      </c>
-      <c r="E17" s="112"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B18" s="6"/>
-      <c r="C18" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D18" s="123" t="str">
-        <f>Costs_final!L31</f>
-        <v/>
-      </c>
-      <c r="E18" s="112">
-        <f>SUM(D19:D25)</f>
-        <v>2970.032664607676</v>
-      </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A19" s="5"/>
-      <c r="B19" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="D19" s="123">
-        <f>Costs_final!L32</f>
-        <v>606.44057104913679</v>
-      </c>
-      <c r="E19" s="112"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A20" s="5"/>
-      <c r="B20" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C20" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" s="123">
-        <f>Costs_final!L33</f>
-        <v>150.12544251565168</v>
-      </c>
-      <c r="E20" s="112"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="5"/>
-      <c r="B21" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" s="123">
-        <f>Costs_final!L34</f>
-        <v>442.69333020857749</v>
-      </c>
-      <c r="E21" s="112"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="5"/>
-      <c r="B22" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C22" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D22" s="123">
-        <f>Costs_final!L35</f>
-        <v>221.34666510428875</v>
-      </c>
-      <c r="E22" s="112"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="5"/>
-      <c r="B23" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="D23" s="123">
-        <f>Costs_final!L36</f>
-        <v>332.01999765643308</v>
-      </c>
-      <c r="E23" s="112"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="5"/>
-      <c r="B24" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C24" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="D24" s="123">
-        <f>Costs_final!L37</f>
-        <v>664.03999531286615</v>
-      </c>
-      <c r="E24" s="112"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A25" s="5"/>
-      <c r="B25" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>194</v>
-      </c>
-      <c r="D25" s="123">
-        <f>Costs_final!L38</f>
-        <v>553.36666276072185</v>
-      </c>
-      <c r="E25" s="112"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A26" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="B26" s="6"/>
-      <c r="C26" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="D26" s="123">
-        <f>Costs_final!L39</f>
-        <v>332.01999765643308</v>
-      </c>
-      <c r="E26" s="111">
-        <f>D26</f>
-        <v>332.01999765643308</v>
-      </c>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" s="6"/>
-      <c r="C27" s="7" t="s">
-        <v>56</v>
-      </c>
-      <c r="D27" s="123" t="str">
-        <f>Costs_final!L40</f>
-        <v/>
-      </c>
-      <c r="E27" s="112">
-        <f>SUM(D28:D30)</f>
-        <v>5714.6118305489526</v>
-      </c>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="5"/>
-      <c r="B28" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C28" s="1" t="s">
-        <v>57</v>
-      </c>
-      <c r="D28" s="123">
-        <f>Costs_final!L41</f>
-        <v>363.86434262948211</v>
-      </c>
-      <c r="E28" s="112"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A29" s="5"/>
-      <c r="B29" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="D29" s="123">
-        <f>Costs_final!L42</f>
-        <v>60.644057104913685</v>
-      </c>
-      <c r="E29" s="112"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A30" s="5"/>
-      <c r="B30" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C30" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="D30" s="123">
-        <f>SUM(Costs_final!L44:L50)</f>
-        <v>5290.1034308145572</v>
-      </c>
-      <c r="E30" s="112"/>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B31" s="6"/>
-      <c r="C31" s="7" t="s">
-        <v>66</v>
-      </c>
-      <c r="D31" s="123"/>
-      <c r="E31" s="112">
-        <f>SUM(D32:D40)</f>
-        <v>1762.0532002243128</v>
-      </c>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A32" s="5"/>
-      <c r="B32" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C32" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="D32" s="123">
-        <f>Costs_final!L52</f>
-        <v>300.25088503130337</v>
-      </c>
-      <c r="E32" s="112"/>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A33" s="5"/>
-      <c r="B33" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C33" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="D33" s="123">
-        <f>Costs_final!L53</f>
-        <v>200.1672566875356</v>
-      </c>
-      <c r="E33" s="112"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="5"/>
-      <c r="B34" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C34" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="D34" s="123">
-        <f>Costs_final!L54</f>
-        <v>250.20907085941951</v>
-      </c>
-      <c r="E34" s="112"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="5"/>
-      <c r="B35" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C35" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="D35" s="123">
-        <f>Costs_final!L55</f>
-        <v>150.12544251565168</v>
-      </c>
-      <c r="E35" s="112"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="5"/>
-      <c r="B36" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C36" s="1" t="s">
-        <v>196</v>
-      </c>
-      <c r="D36" s="123">
-        <f>Costs_final!L56</f>
-        <v>200.1672566875356</v>
-      </c>
-      <c r="E36" s="112"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A37" s="5"/>
-      <c r="B37" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C37" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="D37" s="123">
-        <f>Costs_final!L57</f>
-        <v>250.20907085941951</v>
-      </c>
-      <c r="E37" s="112"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="5"/>
-      <c r="B38" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C38" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="D38" s="123">
-        <f>Costs_final!L58</f>
-        <v>150.12544251565168</v>
-      </c>
-      <c r="E38" s="112"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="5"/>
-      <c r="B39" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C39" s="1" t="s">
-        <v>193</v>
-      </c>
-      <c r="D39" s="123">
-        <f>Costs_final!L59</f>
-        <v>150.12544251565168</v>
-      </c>
-      <c r="E39" s="112"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="5"/>
-      <c r="B40" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C40" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D40" s="123">
-        <f>Costs_final!L60</f>
-        <v>110.67333255214437</v>
-      </c>
-      <c r="E40" s="112"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="5" t="s">
-        <v>87</v>
-      </c>
-      <c r="B41" s="6"/>
-      <c r="C41" s="7" t="s">
-        <v>74</v>
-      </c>
-      <c r="D41" s="123" t="str">
-        <f>Costs_final!L61</f>
-        <v/>
-      </c>
-      <c r="E41" s="112">
-        <f>SUM(D42:D53)</f>
-        <v>1607.6436266810585</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A42" s="5"/>
-      <c r="B42" s="6" t="s">
-        <v>7</v>
-      </c>
-      <c r="C42" s="1" t="s">
-        <v>75</v>
-      </c>
-      <c r="D42" s="123">
-        <f>Costs_final!L62</f>
-        <v>61.27212534477475</v>
-      </c>
-      <c r="E42" s="112"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A43" s="5"/>
-      <c r="B43" s="6" t="s">
-        <v>13</v>
-      </c>
-      <c r="C43" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="D43" s="123">
-        <f>Costs_final!L63</f>
-        <v>61.27212534477475</v>
-      </c>
-      <c r="E43" s="112"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A44" s="5"/>
-      <c r="B44" s="6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C44" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="D44" s="123">
-        <f>Costs_final!L64</f>
-        <v>56.710459339114131</v>
-      </c>
-      <c r="E44" s="112"/>
-    </row>
-    <row r="45" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A45" s="5"/>
-      <c r="B45" s="6" t="s">
-        <v>94</v>
-      </c>
-      <c r="C45" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="D45" s="123">
-        <f>Costs_final!L65</f>
-        <v>113.42091867822826</v>
-      </c>
-      <c r="E45" s="112"/>
-    </row>
-    <row r="46" spans="1:5" ht="28.8" x14ac:dyDescent="0.3">
-      <c r="A46" s="5"/>
-      <c r="B46" s="6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C46" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="D46" s="123">
-        <f>Costs_final!L66</f>
-        <v>183.81637603432424</v>
-      </c>
-      <c r="E46" s="112"/>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A47" s="5"/>
-      <c r="B47" s="6" t="s">
-        <v>96</v>
-      </c>
-      <c r="C47" s="1" t="s">
-        <v>80</v>
-      </c>
-      <c r="D47" s="123">
-        <f>Costs_final!L67</f>
-        <v>107.29853834661354</v>
-      </c>
-      <c r="E47" s="112"/>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="5"/>
-      <c r="B48" s="6" t="s">
-        <v>97</v>
-      </c>
-      <c r="C48" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="D48" s="123">
-        <f>Costs_final!L68</f>
-        <v>181.93217131474105</v>
-      </c>
-      <c r="E48" s="112"/>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="5"/>
-      <c r="B49" s="6" t="s">
-        <v>98</v>
-      </c>
-      <c r="C49" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="D49" s="123">
-        <f>Costs_final!L69</f>
-        <v>332.01999765643308</v>
-      </c>
-      <c r="E49" s="112"/>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A50" s="5"/>
-      <c r="B50" s="6" t="s">
-        <v>99</v>
-      </c>
-      <c r="C50" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="D50" s="123">
-        <f>Costs_final!L70</f>
-        <v>110.67333255214437</v>
-      </c>
-      <c r="E50" s="112"/>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A51" s="5"/>
-      <c r="B51" s="6" t="s">
-        <v>100</v>
-      </c>
-      <c r="C51" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="D51" s="123">
-        <f>Costs_final!L71</f>
-        <v>276.68333138036093</v>
-      </c>
-      <c r="E51" s="112"/>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A52" s="5"/>
-      <c r="B52" s="6" t="s">
-        <v>101</v>
-      </c>
-      <c r="C52" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="D52" s="123">
-        <f>Costs_final!L72</f>
-        <v>61.27212534477475</v>
-      </c>
-      <c r="E52" s="112"/>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A53" s="8"/>
-      <c r="B53" s="9" t="s">
-        <v>102</v>
-      </c>
-      <c r="C53" s="10" t="s">
-        <v>86</v>
-      </c>
-      <c r="D53" s="123">
-        <f>Costs_final!L73</f>
-        <v>61.27212534477475</v>
-      </c>
-      <c r="E53" s="113"/>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="127" t="s">
-        <v>4</v>
-      </c>
-      <c r="B54" s="128"/>
-      <c r="C54" s="128"/>
-      <c r="D54" s="128"/>
-      <c r="E54" s="114">
-        <f>SUM(E3:E53)</f>
-        <v>16945.512572529587</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="E55" s="2"/>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A56" s="6"/>
-      <c r="B56" s="6"/>
-    </row>
-  </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="G1:I1"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="A54:D54"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
docs: documents most of the tools and languages
</commit_message>
<xml_diff>
--- a/docs/budget.xlsx
+++ b/docs/budget.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javie\Desktop\proyectos\IRBoard\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACF91FD6-6829-470F-87AD-E183670224AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0BE4025-46F3-4B5F-AD18-B937C6BD7178}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Company definition" sheetId="2" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="221">
   <si>
     <t>I1</t>
   </si>
@@ -691,6 +691,18 @@
   <si>
     <t>deviation from original</t>
   </si>
+  <si>
+    <t>deviation</t>
+  </si>
+  <si>
+    <t>Actual profit</t>
+  </si>
+  <si>
+    <t>Profit deviation</t>
+  </si>
+  <si>
+    <t>estimated client cost:</t>
+  </si>
 </sst>
 </file>
 
@@ -1340,6 +1352,13 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1349,10 +1368,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1364,11 +1380,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -31010,27 +31022,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="130" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="128"/>
-      <c r="C1" s="128"/>
-      <c r="D1" s="128"/>
-      <c r="E1" s="128"/>
-      <c r="F1" s="128"/>
-      <c r="G1" s="128"/>
-      <c r="H1" s="128"/>
-      <c r="I1" s="128"/>
-      <c r="J1" s="128"/>
-      <c r="K1" s="129"/>
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
+      <c r="F1" s="131"/>
+      <c r="G1" s="131"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="131"/>
+      <c r="J1" s="131"/>
+      <c r="K1" s="132"/>
       <c r="L1" s="125" t="s">
         <v>213</v>
       </c>
-      <c r="N1" s="130" t="s">
+      <c r="N1" s="128" t="s">
         <v>203</v>
       </c>
-      <c r="O1" s="131"/>
-      <c r="P1" s="135"/>
+      <c r="O1" s="129"/>
+      <c r="P1" s="133"/>
     </row>
     <row r="2" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -31145,7 +31157,7 @@
       </c>
       <c r="K4" s="112"/>
       <c r="L4" s="110">
-        <f t="shared" ref="L4:L67" si="2">IFERROR(I4+($P$10*F4),"")</f>
+        <f>IFERROR(I4+($P$10*F4),"")</f>
         <v>122.72425068954949</v>
       </c>
       <c r="N4" s="5" t="s">
@@ -31191,13 +31203,13 @@
       </c>
       <c r="K5" s="112"/>
       <c r="L5" s="110">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="L4:L67" si="2">IFERROR(I5+($P$10*F5),"")</f>
         <v>122.72425068954949</v>
       </c>
-      <c r="N5" s="130" t="s">
+      <c r="N5" s="128" t="s">
         <v>115</v>
       </c>
-      <c r="O5" s="131"/>
+      <c r="O5" s="129"/>
       <c r="P5" s="122">
         <f>SUM(P3:P4)</f>
         <v>13199.017352669423</v>
@@ -31419,6 +31431,13 @@
         <f t="shared" si="2"/>
         <v>122.72425068954949</v>
       </c>
+      <c r="O11" t="s">
+        <v>220</v>
+      </c>
+      <c r="P11" s="111">
+        <f>P5+P7</f>
+        <v>16498.77169083678</v>
+      </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.3">
       <c r="A12" s="5"/>
@@ -33605,18 +33624,18 @@
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A74" s="130" t="s">
+      <c r="A74" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="B74" s="131"/>
-      <c r="C74" s="131"/>
-      <c r="D74" s="131"/>
-      <c r="E74" s="131"/>
-      <c r="F74" s="131"/>
-      <c r="G74" s="131"/>
-      <c r="H74" s="131"/>
-      <c r="I74" s="131"/>
-      <c r="J74" s="131"/>
+      <c r="B74" s="129"/>
+      <c r="C74" s="129"/>
+      <c r="D74" s="129"/>
+      <c r="E74" s="129"/>
+      <c r="F74" s="129"/>
+      <c r="G74" s="129"/>
+      <c r="H74" s="129"/>
+      <c r="I74" s="129"/>
+      <c r="J74" s="129"/>
       <c r="K74" s="114">
         <f>SUM(K3:K73)</f>
         <v>13026.517352669423</v>
@@ -33631,19 +33650,19 @@
       <c r="L75" s="2"/>
     </row>
     <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="132" t="s">
+      <c r="A76" s="134" t="s">
         <v>192</v>
       </c>
-      <c r="B76" s="133"/>
-      <c r="C76" s="133"/>
-      <c r="D76" s="133"/>
-      <c r="E76" s="133"/>
-      <c r="F76" s="133"/>
-      <c r="G76" s="133"/>
-      <c r="H76" s="133"/>
-      <c r="I76" s="133"/>
-      <c r="J76" s="133"/>
-      <c r="K76" s="134"/>
+      <c r="B76" s="135"/>
+      <c r="C76" s="135"/>
+      <c r="D76" s="135"/>
+      <c r="E76" s="135"/>
+      <c r="F76" s="135"/>
+      <c r="G76" s="135"/>
+      <c r="H76" s="135"/>
+      <c r="I76" s="135"/>
+      <c r="J76" s="135"/>
+      <c r="K76" s="136"/>
       <c r="L76" s="124"/>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.3">
@@ -33762,18 +33781,18 @@
       <c r="L80" s="116"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A81" s="130" t="s">
+      <c r="A81" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="B81" s="131"/>
-      <c r="C81" s="131"/>
-      <c r="D81" s="131"/>
-      <c r="E81" s="131"/>
-      <c r="F81" s="131"/>
-      <c r="G81" s="131"/>
-      <c r="H81" s="131"/>
-      <c r="I81" s="131"/>
-      <c r="J81" s="131"/>
+      <c r="B81" s="129"/>
+      <c r="C81" s="129"/>
+      <c r="D81" s="129"/>
+      <c r="E81" s="129"/>
+      <c r="F81" s="129"/>
+      <c r="G81" s="129"/>
+      <c r="H81" s="129"/>
+      <c r="I81" s="129"/>
+      <c r="J81" s="129"/>
       <c r="K81" s="114">
         <f>SUM(K78:K80)</f>
         <v>172.5</v>
@@ -33795,7 +33814,7 @@
     <mergeCell ref="N5:O5"/>
   </mergeCells>
   <phoneticPr fontId="4" type="noConversion"/>
-  <dataValidations count="1">
+  <dataValidations disablePrompts="1" count="1">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E3:E73" xr:uid="{2FF9A132-8776-4FE0-B050-ADA1CD0962E0}">
       <formula1>$Q$20:$Q$25</formula1>
     </dataValidation>
@@ -33823,18 +33842,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="130" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="128"/>
-      <c r="C1" s="128"/>
-      <c r="D1" s="128"/>
-      <c r="E1" s="129"/>
-      <c r="G1" s="130" t="s">
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="132"/>
+      <c r="G1" s="128" t="s">
         <v>209</v>
       </c>
-      <c r="H1" s="131"/>
-      <c r="I1" s="135"/>
+      <c r="H1" s="129"/>
+      <c r="I1" s="133"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -33899,10 +33918,10 @@
         <v>122.72425068954949</v>
       </c>
       <c r="E4" s="112"/>
-      <c r="G4" s="130" t="s">
+      <c r="G4" s="128" t="s">
         <v>115</v>
       </c>
-      <c r="H4" s="131"/>
+      <c r="H4" s="129"/>
       <c r="I4" s="122">
         <f>SUM(I3)</f>
         <v>16500.517352669427</v>
@@ -34615,12 +34634,12 @@
       <c r="E53" s="113"/>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="130" t="s">
+      <c r="A54" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="B54" s="131"/>
-      <c r="C54" s="131"/>
-      <c r="D54" s="131"/>
+      <c r="B54" s="129"/>
+      <c r="C54" s="129"/>
+      <c r="D54" s="129"/>
       <c r="E54" s="114">
         <f>SUM(E3:E53)</f>
         <v>16500.517352669427</v>
@@ -34667,27 +34686,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="127" t="s">
+      <c r="A1" s="130" t="s">
         <v>191</v>
       </c>
-      <c r="B1" s="128"/>
-      <c r="C1" s="128"/>
-      <c r="D1" s="128"/>
-      <c r="E1" s="128"/>
-      <c r="F1" s="128"/>
-      <c r="G1" s="128"/>
-      <c r="H1" s="128"/>
-      <c r="I1" s="128"/>
-      <c r="J1" s="128"/>
-      <c r="K1" s="129"/>
-      <c r="L1" s="125" t="s">
-        <v>213</v>
-      </c>
-      <c r="N1" s="130" t="s">
+      <c r="B1" s="131"/>
+      <c r="C1" s="131"/>
+      <c r="D1" s="131"/>
+      <c r="E1" s="131"/>
+      <c r="F1" s="131"/>
+      <c r="G1" s="131"/>
+      <c r="H1" s="131"/>
+      <c r="I1" s="131"/>
+      <c r="J1" s="131"/>
+      <c r="K1" s="132"/>
+      <c r="L1" s="125"/>
+      <c r="N1" s="128" t="s">
         <v>203</v>
       </c>
-      <c r="O1" s="131"/>
-      <c r="P1" s="135"/>
+      <c r="O1" s="129"/>
+      <c r="P1" s="133"/>
     </row>
     <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="12" t="s">
@@ -34723,7 +34740,9 @@
       <c r="K2" s="14" t="s">
         <v>4</v>
       </c>
-      <c r="L2" s="118"/>
+      <c r="L2" s="118" t="s">
+        <v>217</v>
+      </c>
       <c r="N2" s="119" t="s">
         <v>205</v>
       </c>
@@ -34733,7 +34752,7 @@
       <c r="P2" s="120" t="s">
         <v>4</v>
       </c>
-      <c r="Q2" s="136" t="s">
+      <c r="Q2" s="118" t="s">
         <v>216</v>
       </c>
     </row>
@@ -34758,9 +34777,9 @@
         <f>SUM(J4:J19)</f>
         <v>1194.7710082745937</v>
       </c>
-      <c r="L3" s="110" t="str">
-        <f>IFERROR(I3+($P$10*F3),"")</f>
-        <v/>
+      <c r="L3" s="127">
+        <f>((K3-Costs_init!K3)/Costs_init!K3)</f>
+        <v>-0.19999999999999998</v>
       </c>
       <c r="N3" s="5" t="s">
         <v>6</v>
@@ -34772,7 +34791,7 @@
         <f>K74</f>
         <v>13383.612572529586</v>
       </c>
-      <c r="Q3" s="137">
+      <c r="Q3" s="127">
         <f>((P3-Costs_init!P3)/Costs_init!P3)</f>
         <v>2.7412946238235029E-2</v>
       </c>
@@ -34808,9 +34827,9 @@
         <v>99.564250689549496</v>
       </c>
       <c r="K4" s="112"/>
-      <c r="L4" s="110">
-        <f t="shared" ref="L4:L67" si="2">IFERROR(I4+($P$10*F4),"")</f>
-        <v>121.9842506895495</v>
+      <c r="L4" s="127">
+        <f>((J4-Costs_init!J4)/Costs_init!J4)</f>
+        <v>0</v>
       </c>
       <c r="N4" s="5" t="s">
         <v>8</v>
@@ -34822,7 +34841,7 @@
         <f>K81</f>
         <v>172.5</v>
       </c>
-      <c r="Q4" s="137">
+      <c r="Q4" s="127">
         <f>((P4-Costs_init!P4)/Costs_init!P4)</f>
         <v>0</v>
       </c>
@@ -34858,19 +34877,19 @@
         <v>99.564250689549496</v>
       </c>
       <c r="K5" s="112"/>
-      <c r="L5" s="110">
-        <f t="shared" si="2"/>
-        <v>121.9842506895495</v>
-      </c>
-      <c r="N5" s="130" t="s">
+      <c r="L5" s="127">
+        <f>((J5-Costs_init!J5)/Costs_init!J5)</f>
+        <v>0</v>
+      </c>
+      <c r="N5" s="128" t="s">
         <v>115</v>
       </c>
-      <c r="O5" s="131"/>
+      <c r="O5" s="129"/>
       <c r="P5" s="122">
         <f>SUM(P3:P4)</f>
         <v>13556.112572529586</v>
       </c>
-      <c r="Q5" s="137">
+      <c r="Q5" s="127">
         <f>((P5-Costs_init!P5)/Costs_init!P5)</f>
         <v>2.7054682202379422E-2</v>
       </c>
@@ -34897,8 +34916,11 @@
         <v>995.64250689549476</v>
       </c>
       <c r="K6" s="112"/>
-      <c r="L6" s="110"/>
-      <c r="Q6" s="137"/>
+      <c r="L6" s="127">
+        <f>((J6-Costs_init!J6)/Costs_init!J6)</f>
+        <v>-0.23076923076923073</v>
+      </c>
+      <c r="Q6" s="127"/>
     </row>
     <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A7" s="5"/>
@@ -34928,18 +34950,18 @@
       </c>
       <c r="J7" s="111"/>
       <c r="K7" s="112"/>
-      <c r="L7" s="110">
-        <f t="shared" si="2"/>
-        <v>60.992125344774749</v>
+      <c r="L7" s="127">
+        <f>((I7-Costs_init!I7)/Costs_init!I7)</f>
+        <v>-0.5</v>
       </c>
       <c r="O7" t="s">
-        <v>208</v>
-      </c>
-      <c r="P7">
-        <f>Costs_init!P7</f>
-        <v>3299.7543381673559</v>
-      </c>
-      <c r="Q7" s="137"/>
+        <v>218</v>
+      </c>
+      <c r="P7" s="111">
+        <f>Client_init!I4-Costs_final!P5</f>
+        <v>2944.404780139841</v>
+      </c>
+      <c r="Q7" s="127"/>
     </row>
     <row r="8" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A8" s="5"/>
@@ -34969,16 +34991,16 @@
       </c>
       <c r="J8" s="111"/>
       <c r="K8" s="112"/>
-      <c r="L8" s="110">
-        <f t="shared" si="2"/>
-        <v>121.9842506895495</v>
+      <c r="L8" s="127">
+        <f>((I8-Costs_init!I8)/Costs_init!I8)</f>
+        <v>0</v>
       </c>
       <c r="O8" t="s">
-        <v>211</v>
-      </c>
-      <c r="P8" s="111">
-        <f>P5+P7-P3</f>
-        <v>3472.2543381673568</v>
+        <v>219</v>
+      </c>
+      <c r="P8" s="127">
+        <f>((P7-Costs_init!P7)/Costs_init!P7)</f>
+        <v>-0.10768970099297505</v>
       </c>
     </row>
     <row r="9" spans="1:17" x14ac:dyDescent="0.3">
@@ -35009,16 +35031,13 @@
       </c>
       <c r="J9" s="111"/>
       <c r="K9" s="112"/>
-      <c r="L9" s="110">
-        <f t="shared" si="2"/>
-        <v>60.992125344774749</v>
-      </c>
-      <c r="O9" t="s">
-        <v>214</v>
-      </c>
-      <c r="P9" s="126">
-        <f>SUM(F4:F73)</f>
-        <v>310</v>
+      <c r="L9" s="127">
+        <f>((I9-Costs_init!I9)/Costs_init!I9)</f>
+        <v>-0.5</v>
+      </c>
+      <c r="P9" s="123">
+        <f>(0.21)*(P3+P4)</f>
+        <v>2846.7836402312128</v>
       </c>
     </row>
     <row r="10" spans="1:17" x14ac:dyDescent="0.3">
@@ -35049,16 +35068,13 @@
       </c>
       <c r="J10" s="111"/>
       <c r="K10" s="112"/>
-      <c r="L10" s="110">
-        <f t="shared" si="2"/>
-        <v>121.9842506895495</v>
-      </c>
-      <c r="O10" t="s">
-        <v>215</v>
-      </c>
-      <c r="P10" s="123">
-        <f>ROUNDUP(P8/P9,2)</f>
-        <v>11.209999999999999</v>
+      <c r="L10" s="127">
+        <f>((I10-Costs_init!I10)/Costs_init!I10)</f>
+        <v>0</v>
+      </c>
+      <c r="P10" s="137">
+        <f>P5+P9</f>
+        <v>16402.896212760799</v>
       </c>
     </row>
     <row r="11" spans="1:17" x14ac:dyDescent="0.3">
@@ -35089,9 +35105,9 @@
       </c>
       <c r="J11" s="111"/>
       <c r="K11" s="112"/>
-      <c r="L11" s="110">
-        <f t="shared" si="2"/>
-        <v>60.992125344774749</v>
+      <c r="L11" s="127">
+        <f>((I11-Costs_init!I11)/Costs_init!I11)</f>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="12" spans="1:17" x14ac:dyDescent="0.3">
@@ -35122,9 +35138,9 @@
       </c>
       <c r="J12" s="111"/>
       <c r="K12" s="112"/>
-      <c r="L12" s="110">
-        <f t="shared" si="2"/>
-        <v>60.992125344774749</v>
+      <c r="L12" s="127">
+        <f>((I12-Costs_init!I12)/Costs_init!I12)</f>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="13" spans="1:17" x14ac:dyDescent="0.3">
@@ -35155,9 +35171,9 @@
       </c>
       <c r="J13" s="111"/>
       <c r="K13" s="112"/>
-      <c r="L13" s="110">
-        <f t="shared" si="2"/>
-        <v>121.9842506895495</v>
+      <c r="L13" s="127">
+        <f>((I13-Costs_init!I13)/Costs_init!I13)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:17" x14ac:dyDescent="0.3">
@@ -35188,9 +35204,9 @@
       </c>
       <c r="J14" s="111"/>
       <c r="K14" s="112"/>
-      <c r="L14" s="110">
-        <f t="shared" si="2"/>
-        <v>121.9842506895495</v>
+      <c r="L14" s="127">
+        <f>((I14-Costs_init!I14)/Costs_init!I14)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:17" x14ac:dyDescent="0.3">
@@ -35221,9 +35237,9 @@
       </c>
       <c r="J15" s="111"/>
       <c r="K15" s="112"/>
-      <c r="L15" s="110">
-        <f t="shared" si="2"/>
-        <v>121.9842506895495</v>
+      <c r="L15" s="127">
+        <f>((I15-Costs_init!I15)/Costs_init!I15)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="16" spans="1:17" x14ac:dyDescent="0.3">
@@ -35254,9 +35270,9 @@
       </c>
       <c r="J16" s="111"/>
       <c r="K16" s="112"/>
-      <c r="L16" s="110">
-        <f t="shared" si="2"/>
-        <v>121.9842506895495</v>
+      <c r="L16" s="127">
+        <f>((I16-Costs_init!I16)/Costs_init!I16)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:18" x14ac:dyDescent="0.3">
@@ -35287,9 +35303,9 @@
       </c>
       <c r="J17" s="111"/>
       <c r="K17" s="112"/>
-      <c r="L17" s="110">
-        <f t="shared" si="2"/>
-        <v>60.992125344774749</v>
+      <c r="L17" s="127">
+        <f>((I17-Costs_init!I17)/Costs_init!I17)</f>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="18" spans="1:18" x14ac:dyDescent="0.3">
@@ -35320,9 +35336,9 @@
       </c>
       <c r="J18" s="111"/>
       <c r="K18" s="112"/>
-      <c r="L18" s="110">
-        <f t="shared" si="2"/>
-        <v>60.992125344774749</v>
+      <c r="L18" s="127">
+        <f>((I18-Costs_init!I18)/Costs_init!I18)</f>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="19" spans="1:18" x14ac:dyDescent="0.3">
@@ -35353,9 +35369,9 @@
       </c>
       <c r="J19" s="111"/>
       <c r="K19" s="112"/>
-      <c r="L19" s="110">
-        <f t="shared" si="2"/>
-        <v>121.9842506895495</v>
+      <c r="L19" s="127">
+        <f>((I19-Costs_init!I19)/Costs_init!I19)</f>
+        <v>0</v>
       </c>
       <c r="Q19" s="7" t="s">
         <v>105</v>
@@ -35386,9 +35402,9 @@
         <f>SUM(J21:J30)</f>
         <v>2433.690244536559</v>
       </c>
-      <c r="L20" s="110" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+      <c r="L20" s="127">
+        <f>((K20-Costs_init!K20)/Costs_init!K20)</f>
+        <v>5.4818449090653899E-2</v>
       </c>
       <c r="Q20" t="s">
         <v>104</v>
@@ -35425,13 +35441,13 @@
         <v>42.159269173306768</v>
       </c>
       <c r="J21" s="111">
-        <f t="shared" ref="J21:J30" si="3">I21</f>
+        <f t="shared" ref="J21:J30" si="2">I21</f>
         <v>42.159269173306768</v>
       </c>
       <c r="K21" s="112"/>
-      <c r="L21" s="110">
-        <f t="shared" si="2"/>
-        <v>53.369269173306769</v>
+      <c r="L21" s="127">
+        <f>((J21-Costs_init!J21)/Costs_init!J21)</f>
+        <v>0</v>
       </c>
       <c r="Q21" t="s">
         <v>107</v>
@@ -35468,13 +35484,13 @@
         <v>180.88183735645651</v>
       </c>
       <c r="J22" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>180.88183735645651</v>
       </c>
       <c r="K22" s="112"/>
-      <c r="L22" s="110">
-        <f t="shared" si="2"/>
-        <v>225.72183735645652</v>
+      <c r="L22" s="127">
+        <f>((J22-Costs_init!J22)/Costs_init!J22)</f>
+        <v>0</v>
       </c>
       <c r="Q22" t="s">
         <v>106</v>
@@ -35511,13 +35527,13 @@
         <v>42.159269173306768</v>
       </c>
       <c r="J23" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>42.159269173306768</v>
       </c>
       <c r="K23" s="112"/>
-      <c r="L23" s="110">
-        <f t="shared" si="2"/>
-        <v>53.369269173306769</v>
+      <c r="L23" s="127">
+        <f>((J23-Costs_init!J23)/Costs_init!J23)</f>
+        <v>-0.5</v>
       </c>
       <c r="Q23" t="s">
         <v>108</v>
@@ -35554,13 +35570,13 @@
         <v>42.159269173306768</v>
       </c>
       <c r="J24" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>42.159269173306768</v>
       </c>
       <c r="K24" s="112"/>
-      <c r="L24" s="110">
-        <f t="shared" si="2"/>
-        <v>53.369269173306769</v>
+      <c r="L24" s="127">
+        <f>((J24-Costs_init!J24)/Costs_init!J24)</f>
+        <v>0</v>
       </c>
       <c r="Q24" t="s">
         <v>109</v>
@@ -35597,13 +35613,13 @@
         <v>84.318538346613536</v>
       </c>
       <c r="J25" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>84.318538346613536</v>
       </c>
       <c r="K25" s="112"/>
-      <c r="L25" s="110">
-        <f t="shared" si="2"/>
-        <v>106.73853834661354</v>
+      <c r="L25" s="127">
+        <f>((J25-Costs_init!J25)/Costs_init!J25)</f>
+        <v>0</v>
       </c>
       <c r="Q25" t="s">
         <v>110</v>
@@ -35640,13 +35656,13 @@
         <v>271.32275603468474</v>
       </c>
       <c r="J26" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>271.32275603468474</v>
       </c>
       <c r="K26" s="112"/>
-      <c r="L26" s="110">
-        <f t="shared" si="2"/>
-        <v>338.58275603468473</v>
+      <c r="L26" s="127">
+        <f>((J26-Costs_init!J26)/Costs_init!J26)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:18" x14ac:dyDescent="0.3">
@@ -35676,13 +35692,13 @@
         <v>927.5039218127489</v>
       </c>
       <c r="J27" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>927.5039218127489</v>
       </c>
       <c r="K27" s="112"/>
-      <c r="L27" s="110">
-        <f t="shared" si="2"/>
-        <v>1174.1239218127489</v>
+      <c r="L27" s="127">
+        <f>((J27-Costs_init!J27)/Costs_init!J27)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:18" x14ac:dyDescent="0.3">
@@ -35712,13 +35728,13 @@
         <v>337.27415338645415</v>
       </c>
       <c r="J28" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>337.27415338645415</v>
       </c>
       <c r="K28" s="112"/>
-      <c r="L28" s="110">
-        <f t="shared" si="2"/>
-        <v>426.95415338645415</v>
+      <c r="L28" s="127">
+        <f>((J28-Costs_init!J28)/Costs_init!J28)</f>
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="29" spans="1:18" x14ac:dyDescent="0.3">
@@ -35748,13 +35764,13 @@
         <v>168.63707669322707</v>
       </c>
       <c r="J29" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>168.63707669322707</v>
       </c>
       <c r="K29" s="112"/>
-      <c r="L29" s="110">
-        <f t="shared" si="2"/>
-        <v>213.47707669322708</v>
+      <c r="L29" s="127">
+        <f>((J29-Costs_init!J29)/Costs_init!J29)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="30" spans="1:18" x14ac:dyDescent="0.3">
@@ -35784,13 +35800,13 @@
         <v>337.27415338645415</v>
       </c>
       <c r="J30" s="111">
-        <f t="shared" si="3"/>
+        <f t="shared" si="2"/>
         <v>337.27415338645415</v>
       </c>
       <c r="K30" s="112"/>
-      <c r="L30" s="110">
-        <f t="shared" si="2"/>
-        <v>426.95415338645415</v>
+      <c r="L30" s="127">
+        <f>((J30-Costs_init!J30)/Costs_init!J30)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:18" x14ac:dyDescent="0.3">
@@ -35815,9 +35831,9 @@
         <f>SUM(J32:J38)</f>
         <v>2361.0626646076757</v>
       </c>
-      <c r="L31" s="110" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+      <c r="L31" s="127">
+        <f>((K31-Costs_init!K31)/Costs_init!K31)</f>
+        <v>3.8574168884760181E-2</v>
       </c>
     </row>
     <row r="32" spans="1:18" x14ac:dyDescent="0.3">
@@ -35847,13 +35863,13 @@
         <v>491.54057104913682</v>
       </c>
       <c r="J32" s="111">
-        <f t="shared" ref="J32:J38" si="4">I32</f>
+        <f t="shared" ref="J32:J38" si="3">I32</f>
         <v>491.54057104913682</v>
       </c>
       <c r="K32" s="112"/>
-      <c r="L32" s="110">
-        <f t="shared" si="2"/>
-        <v>603.64057104913684</v>
+      <c r="L32" s="127">
+        <f>((J32-Costs_init!J32)/Costs_init!J32)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:12" x14ac:dyDescent="0.3">
@@ -35883,13 +35899,13 @@
         <v>115.65544251565169</v>
       </c>
       <c r="J33" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>115.65544251565169</v>
       </c>
       <c r="K33" s="112"/>
-      <c r="L33" s="110">
-        <f t="shared" si="2"/>
-        <v>149.28544251565168</v>
+      <c r="L33" s="127">
+        <f>((J33-Costs_init!J33)/Costs_init!J33)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="34" spans="1:12" x14ac:dyDescent="0.3">
@@ -35919,13 +35935,13 @@
         <v>350.77333020857748</v>
       </c>
       <c r="J34" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>350.77333020857748</v>
       </c>
       <c r="K34" s="112"/>
-      <c r="L34" s="110">
-        <f t="shared" si="2"/>
-        <v>440.45333020857748</v>
+      <c r="L34" s="127">
+        <f>((J34-Costs_init!J34)/Costs_init!J34)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="35" spans="1:12" x14ac:dyDescent="0.3">
@@ -35955,13 +35971,13 @@
         <v>175.38666510428874</v>
       </c>
       <c r="J35" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>175.38666510428874</v>
       </c>
       <c r="K35" s="112"/>
-      <c r="L35" s="110">
-        <f t="shared" si="2"/>
-        <v>220.22666510428874</v>
+      <c r="L35" s="127">
+        <f>((J35-Costs_init!J35)/Costs_init!J35)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:12" x14ac:dyDescent="0.3">
@@ -35991,13 +36007,13 @@
         <v>263.07999765643308</v>
       </c>
       <c r="J36" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>263.07999765643308</v>
       </c>
       <c r="K36" s="112"/>
-      <c r="L36" s="110">
-        <f t="shared" si="2"/>
-        <v>330.33999765643307</v>
+      <c r="L36" s="127">
+        <f>((J36-Costs_init!J36)/Costs_init!J36)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="37" spans="1:12" x14ac:dyDescent="0.3">
@@ -36027,13 +36043,13 @@
         <v>526.15999531286616</v>
       </c>
       <c r="J37" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>526.15999531286616</v>
       </c>
       <c r="K37" s="112"/>
-      <c r="L37" s="110">
-        <f t="shared" si="2"/>
-        <v>660.67999531286614</v>
+      <c r="L37" s="127">
+        <f>((J37-Costs_init!J37)/Costs_init!J37)</f>
+        <v>0.19999999999999979</v>
       </c>
     </row>
     <row r="38" spans="1:12" x14ac:dyDescent="0.3">
@@ -36063,13 +36079,13 @@
         <v>438.46666276072187</v>
       </c>
       <c r="J38" s="111">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>438.46666276072187</v>
       </c>
       <c r="K38" s="112"/>
-      <c r="L38" s="110">
-        <f t="shared" si="2"/>
-        <v>550.5666627607219</v>
+      <c r="L38" s="127">
+        <f>((J38-Costs_init!J38)/Costs_init!J38)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="39" spans="1:12" x14ac:dyDescent="0.3">
@@ -36106,9 +36122,9 @@
         <f>SUM(J39)</f>
         <v>263.07999765643308</v>
       </c>
-      <c r="L39" s="110">
-        <f t="shared" si="2"/>
-        <v>330.33999765643307</v>
+      <c r="L39" s="127">
+        <f>((K39-Costs_init!K39)/Costs_init!K39)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="40" spans="1:12" x14ac:dyDescent="0.3">
@@ -36133,9 +36149,9 @@
         <f>SUM(J41:J50)</f>
         <v>4485.1818305489533</v>
       </c>
-      <c r="L40" s="110" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+      <c r="L40" s="127">
+        <f>((K40-Costs_init!K40)/Costs_init!K40)</f>
+        <v>2.240376206072581E-2</v>
       </c>
     </row>
     <row r="41" spans="1:12" x14ac:dyDescent="0.3">
@@ -36169,9 +36185,9 @@
         <v>294.92434262948211</v>
       </c>
       <c r="K41" s="112"/>
-      <c r="L41" s="110">
-        <f t="shared" si="2"/>
-        <v>362.1843426294821</v>
+      <c r="L41" s="127">
+        <f>((J41-Costs_init!J41)/Costs_init!J41)</f>
+        <v>0.50000000000000011</v>
       </c>
     </row>
     <row r="42" spans="1:12" x14ac:dyDescent="0.3">
@@ -36205,9 +36221,9 @@
         <v>49.154057104913683</v>
       </c>
       <c r="K42" s="112"/>
-      <c r="L42" s="110">
-        <f t="shared" si="2"/>
-        <v>60.364057104913684</v>
+      <c r="L42" s="127">
+        <f>((J42-Costs_init!J42)/Costs_init!J42)</f>
+        <v>-0.66666666666666674</v>
       </c>
     </row>
     <row r="43" spans="1:12" x14ac:dyDescent="0.3">
@@ -36232,9 +36248,9 @@
         <v>4141.1034308145572</v>
       </c>
       <c r="K43" s="112"/>
-      <c r="L43" s="110" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+      <c r="L43" s="127">
+        <f>((J43-Costs_init!J43)/Costs_init!J43)</f>
+        <v>2.4310512756161532E-2</v>
       </c>
     </row>
     <row r="44" spans="1:12" x14ac:dyDescent="0.3">
@@ -36265,9 +36281,9 @@
       </c>
       <c r="J44" s="111"/>
       <c r="K44" s="112"/>
-      <c r="L44" s="110">
-        <f t="shared" si="2"/>
-        <v>1094.7599117814457</v>
+      <c r="L44" s="127">
+        <f>((I44-Costs_init!I44)/Costs_init!I44)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="45" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -36298,9 +36314,9 @@
       </c>
       <c r="J45" s="111"/>
       <c r="K45" s="112"/>
-      <c r="L45" s="110">
-        <f t="shared" si="2"/>
-        <v>298.57088503130336</v>
+      <c r="L45" s="127">
+        <f>((I45-Costs_init!I45)/Costs_init!I45)</f>
+        <v>-0.40000000000000008</v>
       </c>
     </row>
     <row r="46" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -36331,9 +36347,9 @@
       </c>
       <c r="J46" s="111"/>
       <c r="K46" s="112"/>
-      <c r="L46" s="110">
-        <f t="shared" si="2"/>
-        <v>1321.3599906257323</v>
+      <c r="L46" s="127">
+        <f>((I46-Costs_init!I46)/Costs_init!I46)</f>
+        <v>-4.0000000000000063E-2</v>
       </c>
     </row>
     <row r="47" spans="1:12" x14ac:dyDescent="0.3">
@@ -36364,9 +36380,9 @@
       </c>
       <c r="J47" s="111"/>
       <c r="K47" s="112"/>
-      <c r="L47" s="110">
-        <f t="shared" si="2"/>
-        <v>597.14177006260672</v>
+      <c r="L47" s="127">
+        <f>((I47-Costs_init!I47)/Costs_init!I47)</f>
+        <v>1</v>
       </c>
     </row>
     <row r="48" spans="1:12" x14ac:dyDescent="0.3">
@@ -36397,9 +36413,9 @@
       </c>
       <c r="J48" s="111"/>
       <c r="K48" s="112"/>
-      <c r="L48" s="110">
-        <f t="shared" si="2"/>
-        <v>1101.1333255214438</v>
+      <c r="L48" s="127">
+        <f>((I48-Costs_init!I48)/Costs_init!I48)</f>
+        <v>0.33333333333333331</v>
       </c>
     </row>
     <row r="49" spans="1:12" x14ac:dyDescent="0.3">
@@ -36430,9 +36446,9 @@
       </c>
       <c r="J49" s="111"/>
       <c r="K49" s="112"/>
-      <c r="L49" s="110">
-        <f t="shared" si="2"/>
-        <v>550.5666627607219</v>
+      <c r="L49" s="127">
+        <f>((I49-Costs_init!I49)/Costs_init!I49)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="50" spans="1:12" x14ac:dyDescent="0.3">
@@ -36463,9 +36479,9 @@
       </c>
       <c r="J50" s="111"/>
       <c r="K50" s="112"/>
-      <c r="L50" s="110">
-        <f t="shared" si="2"/>
-        <v>298.57088503130336</v>
+      <c r="L50" s="127">
+        <f>((I50-Costs_init!I50)/Costs_init!I50)</f>
+        <v>-0.40000000000000008</v>
       </c>
     </row>
     <row r="51" spans="1:12" x14ac:dyDescent="0.3">
@@ -36490,9 +36506,9 @@
         <f>SUM(J52:J60)</f>
         <v>1359.9032002243127</v>
       </c>
-      <c r="L51" s="110" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+      <c r="L51" s="127">
+        <f>((K51-Costs_init!K51)/Costs_init!K51)</f>
+        <v>0.29331225074729717</v>
       </c>
     </row>
     <row r="52" spans="1:12" x14ac:dyDescent="0.3">
@@ -36522,13 +36538,13 @@
         <v>231.31088503130337</v>
       </c>
       <c r="J52" s="111">
-        <f t="shared" ref="J52:J60" si="5">I52</f>
+        <f t="shared" ref="J52:J60" si="4">I52</f>
         <v>231.31088503130337</v>
       </c>
       <c r="K52" s="112"/>
-      <c r="L52" s="110">
-        <f t="shared" si="2"/>
-        <v>298.57088503130336</v>
+      <c r="L52" s="127">
+        <f>((J52-Costs_init!J52)/Costs_init!J52)</f>
+        <v>0.49999999999999989</v>
       </c>
     </row>
     <row r="53" spans="1:12" x14ac:dyDescent="0.3">
@@ -36558,13 +36574,13 @@
         <v>154.20725668753559</v>
       </c>
       <c r="J53" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>154.20725668753559</v>
       </c>
       <c r="K53" s="112"/>
-      <c r="L53" s="110">
-        <f t="shared" si="2"/>
-        <v>199.04725668753559</v>
+      <c r="L53" s="127">
+        <f>((J53-Costs_init!J53)/Costs_init!J53)</f>
+        <v>0.33333333333333343</v>
       </c>
     </row>
     <row r="54" spans="1:12" x14ac:dyDescent="0.3">
@@ -36594,13 +36610,13 @@
         <v>192.7590708594195</v>
       </c>
       <c r="J54" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>192.7590708594195</v>
       </c>
       <c r="K54" s="112"/>
-      <c r="L54" s="110">
-        <f t="shared" si="2"/>
-        <v>248.80907085941948</v>
+      <c r="L54" s="127">
+        <f>((J54-Costs_init!J54)/Costs_init!J54)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:12" x14ac:dyDescent="0.3">
@@ -36630,13 +36646,13 @@
         <v>115.65544251565169</v>
       </c>
       <c r="J55" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>115.65544251565169</v>
       </c>
       <c r="K55" s="112"/>
-      <c r="L55" s="110">
-        <f t="shared" si="2"/>
-        <v>149.28544251565168</v>
+      <c r="L55" s="127">
+        <f>((J55-Costs_init!J55)/Costs_init!J55)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:12" x14ac:dyDescent="0.3">
@@ -36666,13 +36682,13 @@
         <v>154.20725668753559</v>
       </c>
       <c r="J56" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>154.20725668753559</v>
       </c>
       <c r="K56" s="112"/>
-      <c r="L56" s="110">
-        <f t="shared" si="2"/>
-        <v>199.04725668753559</v>
+      <c r="L56" s="127">
+        <f>((J56-Costs_init!J56)/Costs_init!J56)</f>
+        <v>0.33333333333333343</v>
       </c>
     </row>
     <row r="57" spans="1:12" x14ac:dyDescent="0.3">
@@ -36702,13 +36718,13 @@
         <v>192.7590708594195</v>
       </c>
       <c r="J57" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>192.7590708594195</v>
       </c>
       <c r="K57" s="112"/>
-      <c r="L57" s="110">
-        <f t="shared" si="2"/>
-        <v>248.80907085941948</v>
+      <c r="L57" s="127">
+        <f>((J57-Costs_init!J57)/Costs_init!J57)</f>
+        <v>1.5</v>
       </c>
     </row>
     <row r="58" spans="1:12" x14ac:dyDescent="0.3">
@@ -36738,13 +36754,13 @@
         <v>115.65544251565169</v>
       </c>
       <c r="J58" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>115.65544251565169</v>
       </c>
       <c r="K58" s="112"/>
-      <c r="L58" s="110">
-        <f t="shared" si="2"/>
-        <v>149.28544251565168</v>
+      <c r="L58" s="127">
+        <f>((J58-Costs_init!J58)/Costs_init!J58)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="59" spans="1:12" x14ac:dyDescent="0.3">
@@ -36774,13 +36790,13 @@
         <v>115.65544251565169</v>
       </c>
       <c r="J59" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>115.65544251565169</v>
       </c>
       <c r="K59" s="112"/>
-      <c r="L59" s="110">
-        <f t="shared" si="2"/>
-        <v>149.28544251565168</v>
+      <c r="L59" s="127">
+        <f>((J59-Costs_init!J59)/Costs_init!J59)</f>
+        <v>0.49999999999999989</v>
       </c>
     </row>
     <row r="60" spans="1:12" x14ac:dyDescent="0.3">
@@ -36810,13 +36826,13 @@
         <v>87.693332552144369</v>
       </c>
       <c r="J60" s="111">
-        <f t="shared" si="5"/>
+        <f t="shared" si="4"/>
         <v>87.693332552144369</v>
       </c>
       <c r="K60" s="112"/>
-      <c r="L60" s="110">
-        <f t="shared" si="2"/>
-        <v>110.11333255214437</v>
+      <c r="L60" s="127">
+        <f>((J60-Costs_init!J60)/Costs_init!J60)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="61" spans="1:12" x14ac:dyDescent="0.3">
@@ -36841,9 +36857,9 @@
         <f>SUM(J62:J73)</f>
         <v>1285.9236266810587</v>
       </c>
-      <c r="L61" s="110" t="str">
-        <f t="shared" si="2"/>
-        <v/>
+      <c r="L61" s="127">
+        <f>((K61-Costs_init!K61)/Costs_init!K61)</f>
+        <v>-6.9886161367037875E-2</v>
       </c>
     </row>
     <row r="62" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -36873,13 +36889,13 @@
         <v>49.782125344774748</v>
       </c>
       <c r="J62" s="111">
-        <f t="shared" ref="J62:J73" si="6">I62</f>
+        <f t="shared" ref="J62:J73" si="5">I62</f>
         <v>49.782125344774748</v>
       </c>
       <c r="K62" s="112"/>
-      <c r="L62" s="110">
-        <f t="shared" si="2"/>
-        <v>60.992125344774749</v>
+      <c r="L62" s="127">
+        <f>((J62-Costs_init!J62)/Costs_init!J62)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="63" spans="1:12" x14ac:dyDescent="0.3">
@@ -36909,13 +36925,13 @@
         <v>49.782125344774748</v>
       </c>
       <c r="J63" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>49.782125344774748</v>
       </c>
       <c r="K63" s="112"/>
-      <c r="L63" s="110">
-        <f t="shared" si="2"/>
-        <v>60.992125344774749</v>
+      <c r="L63" s="127">
+        <f>((J63-Costs_init!J63)/Costs_init!J63)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="64" spans="1:12" x14ac:dyDescent="0.3">
@@ -36945,13 +36961,13 @@
         <v>45.220459339114129</v>
       </c>
       <c r="J64" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>45.220459339114129</v>
       </c>
       <c r="K64" s="112"/>
-      <c r="L64" s="110">
-        <f t="shared" si="2"/>
-        <v>56.43045933911413</v>
+      <c r="L64" s="127">
+        <f>((J64-Costs_init!J64)/Costs_init!J64)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="65" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -36981,13 +36997,13 @@
         <v>90.440918678228257</v>
       </c>
       <c r="J65" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>90.440918678228257</v>
       </c>
       <c r="K65" s="112"/>
-      <c r="L65" s="110">
-        <f t="shared" si="2"/>
-        <v>112.86091867822826</v>
+      <c r="L65" s="127">
+        <f>((J65-Costs_init!J65)/Costs_init!J65)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="66" spans="1:12" ht="28.8" x14ac:dyDescent="0.3">
@@ -37017,13 +37033,13 @@
         <v>149.34637603432424</v>
       </c>
       <c r="J66" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>149.34637603432424</v>
       </c>
       <c r="K66" s="112"/>
-      <c r="L66" s="110">
-        <f t="shared" si="2"/>
-        <v>182.97637603432423</v>
+      <c r="L66" s="127">
+        <f>((J66-Costs_init!J66)/Costs_init!J66)</f>
+        <v>0.49999999999999994</v>
       </c>
     </row>
     <row r="67" spans="1:12" x14ac:dyDescent="0.3">
@@ -37045,7 +37061,7 @@
         <v>103</v>
       </c>
       <c r="H67" s="111">
-        <f t="shared" ref="H67:H73" si="7">_xlfn.XLOOKUP(E67,$Q$20:$Q$25,$R$20:$R$25,"")</f>
+        <f t="shared" ref="H67:H73" si="6">_xlfn.XLOOKUP(E67,$Q$20:$Q$25,$R$20:$R$25,"")</f>
         <v>42.159269173306768</v>
       </c>
       <c r="I67" s="111">
@@ -37053,13 +37069,13 @@
         <v>84.318538346613536</v>
       </c>
       <c r="J67" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>84.318538346613536</v>
       </c>
       <c r="K67" s="112"/>
-      <c r="L67" s="110">
-        <f t="shared" si="2"/>
-        <v>106.73853834661354</v>
+      <c r="L67" s="127">
+        <f>((J67-Costs_init!J67)/Costs_init!J67)</f>
+        <v>-0.33333333333333331</v>
       </c>
     </row>
     <row r="68" spans="1:12" x14ac:dyDescent="0.3">
@@ -37081,21 +37097,21 @@
         <v>103</v>
       </c>
       <c r="H68" s="111">
-        <f t="shared" si="7"/>
+        <f t="shared" si="6"/>
         <v>49.154057104913683</v>
       </c>
       <c r="I68" s="111">
-        <f t="shared" ref="I68:I73" si="8">IFERROR(H68*F68,"")</f>
+        <f t="shared" ref="I68:I73" si="7">IFERROR(H68*F68,"")</f>
         <v>147.46217131474106</v>
       </c>
       <c r="J68" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>147.46217131474106</v>
       </c>
       <c r="K68" s="112"/>
-      <c r="L68" s="110">
-        <f t="shared" ref="L68:L73" si="9">IFERROR(I68+($P$10*F68),"")</f>
-        <v>181.09217131474105</v>
+      <c r="L68" s="127">
+        <f>((J68-Costs_init!J68)/Costs_init!J68)</f>
+        <v>-0.39999999999999997</v>
       </c>
     </row>
     <row r="69" spans="1:12" x14ac:dyDescent="0.3">
@@ -37117,21 +37133,21 @@
         <v>103</v>
       </c>
       <c r="H69" s="111">
+        <f t="shared" si="6"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I69" s="111">
         <f t="shared" si="7"/>
-        <v>43.846666276072185</v>
-      </c>
-      <c r="I69" s="111">
-        <f t="shared" si="8"/>
         <v>263.07999765643308</v>
       </c>
       <c r="J69" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>263.07999765643308</v>
       </c>
       <c r="K69" s="112"/>
-      <c r="L69" s="110">
-        <f t="shared" si="9"/>
-        <v>330.33999765643307</v>
+      <c r="L69" s="127">
+        <f>((J69-Costs_init!J69)/Costs_init!J69)</f>
+        <v>0.19999999999999979</v>
       </c>
     </row>
     <row r="70" spans="1:12" x14ac:dyDescent="0.3">
@@ -37153,21 +37169,21 @@
         <v>103</v>
       </c>
       <c r="H70" s="111">
+        <f t="shared" si="6"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I70" s="111">
         <f t="shared" si="7"/>
-        <v>43.846666276072185</v>
-      </c>
-      <c r="I70" s="111">
-        <f t="shared" si="8"/>
         <v>87.693332552144369</v>
       </c>
       <c r="J70" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>87.693332552144369</v>
       </c>
       <c r="K70" s="112"/>
-      <c r="L70" s="110">
-        <f t="shared" si="9"/>
-        <v>110.11333255214437</v>
+      <c r="L70" s="127">
+        <f>((J70-Costs_init!J70)/Costs_init!J70)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="71" spans="1:12" x14ac:dyDescent="0.3">
@@ -37189,21 +37205,21 @@
         <v>103</v>
       </c>
       <c r="H71" s="111">
+        <f t="shared" si="6"/>
+        <v>43.846666276072185</v>
+      </c>
+      <c r="I71" s="111">
         <f t="shared" si="7"/>
-        <v>43.846666276072185</v>
-      </c>
-      <c r="I71" s="111">
-        <f t="shared" si="8"/>
         <v>219.23333138036094</v>
       </c>
       <c r="J71" s="111">
-        <f t="shared" si="6"/>
+        <f t="shared" si="5"/>
         <v>219.23333138036094</v>
       </c>
       <c r="K71" s="112"/>
-      <c r="L71" s="110">
-        <f t="shared" si="9"/>
-        <v>275.28333138036095</v>
+      <c r="L71" s="127">
+        <f>((J71-Costs_init!J71)/Costs_init!J71)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="72" spans="1:12" x14ac:dyDescent="0.3">
@@ -37225,21 +37241,21 @@
         <v>103</v>
       </c>
       <c r="H72" s="111">
+        <f t="shared" si="6"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I72" s="111">
         <f t="shared" si="7"/>
         <v>49.782125344774748</v>
       </c>
-      <c r="I72" s="111">
-        <f t="shared" si="8"/>
+      <c r="J72" s="111">
+        <f t="shared" si="5"/>
         <v>49.782125344774748</v>
       </c>
-      <c r="J72" s="111">
-        <f t="shared" si="6"/>
-        <v>49.782125344774748</v>
-      </c>
       <c r="K72" s="112"/>
-      <c r="L72" s="110">
-        <f t="shared" si="9"/>
-        <v>60.992125344774749</v>
+      <c r="L72" s="127">
+        <f>((J72-Costs_init!J72)/Costs_init!J72)</f>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="73" spans="1:12" x14ac:dyDescent="0.3">
@@ -37261,43 +37277,43 @@
         <v>103</v>
       </c>
       <c r="H73" s="111">
+        <f t="shared" si="6"/>
+        <v>49.782125344774748</v>
+      </c>
+      <c r="I73" s="111">
         <f t="shared" si="7"/>
         <v>49.782125344774748</v>
       </c>
-      <c r="I73" s="111">
-        <f t="shared" si="8"/>
+      <c r="J73" s="111">
+        <f t="shared" si="5"/>
         <v>49.782125344774748</v>
       </c>
-      <c r="J73" s="111">
-        <f t="shared" si="6"/>
-        <v>49.782125344774748</v>
-      </c>
       <c r="K73" s="113"/>
-      <c r="L73" s="110">
-        <f t="shared" si="9"/>
-        <v>60.992125344774749</v>
+      <c r="L73" s="127">
+        <f>((J73-Costs_init!J73)/Costs_init!J73)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="74" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A74" s="130" t="s">
+      <c r="A74" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="B74" s="131"/>
-      <c r="C74" s="131"/>
-      <c r="D74" s="131"/>
-      <c r="E74" s="131"/>
-      <c r="F74" s="131"/>
-      <c r="G74" s="131"/>
-      <c r="H74" s="131"/>
-      <c r="I74" s="131"/>
-      <c r="J74" s="131"/>
+      <c r="B74" s="129"/>
+      <c r="C74" s="129"/>
+      <c r="D74" s="129"/>
+      <c r="E74" s="129"/>
+      <c r="F74" s="129"/>
+      <c r="G74" s="129"/>
+      <c r="H74" s="129"/>
+      <c r="I74" s="129"/>
+      <c r="J74" s="129"/>
       <c r="K74" s="114">
         <f>SUM(K3:K73)</f>
         <v>13383.612572529586</v>
       </c>
-      <c r="L74" s="111">
-        <f>SUM(L3:L73)</f>
-        <v>16858.712572529592</v>
+      <c r="L74" s="127">
+        <f>((K74-Costs_init!K74)/Costs_init!K74)</f>
+        <v>2.7412946238235029E-2</v>
       </c>
     </row>
     <row r="75" spans="1:12" x14ac:dyDescent="0.3">
@@ -37305,19 +37321,19 @@
       <c r="L75" s="2"/>
     </row>
     <row r="76" spans="1:12" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A76" s="132" t="s">
+      <c r="A76" s="134" t="s">
         <v>192</v>
       </c>
-      <c r="B76" s="133"/>
-      <c r="C76" s="133"/>
-      <c r="D76" s="133"/>
-      <c r="E76" s="133"/>
-      <c r="F76" s="133"/>
-      <c r="G76" s="133"/>
-      <c r="H76" s="133"/>
-      <c r="I76" s="133"/>
-      <c r="J76" s="133"/>
-      <c r="K76" s="134"/>
+      <c r="B76" s="135"/>
+      <c r="C76" s="135"/>
+      <c r="D76" s="135"/>
+      <c r="E76" s="135"/>
+      <c r="F76" s="135"/>
+      <c r="G76" s="135"/>
+      <c r="H76" s="135"/>
+      <c r="I76" s="135"/>
+      <c r="J76" s="135"/>
+      <c r="K76" s="136"/>
       <c r="L76" s="124"/>
     </row>
     <row r="77" spans="1:12" x14ac:dyDescent="0.3">
@@ -37436,18 +37452,18 @@
       <c r="L80" s="116"/>
     </row>
     <row r="81" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A81" s="130" t="s">
+      <c r="A81" s="128" t="s">
         <v>4</v>
       </c>
-      <c r="B81" s="131"/>
-      <c r="C81" s="131"/>
-      <c r="D81" s="131"/>
-      <c r="E81" s="131"/>
-      <c r="F81" s="131"/>
-      <c r="G81" s="131"/>
-      <c r="H81" s="131"/>
-      <c r="I81" s="131"/>
-      <c r="J81" s="131"/>
+      <c r="B81" s="129"/>
+      <c r="C81" s="129"/>
+      <c r="D81" s="129"/>
+      <c r="E81" s="129"/>
+      <c r="F81" s="129"/>
+      <c r="G81" s="129"/>
+      <c r="H81" s="129"/>
+      <c r="I81" s="129"/>
+      <c r="J81" s="129"/>
       <c r="K81" s="114">
         <f>SUM(K78:K80)</f>
         <v>172.5</v>

</xml_diff>